<commit_message>
Sumando ilustraciones y mejoras Cla
</commit_message>
<xml_diff>
--- a/data/PortfolioArTeV1.xlsx
+++ b/data/PortfolioArTeV1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arturompw/portfolio/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DBE69E1-ABD8-444C-AEF1-7C319B14E731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CFB46FF-D57C-3B4B-8683-52A9C2FFB76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2503" uniqueCount="693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2764" uniqueCount="751">
   <si>
     <t>id</t>
   </si>
@@ -850,9 +850,6 @@
     <t>Camiseta Da Vida 2025 (espalda)</t>
   </si>
   <si>
-    <t>Sticker G de Grupos</t>
-  </si>
-  <si>
     <t>Camiseta a better World 2016</t>
   </si>
   <si>
@@ -1075,9 +1072,6 @@
     <t>Eucaristía</t>
   </si>
   <si>
-    <t>Para Primera Eucaristía Sevilla 2017</t>
-  </si>
-  <si>
     <t>evangelio;GVX</t>
   </si>
   <si>
@@ -1126,9 +1120,6 @@
     <t>Faros de Esperanza</t>
   </si>
   <si>
-    <t>Para Capítulo Prov Mediterránea</t>
-  </si>
-  <si>
     <t>…una casa acogliente</t>
   </si>
   <si>
@@ -1468,12 +1459,6 @@
     <t>Change &lt; &gt; Chance</t>
   </si>
   <si>
-    <t>Cartel 2025 Mediterránea</t>
-  </si>
-  <si>
-    <t>Cartel 2022 Mediterránea</t>
-  </si>
-  <si>
     <t>Recordando al Hno Boni FQ</t>
   </si>
   <si>
@@ -1939,9 +1924,6 @@
     <t>A_Arroyo</t>
   </si>
   <si>
-    <t>Be Marist Brother punto com</t>
-  </si>
-  <si>
     <t>DIS-0070</t>
   </si>
   <si>
@@ -2008,9 +1990,6 @@
     <t>textil;sticker;taza</t>
   </si>
   <si>
-    <t>Nueva versión de camiseta GVX Sevilla 1993</t>
-  </si>
-  <si>
     <t>Mi Buena Madre (esp)</t>
   </si>
   <si>
@@ -2099,6 +2078,201 @@
   </si>
   <si>
     <t>Viñeta 'Al fin, luz'</t>
+  </si>
+  <si>
+    <t>Para Asamblea Mediterránea 2018</t>
+  </si>
+  <si>
+    <t>Para Capítulo Prov Mediterránea 2021</t>
+  </si>
+  <si>
+    <t>Nueva versión de camiseta GVX Sevilla (1993)</t>
+  </si>
+  <si>
+    <t>ILU-0106</t>
+  </si>
+  <si>
+    <t>ILU-0107</t>
+  </si>
+  <si>
+    <t>ILU-0108</t>
+  </si>
+  <si>
+    <t>ILU-0109</t>
+  </si>
+  <si>
+    <t>ILU-0110</t>
+  </si>
+  <si>
+    <t>ILU-0111</t>
+  </si>
+  <si>
+    <t>ILU-0112</t>
+  </si>
+  <si>
+    <t>ILU-0113</t>
+  </si>
+  <si>
+    <t>ILU-0114</t>
+  </si>
+  <si>
+    <t>ILU-0115</t>
+  </si>
+  <si>
+    <t>ILU-0116</t>
+  </si>
+  <si>
+    <t>DIS-0078</t>
+  </si>
+  <si>
+    <t>DIS-0079</t>
+  </si>
+  <si>
+    <t>DIS-0080</t>
+  </si>
+  <si>
+    <t>DIS-0081</t>
+  </si>
+  <si>
+    <t>DIS-0082</t>
+  </si>
+  <si>
+    <t>DIS-0083</t>
+  </si>
+  <si>
+    <t>DIS-0084</t>
+  </si>
+  <si>
+    <t>DIS-0085</t>
+  </si>
+  <si>
+    <t>DIS-0086</t>
+  </si>
+  <si>
+    <t>Cartel Asamblea Mediterránea 2018</t>
+  </si>
+  <si>
+    <t>Maristas Champions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camiseta Voluntarios </t>
+  </si>
+  <si>
+    <t>II Jornadas Educadores Maristas</t>
+  </si>
+  <si>
+    <t>Cartel Jornadas 2017 Mediterránea</t>
+  </si>
+  <si>
+    <t>III Jornadas Educadores Maristas (fra)</t>
+  </si>
+  <si>
+    <t>Cartel Jornadas 2019 Mediterránea</t>
+  </si>
+  <si>
+    <t>Cartel Jornadas 2022 Mediterránea</t>
+  </si>
+  <si>
+    <t>Cartel Jornadas 2025 Mediterránea</t>
+  </si>
+  <si>
+    <t>Para GIX Sevilla 2017</t>
+  </si>
+  <si>
+    <t>Be Marist Brother (punto) com</t>
+  </si>
+  <si>
+    <t>G de Grupos</t>
+  </si>
+  <si>
+    <t>Maristas Innova 2017</t>
+  </si>
+  <si>
+    <t>Para Jornadas 2017 Mediterránea</t>
+  </si>
+  <si>
+    <t>Agenda Escolar Sevilla 2012-2013</t>
+  </si>
+  <si>
+    <t>Portada y contraportada</t>
+  </si>
+  <si>
+    <t>Agenda Escolar Sevilla 2011-2012</t>
+  </si>
+  <si>
+    <t>Portada y contraportada (con escudos maristas)</t>
+  </si>
+  <si>
+    <t>Occupiamo il futuro</t>
+  </si>
+  <si>
+    <t>Para asamblea zona Italia</t>
+  </si>
+  <si>
+    <t>Buen Camino</t>
+  </si>
+  <si>
+    <t>Camiseta Camino Pastoral Sevilla 2018</t>
+  </si>
+  <si>
+    <t>Mascota asamblea</t>
+  </si>
+  <si>
+    <t>Probando ideas</t>
+  </si>
+  <si>
+    <t>Real wi-fi</t>
+  </si>
+  <si>
+    <t>También parte del cartel 'Sonríe de corazón' MRE</t>
+  </si>
+  <si>
+    <t>Avión de papel</t>
+  </si>
+  <si>
+    <t>Maori Marist Pillars I</t>
+  </si>
+  <si>
+    <t>Maori Marist Pillars II</t>
+  </si>
+  <si>
+    <t>Maori Marist Pillars III</t>
+  </si>
+  <si>
+    <t>Maori Marist Pillars IV</t>
+  </si>
+  <si>
+    <t>Maori Marist Pillars V</t>
+  </si>
+  <si>
+    <t>Marist_NewZealand</t>
+  </si>
+  <si>
+    <t>Amor al trabajo (eng, mao)</t>
+  </si>
+  <si>
+    <t>Sencillez (eng, mao)</t>
+  </si>
+  <si>
+    <t>Al estilo de María (eng, mao)</t>
+  </si>
+  <si>
+    <t>Presencia (eng, mao)</t>
+  </si>
+  <si>
+    <t>Espíritu de familia (eng, mao)</t>
+  </si>
+  <si>
+    <t>La chasca</t>
+  </si>
+  <si>
+    <t>María, Buena Madre V</t>
+  </si>
+  <si>
+    <t>Para capilla colegio S Pio XII Roma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pasión </t>
   </si>
 </sst>
 </file>
@@ -2455,15 +2629,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N183"/>
+  <dimension ref="A1:N203"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="29" customWidth="1"/>
-    <col min="3" max="3" width="36.6640625" customWidth="1"/>
+    <col min="2" max="2" width="32.33203125" customWidth="1"/>
+    <col min="3" max="3" width="38.33203125" customWidth="1"/>
     <col min="4" max="4" width="10.33203125" customWidth="1"/>
     <col min="5" max="5" width="7.83203125" customWidth="1"/>
     <col min="6" max="6" width="9.5" customWidth="1"/>
-    <col min="7" max="7" width="19.5" customWidth="1"/>
+    <col min="7" max="7" width="26.1640625" customWidth="1"/>
     <col min="8" max="8" width="30.1640625" customWidth="1"/>
     <col min="9" max="10" width="18.83203125" customWidth="1"/>
     <col min="11" max="11" width="15.5" customWidth="1"/>
@@ -2521,7 +2695,7 @@
         <v>175</v>
       </c>
       <c r="C2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D2" t="s">
         <v>54</v>
@@ -2565,7 +2739,7 @@
         <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D3" t="s">
         <v>54</v>
@@ -2583,7 +2757,7 @@
         <v>28</v>
       </c>
       <c r="I3" t="s">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="J3" t="s">
         <v>208</v>
@@ -2606,7 +2780,7 @@
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>551</v>
+        <v>546</v>
       </c>
       <c r="C4" t="s">
         <v>86</v>
@@ -2776,7 +2950,7 @@
         <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D8" t="s">
         <v>54</v>
@@ -2797,7 +2971,7 @@
         <v>61</v>
       </c>
       <c r="J8" t="s">
-        <v>570</v>
+        <v>565</v>
       </c>
       <c r="K8" t="s">
         <v>55</v>
@@ -2861,7 +3035,7 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>550</v>
+        <v>545</v>
       </c>
       <c r="C10" t="s">
         <v>90</v>
@@ -2905,7 +3079,7 @@
         <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>551</v>
+        <v>546</v>
       </c>
       <c r="C11" t="s">
         <v>91</v>
@@ -2949,7 +3123,7 @@
         <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>551</v>
+        <v>546</v>
       </c>
       <c r="C12" t="s">
         <v>92</v>
@@ -2993,7 +3167,7 @@
         <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>551</v>
+        <v>546</v>
       </c>
       <c r="C13" t="s">
         <v>93</v>
@@ -3037,7 +3211,7 @@
         <v>38</v>
       </c>
       <c r="B14" t="s">
-        <v>551</v>
+        <v>546</v>
       </c>
       <c r="C14" t="s">
         <v>94</v>
@@ -3099,7 +3273,7 @@
         <v>251</v>
       </c>
       <c r="H15" t="s">
-        <v>552</v>
+        <v>547</v>
       </c>
       <c r="I15" t="s">
         <v>101</v>
@@ -3140,7 +3314,7 @@
         <v>13</v>
       </c>
       <c r="G16" t="s">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="H16" t="s">
         <v>28</v>
@@ -3184,7 +3358,7 @@
         <v>32</v>
       </c>
       <c r="G17" t="s">
-        <v>636</v>
+        <v>631</v>
       </c>
       <c r="H17" t="s">
         <v>59</v>
@@ -3228,10 +3402,10 @@
         <v>32</v>
       </c>
       <c r="G18" t="s">
-        <v>636</v>
+        <v>631</v>
       </c>
       <c r="H18" t="s">
-        <v>553</v>
+        <v>548</v>
       </c>
       <c r="J18" t="s">
         <v>208</v>
@@ -3269,7 +3443,7 @@
         <v>32</v>
       </c>
       <c r="G19" t="s">
-        <v>637</v>
+        <v>632</v>
       </c>
       <c r="H19" t="s">
         <v>28</v>
@@ -3398,7 +3572,7 @@
         <v>167</v>
       </c>
       <c r="H22" t="s">
-        <v>554</v>
+        <v>549</v>
       </c>
       <c r="I22" t="s">
         <v>61</v>
@@ -3483,7 +3657,7 @@
         <v>32</v>
       </c>
       <c r="G24" t="s">
-        <v>637</v>
+        <v>632</v>
       </c>
       <c r="H24" t="s">
         <v>28</v>
@@ -3527,7 +3701,7 @@
         <v>169</v>
       </c>
       <c r="H25" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="J25" t="s">
         <v>83</v>
@@ -3568,7 +3742,7 @@
         <v>169</v>
       </c>
       <c r="H26" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="J26" t="s">
         <v>102</v>
@@ -3656,7 +3830,7 @@
         <v>61</v>
       </c>
       <c r="J28" t="s">
-        <v>635</v>
+        <v>630</v>
       </c>
       <c r="K28" t="s">
         <v>56</v>
@@ -3694,7 +3868,7 @@
         <v>97</v>
       </c>
       <c r="H29" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="I29" t="s">
         <v>82</v>
@@ -3820,7 +3994,7 @@
         <v>167</v>
       </c>
       <c r="H32" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="J32" t="s">
         <v>102</v>
@@ -3861,7 +4035,7 @@
         <v>167</v>
       </c>
       <c r="H33" t="s">
-        <v>555</v>
+        <v>550</v>
       </c>
       <c r="J33" t="s">
         <v>102</v>
@@ -3993,7 +4167,7 @@
         <v>166</v>
       </c>
       <c r="J36" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="K36" t="s">
         <v>55</v>
@@ -4251,7 +4425,7 @@
         <v>167</v>
       </c>
       <c r="H42" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="I42" t="s">
         <v>61</v>
@@ -4280,7 +4454,7 @@
         <v>246</v>
       </c>
       <c r="C43" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="D43" t="s">
         <v>54</v>
@@ -4295,7 +4469,7 @@
         <v>167</v>
       </c>
       <c r="H43" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="I43" t="s">
         <v>61</v>
@@ -4339,7 +4513,7 @@
         <v>167</v>
       </c>
       <c r="H44" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="I44" t="s">
         <v>61</v>
@@ -4383,7 +4557,7 @@
         <v>167</v>
       </c>
       <c r="H45" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="I45" t="s">
         <v>156</v>
@@ -4406,13 +4580,13 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B46" t="s">
         <v>281</v>
       </c>
-      <c r="B46" t="s">
-        <v>282</v>
-      </c>
       <c r="C46" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="D46" t="s">
         <v>54</v>
@@ -4427,7 +4601,7 @@
         <v>167</v>
       </c>
       <c r="H46" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I46" t="s">
         <v>166</v>
@@ -4450,13 +4624,13 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="B47" t="s">
         <v>283</v>
       </c>
-      <c r="B47" t="s">
-        <v>284</v>
-      </c>
       <c r="C47" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="D47" t="s">
         <v>54</v>
@@ -4471,7 +4645,7 @@
         <v>167</v>
       </c>
       <c r="H47" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I47" t="s">
         <v>166</v>
@@ -4494,13 +4668,13 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B48" t="s">
+        <v>294</v>
+      </c>
+      <c r="C48" t="s">
         <v>295</v>
-      </c>
-      <c r="C48" t="s">
-        <v>296</v>
       </c>
       <c r="D48" t="s">
         <v>54</v>
@@ -4521,7 +4695,7 @@
         <v>60</v>
       </c>
       <c r="J48" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="K48" t="s">
         <v>55</v>
@@ -4538,13 +4712,13 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B49" t="s">
+        <v>296</v>
+      </c>
+      <c r="C49" t="s">
         <v>297</v>
-      </c>
-      <c r="C49" t="s">
-        <v>298</v>
       </c>
       <c r="D49" t="s">
         <v>54</v>
@@ -4559,7 +4733,7 @@
         <v>167</v>
       </c>
       <c r="H49" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I49" t="s">
         <v>156</v>
@@ -4582,13 +4756,13 @@
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B50" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C50" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D50" t="s">
         <v>54</v>
@@ -4603,7 +4777,7 @@
         <v>119</v>
       </c>
       <c r="H50" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I50" t="s">
         <v>156</v>
@@ -4626,13 +4800,13 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B51" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C51" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D51" t="s">
         <v>54</v>
@@ -4647,7 +4821,7 @@
         <v>119</v>
       </c>
       <c r="H51" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I51" t="s">
         <v>156</v>
@@ -4670,13 +4844,13 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B52" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="C52" t="s">
-        <v>306</v>
+        <v>686</v>
       </c>
       <c r="D52" t="s">
         <v>54</v>
@@ -4688,7 +4862,7 @@
         <v>13</v>
       </c>
       <c r="G52" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H52" t="s">
         <v>120</v>
@@ -4714,13 +4888,13 @@
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B53" t="s">
+        <v>312</v>
+      </c>
+      <c r="C53" t="s">
         <v>313</v>
-      </c>
-      <c r="C53" t="s">
-        <v>314</v>
       </c>
       <c r="D53" t="s">
         <v>54</v>
@@ -4735,7 +4909,7 @@
         <v>167</v>
       </c>
       <c r="H53" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="I53" t="s">
         <v>61</v>
@@ -4758,13 +4932,13 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B54" t="s">
+        <v>315</v>
+      </c>
+      <c r="C54" t="s">
         <v>316</v>
-      </c>
-      <c r="C54" t="s">
-        <v>317</v>
       </c>
       <c r="D54" t="s">
         <v>54</v>
@@ -4779,7 +4953,7 @@
         <v>167</v>
       </c>
       <c r="H54" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J54" t="s">
         <v>102</v>
@@ -4799,13 +4973,13 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B55" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C55" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D55" t="s">
         <v>54</v>
@@ -4817,16 +4991,16 @@
         <v>13</v>
       </c>
       <c r="G55" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H55" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="I55" t="s">
         <v>156</v>
       </c>
       <c r="J55" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="K55" t="s">
         <v>55</v>
@@ -4843,13 +5017,13 @@
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B56" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C56" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D56" t="s">
         <v>54</v>
@@ -4864,13 +5038,13 @@
         <v>167</v>
       </c>
       <c r="H56" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="I56" t="s">
         <v>166</v>
       </c>
       <c r="J56" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="K56" t="s">
         <v>55</v>
@@ -4887,13 +5061,13 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B57" t="s">
+        <v>324</v>
+      </c>
+      <c r="C57" t="s">
         <v>325</v>
-      </c>
-      <c r="C57" t="s">
-        <v>326</v>
       </c>
       <c r="D57" t="s">
         <v>54</v>
@@ -4928,13 +5102,13 @@
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="B58" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="C58" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="D58" t="s">
         <v>54</v>
@@ -4946,10 +5120,10 @@
         <v>32</v>
       </c>
       <c r="G58" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="H58" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="I58" t="s">
         <v>237</v>
@@ -4972,13 +5146,13 @@
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="B59" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="C59" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="D59" t="s">
         <v>54</v>
@@ -4993,7 +5167,7 @@
         <v>171</v>
       </c>
       <c r="H59" t="s">
-        <v>556</v>
+        <v>551</v>
       </c>
       <c r="J59" t="s">
         <v>102</v>
@@ -5013,13 +5187,13 @@
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="B60" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="C60" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="D60" t="s">
         <v>54</v>
@@ -5031,10 +5205,10 @@
         <v>32</v>
       </c>
       <c r="G60" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="H60" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="I60" t="s">
         <v>60</v>
@@ -5057,13 +5231,13 @@
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="B61" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="C61" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D61" t="s">
         <v>54</v>
@@ -5075,13 +5249,13 @@
         <v>13</v>
       </c>
       <c r="G61" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H61" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J61" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="K61" t="s">
         <v>55</v>
@@ -5098,13 +5272,13 @@
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="B62" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="C62" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="D62" t="s">
         <v>54</v>
@@ -5116,10 +5290,10 @@
         <v>13</v>
       </c>
       <c r="G62" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H62" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I62" t="s">
         <v>82</v>
@@ -5142,13 +5316,13 @@
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="B63" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="C63" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="D63" t="s">
         <v>54</v>
@@ -5160,16 +5334,16 @@
         <v>13</v>
       </c>
       <c r="G63" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H63" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I63" t="s">
         <v>166</v>
       </c>
       <c r="J63" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="K63" t="s">
         <v>55</v>
@@ -5186,13 +5360,13 @@
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="B64" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C64" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D64" t="s">
         <v>54</v>
@@ -5204,10 +5378,10 @@
         <v>13</v>
       </c>
       <c r="G64" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="H64" t="s">
-        <v>564</v>
+        <v>559</v>
       </c>
       <c r="J64" t="s">
         <v>172</v>
@@ -5227,13 +5401,13 @@
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="B65" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="C65" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="D65" t="s">
         <v>54</v>
@@ -5268,13 +5442,13 @@
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="B66" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="C66" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="D66" t="s">
         <v>54</v>
@@ -5289,7 +5463,7 @@
         <v>253</v>
       </c>
       <c r="H66" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="I66" t="s">
         <v>61</v>
@@ -5312,13 +5486,13 @@
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="B67" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="C67" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="D67" t="s">
         <v>54</v>
@@ -5330,13 +5504,13 @@
         <v>13</v>
       </c>
       <c r="G67" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H67" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="J67" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="K67" t="s">
         <v>55</v>
@@ -5353,13 +5527,13 @@
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="B68" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="C68" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="D68" t="s">
         <v>54</v>
@@ -5374,10 +5548,10 @@
         <v>167</v>
       </c>
       <c r="H68" t="s">
-        <v>601</v>
+        <v>596</v>
       </c>
       <c r="J68" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="K68" t="s">
         <v>55</v>
@@ -5394,13 +5568,13 @@
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="B69" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="C69" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="D69" t="s">
         <v>54</v>
@@ -5438,13 +5612,13 @@
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B70" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="C70" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="D70" t="s">
         <v>54</v>
@@ -5459,7 +5633,7 @@
         <v>119</v>
       </c>
       <c r="H70" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J70" t="s">
         <v>207</v>
@@ -5479,13 +5653,13 @@
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="B71" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="C71" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="D71" t="s">
         <v>54</v>
@@ -5500,7 +5674,7 @@
         <v>169</v>
       </c>
       <c r="H71" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I71" t="s">
         <v>61</v>
@@ -5523,13 +5697,13 @@
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="B72" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="C72" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="D72" t="s">
         <v>54</v>
@@ -5544,7 +5718,7 @@
         <v>167</v>
       </c>
       <c r="H72" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J72" t="s">
         <v>227</v>
@@ -5564,13 +5738,13 @@
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="B73" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="C73" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="D73" t="s">
         <v>54</v>
@@ -5585,7 +5759,7 @@
         <v>167</v>
       </c>
       <c r="H73" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="J73" t="s">
         <v>208</v>
@@ -5605,13 +5779,13 @@
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="B74" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="C74" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="D74" t="s">
         <v>54</v>
@@ -5629,7 +5803,7 @@
         <v>153</v>
       </c>
       <c r="I74" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="J74" t="s">
         <v>208</v>
@@ -5649,13 +5823,13 @@
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="B75" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="C75" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="D75" t="s">
         <v>54</v>
@@ -5693,13 +5867,13 @@
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="B76" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="C76" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="D76" t="s">
         <v>54</v>
@@ -5714,7 +5888,7 @@
         <v>167</v>
       </c>
       <c r="H76" t="s">
-        <v>566</v>
+        <v>561</v>
       </c>
       <c r="I76" t="s">
         <v>61</v>
@@ -5737,13 +5911,13 @@
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="B77" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="C77" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="D77" t="s">
         <v>54</v>
@@ -5758,7 +5932,7 @@
         <v>167</v>
       </c>
       <c r="H77" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="I77" t="s">
         <v>61</v>
@@ -5781,13 +5955,13 @@
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B78" t="s">
+        <v>488</v>
+      </c>
+      <c r="C78" t="s">
         <v>489</v>
-      </c>
-      <c r="B78" t="s">
-        <v>493</v>
-      </c>
-      <c r="C78" t="s">
-        <v>494</v>
       </c>
       <c r="D78" t="s">
         <v>54</v>
@@ -5802,7 +5976,7 @@
         <v>167</v>
       </c>
       <c r="H78" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="I78" t="s">
         <v>61</v>
@@ -5825,13 +5999,13 @@
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B79" t="s">
         <v>490</v>
       </c>
-      <c r="B79" t="s">
-        <v>495</v>
-      </c>
       <c r="C79" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="D79" t="s">
         <v>54</v>
@@ -5843,16 +6017,16 @@
         <v>32</v>
       </c>
       <c r="G79" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="H79" t="s">
-        <v>496</v>
+        <v>491</v>
       </c>
       <c r="I79" t="s">
         <v>61</v>
       </c>
       <c r="J79" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="K79" t="s">
         <v>55</v>
@@ -5869,13 +6043,13 @@
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
       <c r="B80" t="s">
-        <v>498</v>
+        <v>493</v>
       </c>
       <c r="C80" t="s">
-        <v>499</v>
+        <v>494</v>
       </c>
       <c r="D80" t="s">
         <v>54</v>
@@ -5890,7 +6064,7 @@
         <v>167</v>
       </c>
       <c r="H80" t="s">
-        <v>603</v>
+        <v>598</v>
       </c>
       <c r="I80" t="s">
         <v>61</v>
@@ -5913,13 +6087,13 @@
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
       <c r="B81" t="s">
-        <v>500</v>
+        <v>495</v>
       </c>
       <c r="C81" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="D81" t="s">
         <v>54</v>
@@ -5934,7 +6108,7 @@
         <v>167</v>
       </c>
       <c r="H81" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="I81" t="s">
         <v>61</v>
@@ -5957,13 +6131,13 @@
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
-        <v>504</v>
+        <v>499</v>
       </c>
       <c r="B82" t="s">
-        <v>513</v>
+        <v>508</v>
       </c>
       <c r="C82" t="s">
-        <v>516</v>
+        <v>511</v>
       </c>
       <c r="D82" t="s">
         <v>54</v>
@@ -5978,7 +6152,7 @@
         <v>119</v>
       </c>
       <c r="H82" t="s">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="I82" t="s">
         <v>61</v>
@@ -6001,13 +6175,13 @@
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="B83" t="s">
-        <v>515</v>
+        <v>510</v>
       </c>
       <c r="C83" t="s">
-        <v>516</v>
+        <v>511</v>
       </c>
       <c r="D83" t="s">
         <v>54</v>
@@ -6045,13 +6219,13 @@
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
-        <v>506</v>
+        <v>501</v>
       </c>
       <c r="B84" t="s">
-        <v>517</v>
+        <v>512</v>
       </c>
       <c r="C84" t="s">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="D84" t="s">
         <v>54</v>
@@ -6066,7 +6240,7 @@
         <v>167</v>
       </c>
       <c r="H84" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="I84" t="s">
         <v>61</v>
@@ -6089,13 +6263,13 @@
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
-        <v>507</v>
+        <v>502</v>
       </c>
       <c r="B85" t="s">
-        <v>521</v>
+        <v>516</v>
       </c>
       <c r="C85" t="s">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="D85" t="s">
         <v>54</v>
@@ -6107,10 +6281,10 @@
         <v>32</v>
       </c>
       <c r="G85" t="s">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="H85" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="I85" t="s">
         <v>61</v>
@@ -6133,13 +6307,13 @@
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
-        <v>508</v>
+        <v>503</v>
       </c>
       <c r="B86" t="s">
-        <v>522</v>
+        <v>517</v>
       </c>
       <c r="C86" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="D86" t="s">
         <v>54</v>
@@ -6154,7 +6328,7 @@
         <v>118</v>
       </c>
       <c r="H86" t="s">
-        <v>604</v>
+        <v>599</v>
       </c>
       <c r="I86" t="s">
         <v>61</v>
@@ -6177,13 +6351,13 @@
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
-        <v>509</v>
+        <v>504</v>
       </c>
       <c r="B87" t="s">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="C87" t="s">
-        <v>525</v>
+        <v>520</v>
       </c>
       <c r="D87" t="s">
         <v>54</v>
@@ -6198,7 +6372,7 @@
         <v>167</v>
       </c>
       <c r="H87" t="s">
-        <v>605</v>
+        <v>600</v>
       </c>
       <c r="I87" t="s">
         <v>61</v>
@@ -6221,13 +6395,13 @@
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
-        <v>510</v>
+        <v>505</v>
       </c>
       <c r="B88" t="s">
-        <v>527</v>
+        <v>522</v>
       </c>
       <c r="C88" t="s">
-        <v>528</v>
+        <v>523</v>
       </c>
       <c r="D88" t="s">
         <v>54</v>
@@ -6265,13 +6439,13 @@
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
-        <v>511</v>
+        <v>506</v>
       </c>
       <c r="B89" t="s">
-        <v>529</v>
+        <v>524</v>
       </c>
       <c r="C89" t="s">
-        <v>530</v>
+        <v>525</v>
       </c>
       <c r="D89" t="s">
         <v>54</v>
@@ -6286,7 +6460,7 @@
         <v>169</v>
       </c>
       <c r="H89" t="s">
-        <v>606</v>
+        <v>601</v>
       </c>
       <c r="I89" t="s">
         <v>61</v>
@@ -6309,13 +6483,13 @@
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="B90" t="s">
-        <v>531</v>
+        <v>526</v>
       </c>
       <c r="C90" t="s">
-        <v>516</v>
+        <v>511</v>
       </c>
       <c r="D90" t="s">
         <v>54</v>
@@ -6353,13 +6527,13 @@
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="B91" t="s">
         <v>572</v>
       </c>
-      <c r="B91" t="s">
-        <v>577</v>
-      </c>
       <c r="C91" t="s">
-        <v>578</v>
+        <v>573</v>
       </c>
       <c r="D91" t="s">
         <v>54</v>
@@ -6374,13 +6548,13 @@
         <v>253</v>
       </c>
       <c r="H91" t="s">
-        <v>607</v>
+        <v>602</v>
       </c>
       <c r="I91" t="s">
         <v>82</v>
       </c>
       <c r="J91" t="s">
-        <v>579</v>
+        <v>574</v>
       </c>
       <c r="K91" t="s">
         <v>55</v>
@@ -6397,13 +6571,13 @@
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
-        <v>573</v>
+        <v>568</v>
       </c>
       <c r="B92" t="s">
-        <v>580</v>
+        <v>575</v>
       </c>
       <c r="C92" t="s">
-        <v>581</v>
+        <v>576</v>
       </c>
       <c r="D92" t="s">
         <v>54</v>
@@ -6418,7 +6592,7 @@
         <v>253</v>
       </c>
       <c r="H92" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J92" t="s">
         <v>84</v>
@@ -6438,13 +6612,13 @@
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
-        <v>574</v>
+        <v>569</v>
       </c>
       <c r="B93" t="s">
-        <v>582</v>
+        <v>577</v>
       </c>
       <c r="C93" t="s">
-        <v>583</v>
+        <v>578</v>
       </c>
       <c r="D93" t="s">
         <v>54</v>
@@ -6459,7 +6633,7 @@
         <v>253</v>
       </c>
       <c r="H93" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I93" t="s">
         <v>61</v>
@@ -6482,13 +6656,13 @@
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
-        <v>575</v>
+        <v>570</v>
       </c>
       <c r="B94" t="s">
-        <v>584</v>
+        <v>579</v>
       </c>
       <c r="C94" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
       <c r="D94" t="s">
         <v>54</v>
@@ -6503,13 +6677,13 @@
         <v>167</v>
       </c>
       <c r="H94" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I94" t="s">
         <v>61</v>
       </c>
       <c r="J94" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="K94" t="s">
         <v>55</v>
@@ -6526,13 +6700,13 @@
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="B95" t="s">
-        <v>585</v>
+        <v>580</v>
       </c>
       <c r="C95" t="s">
-        <v>586</v>
+        <v>581</v>
       </c>
       <c r="D95" t="s">
         <v>54</v>
@@ -6547,7 +6721,7 @@
         <v>169</v>
       </c>
       <c r="H95" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I95" t="s">
         <v>61</v>
@@ -6570,13 +6744,13 @@
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
-        <v>624</v>
+        <v>619</v>
       </c>
       <c r="B96" t="s">
-        <v>626</v>
+        <v>621</v>
       </c>
       <c r="C96" t="s">
-        <v>627</v>
+        <v>622</v>
       </c>
       <c r="D96" t="s">
         <v>54</v>
@@ -6591,7 +6765,7 @@
         <v>167</v>
       </c>
       <c r="H96" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I96" t="s">
         <v>61</v>
@@ -6614,13 +6788,13 @@
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
-        <v>625</v>
+        <v>620</v>
       </c>
       <c r="B97" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
       <c r="C97" t="s">
-        <v>629</v>
+        <v>624</v>
       </c>
       <c r="D97" t="s">
         <v>54</v>
@@ -6635,13 +6809,13 @@
         <v>167</v>
       </c>
       <c r="H97" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I97" t="s">
         <v>82</v>
       </c>
       <c r="J97" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="K97" t="s">
         <v>55</v>
@@ -6661,7 +6835,7 @@
         <v>63</v>
       </c>
       <c r="B98" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C98" t="s">
         <v>70</v>
@@ -6679,7 +6853,7 @@
         <v>167</v>
       </c>
       <c r="H98" t="s">
-        <v>608</v>
+        <v>603</v>
       </c>
       <c r="I98" t="s">
         <v>103</v>
@@ -6723,7 +6897,7 @@
         <v>167</v>
       </c>
       <c r="H99" t="s">
-        <v>609</v>
+        <v>604</v>
       </c>
       <c r="I99" t="s">
         <v>82</v>
@@ -6749,7 +6923,7 @@
         <v>65</v>
       </c>
       <c r="B100" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C100" t="s">
         <v>73</v>
@@ -6767,7 +6941,7 @@
         <v>167</v>
       </c>
       <c r="H100" t="s">
-        <v>610</v>
+        <v>605</v>
       </c>
       <c r="I100" t="s">
         <v>101</v>
@@ -6796,7 +6970,7 @@
         <v>74</v>
       </c>
       <c r="C101" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D101" t="s">
         <v>85</v>
@@ -6811,7 +6985,7 @@
         <v>167</v>
       </c>
       <c r="H101" t="s">
-        <v>557</v>
+        <v>552</v>
       </c>
       <c r="J101" t="s">
         <v>99</v>
@@ -6852,7 +7026,7 @@
         <v>119</v>
       </c>
       <c r="H102" t="s">
-        <v>552</v>
+        <v>547</v>
       </c>
       <c r="I102" t="s">
         <v>82</v>
@@ -6881,7 +7055,7 @@
         <v>77</v>
       </c>
       <c r="C103" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D103" t="s">
         <v>85</v>
@@ -6896,7 +7070,7 @@
         <v>167</v>
       </c>
       <c r="H103" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="J103" t="s">
         <v>208</v>
@@ -6937,7 +7111,7 @@
         <v>254</v>
       </c>
       <c r="H104" t="s">
-        <v>558</v>
+        <v>553</v>
       </c>
       <c r="I104" t="s">
         <v>82</v>
@@ -7136,13 +7310,13 @@
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
       <c r="B109" t="s">
-        <v>546</v>
+        <v>541</v>
       </c>
       <c r="C109" t="s">
-        <v>547</v>
+        <v>542</v>
       </c>
       <c r="D109" t="s">
         <v>85</v>
@@ -7154,10 +7328,10 @@
         <v>32</v>
       </c>
       <c r="G109" t="s">
-        <v>638</v>
+        <v>633</v>
       </c>
       <c r="H109" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J109" t="s">
         <v>218</v>
@@ -7177,13 +7351,13 @@
     </row>
     <row r="110" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
-        <v>590</v>
+        <v>585</v>
       </c>
       <c r="B110" t="s">
-        <v>598</v>
+        <v>593</v>
       </c>
       <c r="C110" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="D110" t="s">
         <v>85</v>
@@ -7198,7 +7372,7 @@
         <v>167</v>
       </c>
       <c r="H110" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J110" t="s">
         <v>218</v>
@@ -7236,10 +7410,10 @@
         <v>13</v>
       </c>
       <c r="G111" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H111" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J111" t="s">
         <v>218</v>
@@ -7277,10 +7451,10 @@
         <v>13</v>
       </c>
       <c r="G112" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H112" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I112" t="s">
         <v>82</v>
@@ -7321,10 +7495,10 @@
         <v>13</v>
       </c>
       <c r="G113" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H113" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J113" t="s">
         <v>218</v>
@@ -7362,10 +7536,10 @@
         <v>13</v>
       </c>
       <c r="G114" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H114" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I114" t="s">
         <v>82</v>
@@ -7394,7 +7568,7 @@
         <v>193</v>
       </c>
       <c r="C115" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D115" t="s">
         <v>85</v>
@@ -7406,10 +7580,10 @@
         <v>13</v>
       </c>
       <c r="G115" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H115" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I115" t="s">
         <v>82</v>
@@ -7432,13 +7606,13 @@
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="B116" t="s">
         <v>588</v>
       </c>
-      <c r="B116" t="s">
-        <v>593</v>
-      </c>
       <c r="C116" t="s">
-        <v>594</v>
+        <v>589</v>
       </c>
       <c r="D116" t="s">
         <v>85</v>
@@ -7450,10 +7624,10 @@
         <v>13</v>
       </c>
       <c r="G116" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H116" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J116" t="s">
         <v>218</v>
@@ -7473,13 +7647,13 @@
     </row>
     <row r="117" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="B117" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="C117" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="D117" t="s">
         <v>85</v>
@@ -7491,10 +7665,10 @@
         <v>32</v>
       </c>
       <c r="G117" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="H117" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I117" t="s">
         <v>82</v>
@@ -7517,13 +7691,13 @@
     </row>
     <row r="118" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="B118" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="C118" t="s">
-        <v>623</v>
+        <v>618</v>
       </c>
       <c r="D118" t="s">
         <v>85</v>
@@ -7535,10 +7709,10 @@
         <v>13</v>
       </c>
       <c r="G118" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H118" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="J118" t="s">
         <v>218</v>
@@ -7561,7 +7735,7 @@
         <v>181</v>
       </c>
       <c r="B119" t="s">
-        <v>600</v>
+        <v>595</v>
       </c>
       <c r="C119" t="s">
         <v>194</v>
@@ -7576,10 +7750,10 @@
         <v>13</v>
       </c>
       <c r="G119" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H119" t="s">
-        <v>559</v>
+        <v>554</v>
       </c>
       <c r="J119" t="s">
         <v>218</v>
@@ -7617,10 +7791,10 @@
         <v>13</v>
       </c>
       <c r="G120" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H120" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J120" t="s">
         <v>218</v>
@@ -7640,13 +7814,13 @@
     </row>
     <row r="121" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="B121" t="s">
+        <v>586</v>
+      </c>
+      <c r="C121" t="s">
         <v>587</v>
-      </c>
-      <c r="B121" t="s">
-        <v>591</v>
-      </c>
-      <c r="C121" t="s">
-        <v>592</v>
       </c>
       <c r="D121" t="s">
         <v>85</v>
@@ -7658,10 +7832,10 @@
         <v>13</v>
       </c>
       <c r="G121" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H121" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I121" t="s">
         <v>82</v>
@@ -7702,10 +7876,10 @@
         <v>13</v>
       </c>
       <c r="G122" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H122" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J122" t="s">
         <v>218</v>
@@ -7743,10 +7917,10 @@
         <v>13</v>
       </c>
       <c r="G123" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H123" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I123" t="s">
         <v>82</v>
@@ -7775,7 +7949,7 @@
         <v>264</v>
       </c>
       <c r="C124" t="s">
-        <v>633</v>
+        <v>628</v>
       </c>
       <c r="D124" t="s">
         <v>85</v>
@@ -7787,10 +7961,10 @@
         <v>13</v>
       </c>
       <c r="G124" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H124" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I124" t="s">
         <v>265</v>
@@ -7831,10 +8005,10 @@
         <v>13</v>
       </c>
       <c r="G125" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H125" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J125" t="s">
         <v>218</v>
@@ -7860,7 +8034,7 @@
         <v>266</v>
       </c>
       <c r="C126" t="s">
-        <v>632</v>
+        <v>627</v>
       </c>
       <c r="D126" t="s">
         <v>85</v>
@@ -7872,10 +8046,10 @@
         <v>13</v>
       </c>
       <c r="G126" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H126" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I126" t="s">
         <v>82</v>
@@ -7916,10 +8090,10 @@
         <v>13</v>
       </c>
       <c r="G127" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H127" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I127" t="s">
         <v>82</v>
@@ -7942,13 +8116,13 @@
     </row>
     <row r="128" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
       <c r="B128" t="s">
-        <v>615</v>
+        <v>610</v>
       </c>
       <c r="C128" t="s">
-        <v>616</v>
+        <v>611</v>
       </c>
       <c r="D128" t="s">
         <v>85</v>
@@ -7960,10 +8134,10 @@
         <v>13</v>
       </c>
       <c r="G128" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H128" t="s">
-        <v>559</v>
+        <v>554</v>
       </c>
       <c r="I128" t="s">
         <v>61</v>
@@ -7986,13 +8160,13 @@
     </row>
     <row r="129" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="B129" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="C129" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="D129" t="s">
         <v>85</v>
@@ -8004,10 +8178,10 @@
         <v>13</v>
       </c>
       <c r="G129" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H129" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J129" t="s">
         <v>218</v>
@@ -8030,7 +8204,7 @@
         <v>183</v>
       </c>
       <c r="B130" t="s">
-        <v>622</v>
+        <v>617</v>
       </c>
       <c r="C130" t="s">
         <v>198</v>
@@ -8045,10 +8219,10 @@
         <v>13</v>
       </c>
       <c r="G130" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H130" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I130" t="s">
         <v>82</v>
@@ -8089,10 +8263,10 @@
         <v>13</v>
       </c>
       <c r="G131" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H131" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J131" t="s">
         <v>209</v>
@@ -8130,10 +8304,10 @@
         <v>13</v>
       </c>
       <c r="G132" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H132" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J132" t="s">
         <v>218</v>
@@ -8159,7 +8333,7 @@
         <v>205</v>
       </c>
       <c r="C133" t="s">
-        <v>639</v>
+        <v>719</v>
       </c>
       <c r="D133" t="s">
         <v>85</v>
@@ -8215,10 +8389,10 @@
         <v>13</v>
       </c>
       <c r="G134" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H134" t="s">
-        <v>560</v>
+        <v>555</v>
       </c>
       <c r="I134" t="s">
         <v>156</v>
@@ -8259,10 +8433,10 @@
         <v>13</v>
       </c>
       <c r="G135" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H135" t="s">
-        <v>560</v>
+        <v>555</v>
       </c>
       <c r="I135" t="s">
         <v>82</v>
@@ -8291,7 +8465,7 @@
         <v>273</v>
       </c>
       <c r="C136" t="s">
-        <v>276</v>
+        <v>720</v>
       </c>
       <c r="D136" t="s">
         <v>85</v>
@@ -8306,7 +8480,7 @@
         <v>167</v>
       </c>
       <c r="H136" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I136" t="s">
         <v>156</v>
@@ -8329,13 +8503,13 @@
     </row>
     <row r="137" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B137" t="s">
+        <v>279</v>
+      </c>
+      <c r="C137" t="s">
         <v>278</v>
-      </c>
-      <c r="B137" t="s">
-        <v>280</v>
-      </c>
-      <c r="C137" t="s">
-        <v>279</v>
       </c>
       <c r="D137" t="s">
         <v>85</v>
@@ -8350,7 +8524,7 @@
         <v>167</v>
       </c>
       <c r="H137" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J137" t="s">
         <v>218</v>
@@ -8370,13 +8544,13 @@
     </row>
     <row r="138" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B138" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C138" t="s">
-        <v>482</v>
+        <v>717</v>
       </c>
       <c r="D138" t="s">
         <v>85</v>
@@ -8388,7 +8562,7 @@
         <v>13</v>
       </c>
       <c r="G138" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H138" t="s">
         <v>233</v>
@@ -8411,13 +8585,13 @@
     </row>
     <row r="139" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B139" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C139" t="s">
-        <v>351</v>
+        <v>718</v>
       </c>
       <c r="D139" t="s">
         <v>85</v>
@@ -8432,7 +8606,7 @@
         <v>169</v>
       </c>
       <c r="H139" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J139" t="s">
         <v>104</v>
@@ -8452,13 +8626,13 @@
     </row>
     <row r="140" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B140" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C140" t="s">
-        <v>483</v>
+        <v>716</v>
       </c>
       <c r="D140" t="s">
         <v>85</v>
@@ -8470,7 +8644,7 @@
         <v>13</v>
       </c>
       <c r="G140" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H140" t="s">
         <v>233</v>
@@ -8493,13 +8667,13 @@
     </row>
     <row r="141" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B141" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C141" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D141" t="s">
         <v>85</v>
@@ -8511,10 +8685,10 @@
         <v>13</v>
       </c>
       <c r="G141" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H141" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="I141" t="s">
         <v>156</v>
@@ -8537,13 +8711,13 @@
     </row>
     <row r="142" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B142" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C142" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D142" t="s">
         <v>85</v>
@@ -8558,7 +8732,7 @@
         <v>167</v>
       </c>
       <c r="H142" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J142" t="s">
         <v>102</v>
@@ -8578,13 +8752,13 @@
     </row>
     <row r="143" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B143" t="s">
+        <v>356</v>
+      </c>
+      <c r="C143" t="s">
         <v>358</v>
-      </c>
-      <c r="C143" t="s">
-        <v>360</v>
       </c>
       <c r="D143" t="s">
         <v>85</v>
@@ -8596,10 +8770,10 @@
         <v>13</v>
       </c>
       <c r="G143" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H143" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="I143" t="s">
         <v>82</v>
@@ -8622,13 +8796,13 @@
     </row>
     <row r="144" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B144" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C144" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="D144" t="s">
         <v>85</v>
@@ -8640,10 +8814,10 @@
         <v>13</v>
       </c>
       <c r="G144" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="H144" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="I144" t="s">
         <v>82</v>
@@ -8666,13 +8840,13 @@
     </row>
     <row r="145" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B145" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C145" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D145" t="s">
         <v>85</v>
@@ -8687,7 +8861,7 @@
         <v>169</v>
       </c>
       <c r="H145" t="s">
-        <v>563</v>
+        <v>558</v>
       </c>
       <c r="J145" t="s">
         <v>102</v>
@@ -8707,13 +8881,13 @@
     </row>
     <row r="146" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B146" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C146" t="s">
-        <v>368</v>
+        <v>687</v>
       </c>
       <c r="D146" t="s">
         <v>85</v>
@@ -8725,7 +8899,7 @@
         <v>13</v>
       </c>
       <c r="G146" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H146" t="s">
         <v>120</v>
@@ -8748,13 +8922,13 @@
     </row>
     <row r="147" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B147" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C147" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="D147" t="s">
         <v>85</v>
@@ -8766,16 +8940,16 @@
         <v>13</v>
       </c>
       <c r="G147" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H147" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="I147" t="s">
         <v>82</v>
       </c>
       <c r="J147" t="s">
-        <v>172</v>
+        <v>104</v>
       </c>
       <c r="K147" t="s">
         <v>55</v>
@@ -8792,13 +8966,13 @@
     </row>
     <row r="148" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B148" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C148" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="D148" t="s">
         <v>85</v>
@@ -8810,10 +8984,10 @@
         <v>32</v>
       </c>
       <c r="G148" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="H148" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="I148" t="s">
         <v>82</v>
@@ -8836,13 +9010,13 @@
     </row>
     <row r="149" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B149" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="C149" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="D149" t="s">
         <v>85</v>
@@ -8854,7 +9028,7 @@
         <v>13</v>
       </c>
       <c r="G149" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="H149" t="s">
         <v>238</v>
@@ -8863,7 +9037,7 @@
         <v>82</v>
       </c>
       <c r="J149" t="s">
-        <v>211</v>
+        <v>104</v>
       </c>
       <c r="K149" t="s">
         <v>55</v>
@@ -8880,13 +9054,13 @@
     </row>
     <row r="150" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B150" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="C150" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="D150" t="s">
         <v>85</v>
@@ -8898,7 +9072,7 @@
         <v>13</v>
       </c>
       <c r="G150" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H150" t="s">
         <v>238</v>
@@ -8907,7 +9081,7 @@
         <v>82</v>
       </c>
       <c r="J150" t="s">
-        <v>172</v>
+        <v>104</v>
       </c>
       <c r="K150" t="s">
         <v>55</v>
@@ -8924,13 +9098,13 @@
     </row>
     <row r="151" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B151" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="C151" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="D151" t="s">
         <v>85</v>
@@ -8942,7 +9116,7 @@
         <v>13</v>
       </c>
       <c r="G151" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H151" t="s">
         <v>238</v>
@@ -8951,7 +9125,7 @@
         <v>82</v>
       </c>
       <c r="J151" t="s">
-        <v>172</v>
+        <v>104</v>
       </c>
       <c r="K151" t="s">
         <v>55</v>
@@ -8968,13 +9142,13 @@
     </row>
     <row r="152" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B152" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="C152" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="D152" t="s">
         <v>85</v>
@@ -8989,13 +9163,13 @@
         <v>167</v>
       </c>
       <c r="H152" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="I152" t="s">
         <v>156</v>
       </c>
       <c r="J152" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="K152" t="s">
         <v>55</v>
@@ -9012,13 +9186,13 @@
     </row>
     <row r="153" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="B153" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="C153" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="D153" t="s">
         <v>85</v>
@@ -9033,13 +9207,13 @@
         <v>253</v>
       </c>
       <c r="H153" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="I153" t="s">
         <v>156</v>
       </c>
       <c r="J153" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="K153" t="s">
         <v>55</v>
@@ -9056,13 +9230,13 @@
     </row>
     <row r="154" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B154" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="C154" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="D154" t="s">
         <v>85</v>
@@ -9077,7 +9251,7 @@
         <v>167</v>
       </c>
       <c r="H154" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="J154" t="s">
         <v>172</v>
@@ -9097,13 +9271,13 @@
     </row>
     <row r="155" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="B155" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="C155" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="D155" t="s">
         <v>85</v>
@@ -9118,7 +9292,7 @@
         <v>119</v>
       </c>
       <c r="H155" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="I155" t="s">
         <v>82</v>
@@ -9141,13 +9315,13 @@
     </row>
     <row r="156" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="B156" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
       <c r="C156" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="D156" t="s">
         <v>85</v>
@@ -9162,7 +9336,7 @@
         <v>167</v>
       </c>
       <c r="H156" t="s">
-        <v>611</v>
+        <v>606</v>
       </c>
       <c r="I156" t="s">
         <v>82</v>
@@ -9185,13 +9359,13 @@
     </row>
     <row r="157" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="B157" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="C157" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="D157" t="s">
         <v>85</v>
@@ -9206,7 +9380,7 @@
         <v>167</v>
       </c>
       <c r="H157" t="s">
-        <v>567</v>
+        <v>562</v>
       </c>
       <c r="J157" t="s">
         <v>211</v>
@@ -9226,13 +9400,13 @@
     </row>
     <row r="158" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
-        <v>532</v>
+        <v>527</v>
       </c>
       <c r="B158" t="s">
-        <v>630</v>
+        <v>625</v>
       </c>
       <c r="C158" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="D158" t="s">
         <v>85</v>
@@ -9270,13 +9444,13 @@
     </row>
     <row r="159" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
-        <v>533</v>
+        <v>528</v>
       </c>
       <c r="B159" t="s">
-        <v>539</v>
+        <v>534</v>
       </c>
       <c r="C159" t="s">
-        <v>540</v>
+        <v>535</v>
       </c>
       <c r="D159" t="s">
         <v>85</v>
@@ -9291,7 +9465,7 @@
         <v>167</v>
       </c>
       <c r="H159" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I159" t="s">
         <v>82</v>
@@ -9314,13 +9488,13 @@
     </row>
     <row r="160" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
-        <v>534</v>
+        <v>529</v>
       </c>
       <c r="B160" t="s">
-        <v>541</v>
+        <v>536</v>
       </c>
       <c r="C160" t="s">
-        <v>542</v>
+        <v>537</v>
       </c>
       <c r="D160" t="s">
         <v>85</v>
@@ -9332,10 +9506,10 @@
         <v>13</v>
       </c>
       <c r="G160" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H160" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="I160" t="s">
         <v>82</v>
@@ -9358,13 +9532,13 @@
     </row>
     <row r="161" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="B161" t="s">
+        <v>538</v>
+      </c>
+      <c r="C161" t="s">
         <v>535</v>
-      </c>
-      <c r="B161" t="s">
-        <v>543</v>
-      </c>
-      <c r="C161" t="s">
-        <v>540</v>
       </c>
       <c r="D161" t="s">
         <v>85</v>
@@ -9379,7 +9553,7 @@
         <v>167</v>
       </c>
       <c r="H161" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I161" t="s">
         <v>82</v>
@@ -9402,13 +9576,13 @@
     </row>
     <row r="162" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
-        <v>536</v>
+        <v>531</v>
       </c>
       <c r="B162" t="s">
-        <v>544</v>
+        <v>539</v>
       </c>
       <c r="C162" t="s">
-        <v>545</v>
+        <v>540</v>
       </c>
       <c r="D162" t="s">
         <v>85</v>
@@ -9423,10 +9597,10 @@
         <v>167</v>
       </c>
       <c r="H162" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J162" t="s">
-        <v>571</v>
+        <v>566</v>
       </c>
       <c r="K162" t="s">
         <v>55</v>
@@ -9443,13 +9617,13 @@
     </row>
     <row r="163" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
-        <v>538</v>
+        <v>533</v>
       </c>
       <c r="B163" t="s">
-        <v>548</v>
+        <v>543</v>
       </c>
       <c r="C163" t="s">
-        <v>549</v>
+        <v>544</v>
       </c>
       <c r="D163" t="s">
         <v>85</v>
@@ -9484,13 +9658,13 @@
     </row>
     <row r="164" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="s">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="B164" t="s">
-        <v>595</v>
+        <v>590</v>
       </c>
       <c r="C164" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="D164" t="s">
         <v>85</v>
@@ -9502,10 +9676,10 @@
         <v>32</v>
       </c>
       <c r="G164" t="s">
-        <v>597</v>
+        <v>592</v>
       </c>
       <c r="H164" t="s">
-        <v>560</v>
+        <v>555</v>
       </c>
       <c r="I164" t="s">
         <v>82</v>
@@ -9528,13 +9702,13 @@
     </row>
     <row r="165" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="s">
-        <v>613</v>
+        <v>608</v>
       </c>
       <c r="B165" t="s">
-        <v>620</v>
+        <v>615</v>
       </c>
       <c r="C165" t="s">
-        <v>617</v>
+        <v>612</v>
       </c>
       <c r="D165" t="s">
         <v>85</v>
@@ -9546,10 +9720,10 @@
         <v>13</v>
       </c>
       <c r="G165" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H165" t="s">
-        <v>618</v>
+        <v>613</v>
       </c>
       <c r="I165" t="s">
         <v>156</v>
@@ -9572,13 +9746,13 @@
     </row>
     <row r="166" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="s">
+        <v>609</v>
+      </c>
+      <c r="B166" t="s">
         <v>614</v>
       </c>
-      <c r="B166" t="s">
-        <v>619</v>
-      </c>
       <c r="C166" t="s">
-        <v>621</v>
+        <v>616</v>
       </c>
       <c r="D166" t="s">
         <v>85</v>
@@ -9590,10 +9764,10 @@
         <v>13</v>
       </c>
       <c r="G166" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H166" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J166" t="s">
         <v>218</v>
@@ -9613,13 +9787,13 @@
     </row>
     <row r="167" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A167" s="1" t="s">
-        <v>640</v>
+        <v>634</v>
       </c>
       <c r="B167" t="s">
-        <v>644</v>
+        <v>638</v>
       </c>
       <c r="C167" t="s">
-        <v>645</v>
+        <v>639</v>
       </c>
       <c r="D167" t="s">
         <v>85</v>
@@ -9634,7 +9808,7 @@
         <v>167</v>
       </c>
       <c r="H167" t="s">
-        <v>564</v>
+        <v>559</v>
       </c>
       <c r="I167" t="s">
         <v>82</v>
@@ -9657,13 +9831,13 @@
     </row>
     <row r="168" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A168" s="1" t="s">
-        <v>641</v>
+        <v>635</v>
       </c>
       <c r="B168" t="s">
-        <v>646</v>
+        <v>640</v>
       </c>
       <c r="C168" t="s">
-        <v>683</v>
+        <v>676</v>
       </c>
       <c r="D168" t="s">
         <v>85</v>
@@ -9698,13 +9872,13 @@
     </row>
     <row r="169" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A169" s="1" t="s">
+        <v>636</v>
+      </c>
+      <c r="B169" t="s">
+        <v>641</v>
+      </c>
+      <c r="C169" t="s">
         <v>642</v>
-      </c>
-      <c r="B169" t="s">
-        <v>647</v>
-      </c>
-      <c r="C169" t="s">
-        <v>648</v>
       </c>
       <c r="D169" t="s">
         <v>85</v>
@@ -9719,13 +9893,13 @@
         <v>167</v>
       </c>
       <c r="H169" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="I169" t="s">
         <v>61</v>
       </c>
       <c r="J169" t="s">
-        <v>661</v>
+        <v>655</v>
       </c>
       <c r="K169" t="s">
         <v>55</v>
@@ -9742,13 +9916,13 @@
     </row>
     <row r="170" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A170" s="1" t="s">
+        <v>637</v>
+      </c>
+      <c r="B170" t="s">
+        <v>670</v>
+      </c>
+      <c r="C170" t="s">
         <v>643</v>
-      </c>
-      <c r="B170" t="s">
-        <v>677</v>
-      </c>
-      <c r="C170" t="s">
-        <v>649</v>
       </c>
       <c r="D170" t="s">
         <v>85</v>
@@ -9763,13 +9937,13 @@
         <v>167</v>
       </c>
       <c r="H170" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="I170" t="s">
         <v>82</v>
       </c>
       <c r="J170" t="s">
-        <v>650</v>
+        <v>644</v>
       </c>
       <c r="K170" t="s">
         <v>55</v>
@@ -9786,13 +9960,13 @@
     </row>
     <row r="171" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A171" s="1" t="s">
-        <v>652</v>
+        <v>646</v>
       </c>
       <c r="B171" t="s">
-        <v>550</v>
+        <v>545</v>
       </c>
       <c r="C171" t="s">
-        <v>656</v>
+        <v>650</v>
       </c>
       <c r="D171" t="s">
         <v>54</v>
@@ -9827,13 +10001,13 @@
     </row>
     <row r="172" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A172" s="1" t="s">
-        <v>653</v>
+        <v>647</v>
       </c>
       <c r="B172" t="s">
-        <v>657</v>
+        <v>651</v>
       </c>
       <c r="C172" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="D172" t="s">
         <v>54</v>
@@ -9845,13 +10019,13 @@
         <v>13</v>
       </c>
       <c r="G172" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H172" t="s">
         <v>234</v>
       </c>
       <c r="J172" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="K172" t="s">
         <v>55</v>
@@ -9868,13 +10042,13 @@
     </row>
     <row r="173" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A173" s="1" t="s">
-        <v>654</v>
+        <v>648</v>
       </c>
       <c r="B173" t="s">
-        <v>658</v>
+        <v>652</v>
       </c>
       <c r="C173" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="D173" t="s">
         <v>54</v>
@@ -9886,13 +10060,13 @@
         <v>13</v>
       </c>
       <c r="G173" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H173" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="J173" t="s">
-        <v>660</v>
+        <v>654</v>
       </c>
       <c r="K173" t="s">
         <v>55</v>
@@ -9909,13 +10083,13 @@
     </row>
     <row r="174" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A174" s="1" t="s">
-        <v>651</v>
+        <v>645</v>
       </c>
       <c r="B174" t="s">
-        <v>659</v>
+        <v>653</v>
       </c>
       <c r="C174" t="s">
-        <v>662</v>
+        <v>688</v>
       </c>
       <c r="D174" t="s">
         <v>54</v>
@@ -9930,13 +10104,13 @@
         <v>167</v>
       </c>
       <c r="H174" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I174" t="s">
         <v>82</v>
       </c>
       <c r="J174" t="s">
-        <v>650</v>
+        <v>644</v>
       </c>
       <c r="K174" t="s">
         <v>55</v>
@@ -9953,13 +10127,13 @@
     </row>
     <row r="175" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A175" s="1" t="s">
-        <v>655</v>
+        <v>649</v>
       </c>
       <c r="B175" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
       <c r="C175" t="s">
-        <v>664</v>
+        <v>657</v>
       </c>
       <c r="D175" t="s">
         <v>54</v>
@@ -9977,7 +10151,7 @@
         <v>153</v>
       </c>
       <c r="J175" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="K175" t="s">
         <v>55</v>
@@ -9994,13 +10168,13 @@
     </row>
     <row r="176" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A176" s="1" t="s">
-        <v>665</v>
+        <v>658</v>
       </c>
       <c r="B176" t="s">
-        <v>669</v>
+        <v>662</v>
       </c>
       <c r="C176" t="s">
-        <v>670</v>
+        <v>663</v>
       </c>
       <c r="D176" t="s">
         <v>54</v>
@@ -10015,7 +10189,7 @@
         <v>167</v>
       </c>
       <c r="H176" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="I176" t="s">
         <v>166</v>
@@ -10038,13 +10212,13 @@
     </row>
     <row r="177" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A177" s="1" t="s">
-        <v>666</v>
+        <v>659</v>
       </c>
       <c r="B177" t="s">
-        <v>671</v>
+        <v>664</v>
       </c>
       <c r="C177" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="D177" t="s">
         <v>54</v>
@@ -10059,7 +10233,7 @@
         <v>167</v>
       </c>
       <c r="H177" t="s">
-        <v>672</v>
+        <v>665</v>
       </c>
       <c r="I177" t="s">
         <v>156</v>
@@ -10082,13 +10256,13 @@
     </row>
     <row r="178" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A178" s="1" t="s">
-        <v>667</v>
+        <v>660</v>
       </c>
       <c r="B178" t="s">
-        <v>673</v>
+        <v>666</v>
       </c>
       <c r="C178" t="s">
-        <v>682</v>
+        <v>675</v>
       </c>
       <c r="D178" t="s">
         <v>54</v>
@@ -10100,16 +10274,16 @@
         <v>32</v>
       </c>
       <c r="G178" t="s">
-        <v>674</v>
+        <v>667</v>
       </c>
       <c r="H178" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I178" t="s">
         <v>82</v>
       </c>
       <c r="J178" t="s">
-        <v>650</v>
+        <v>644</v>
       </c>
       <c r="K178" t="s">
         <v>55</v>
@@ -10126,13 +10300,13 @@
     </row>
     <row r="179" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A179" s="1" t="s">
+        <v>661</v>
+      </c>
+      <c r="B179" t="s">
         <v>668</v>
       </c>
-      <c r="B179" t="s">
-        <v>675</v>
-      </c>
       <c r="C179" t="s">
-        <v>676</v>
+        <v>669</v>
       </c>
       <c r="D179" t="s">
         <v>54</v>
@@ -10147,7 +10321,7 @@
         <v>167</v>
       </c>
       <c r="H179" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="I179" t="s">
         <v>61</v>
@@ -10170,13 +10344,13 @@
     </row>
     <row r="180" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A180" s="1" t="s">
+        <v>671</v>
+      </c>
+      <c r="B180" t="s">
+        <v>677</v>
+      </c>
+      <c r="C180" t="s">
         <v>678</v>
-      </c>
-      <c r="B180" t="s">
-        <v>684</v>
-      </c>
-      <c r="C180" t="s">
-        <v>685</v>
       </c>
       <c r="D180" t="s">
         <v>85</v>
@@ -10188,16 +10362,16 @@
         <v>13</v>
       </c>
       <c r="G180" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H180" t="s">
-        <v>686</v>
+        <v>679</v>
       </c>
       <c r="I180" t="s">
         <v>60</v>
       </c>
       <c r="J180" t="s">
-        <v>571</v>
+        <v>566</v>
       </c>
       <c r="K180" t="s">
         <v>55</v>
@@ -10214,13 +10388,13 @@
     </row>
     <row r="181" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A181" s="1" t="s">
+        <v>673</v>
+      </c>
+      <c r="B181" t="s">
         <v>680</v>
       </c>
-      <c r="B181" t="s">
-        <v>687</v>
-      </c>
       <c r="C181" t="s">
-        <v>688</v>
+        <v>681</v>
       </c>
       <c r="D181" t="s">
         <v>85</v>
@@ -10232,16 +10406,16 @@
         <v>13</v>
       </c>
       <c r="G181" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H181" t="s">
-        <v>567</v>
+        <v>562</v>
       </c>
       <c r="I181" t="s">
         <v>82</v>
       </c>
       <c r="J181" t="s">
-        <v>172</v>
+        <v>104</v>
       </c>
       <c r="K181" t="s">
         <v>55</v>
@@ -10258,13 +10432,13 @@
     </row>
     <row r="182" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A182" s="1" t="s">
-        <v>679</v>
+        <v>672</v>
       </c>
       <c r="B182" t="s">
-        <v>689</v>
+        <v>682</v>
       </c>
       <c r="C182" t="s">
-        <v>690</v>
+        <v>683</v>
       </c>
       <c r="D182" t="s">
         <v>85</v>
@@ -10279,7 +10453,7 @@
         <v>167</v>
       </c>
       <c r="H182" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="I182" t="s">
         <v>82</v>
@@ -10302,13 +10476,13 @@
     </row>
     <row r="183" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A183" s="1" t="s">
-        <v>681</v>
+        <v>674</v>
       </c>
       <c r="B183" t="s">
-        <v>691</v>
+        <v>684</v>
       </c>
       <c r="C183" t="s">
-        <v>692</v>
+        <v>685</v>
       </c>
       <c r="D183" t="s">
         <v>85</v>
@@ -10323,7 +10497,7 @@
         <v>167</v>
       </c>
       <c r="H183" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I183" t="s">
         <v>82</v>
@@ -10341,6 +10515,829 @@
         <v>15</v>
       </c>
       <c r="N183" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="184" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A184" s="1" t="s">
+        <v>700</v>
+      </c>
+      <c r="B184" t="s">
+        <v>478</v>
+      </c>
+      <c r="C184" t="s">
+        <v>709</v>
+      </c>
+      <c r="D184" t="s">
+        <v>85</v>
+      </c>
+      <c r="E184" t="s">
+        <v>58</v>
+      </c>
+      <c r="F184" t="s">
+        <v>13</v>
+      </c>
+      <c r="G184" t="s">
+        <v>307</v>
+      </c>
+      <c r="H184" t="s">
+        <v>233</v>
+      </c>
+      <c r="J184" t="s">
+        <v>104</v>
+      </c>
+      <c r="K184" t="s">
+        <v>55</v>
+      </c>
+      <c r="L184" t="s">
+        <v>14</v>
+      </c>
+      <c r="M184" t="s">
+        <v>15</v>
+      </c>
+      <c r="N184" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="185" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A185" s="1" t="s">
+        <v>701</v>
+      </c>
+      <c r="B185" t="s">
+        <v>710</v>
+      </c>
+      <c r="C185" t="s">
+        <v>711</v>
+      </c>
+      <c r="D185" t="s">
+        <v>85</v>
+      </c>
+      <c r="E185" t="s">
+        <v>58</v>
+      </c>
+      <c r="F185" t="s">
+        <v>13</v>
+      </c>
+      <c r="G185" t="s">
+        <v>167</v>
+      </c>
+      <c r="H185" t="s">
+        <v>597</v>
+      </c>
+      <c r="J185" t="s">
+        <v>218</v>
+      </c>
+      <c r="K185" t="s">
+        <v>56</v>
+      </c>
+      <c r="L185" t="s">
+        <v>14</v>
+      </c>
+      <c r="M185" t="s">
+        <v>15</v>
+      </c>
+      <c r="N185" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="186" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A186" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="B186" t="s">
+        <v>712</v>
+      </c>
+      <c r="C186" t="s">
+        <v>713</v>
+      </c>
+      <c r="D186" t="s">
+        <v>85</v>
+      </c>
+      <c r="E186" t="s">
+        <v>58</v>
+      </c>
+      <c r="F186" t="s">
+        <v>13</v>
+      </c>
+      <c r="G186" t="s">
+        <v>307</v>
+      </c>
+      <c r="H186" t="s">
+        <v>233</v>
+      </c>
+      <c r="J186" t="s">
+        <v>104</v>
+      </c>
+      <c r="K186" t="s">
+        <v>55</v>
+      </c>
+      <c r="L186" t="s">
+        <v>14</v>
+      </c>
+      <c r="M186" t="s">
+        <v>15</v>
+      </c>
+      <c r="N186" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="187" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A187" s="1" t="s">
+        <v>703</v>
+      </c>
+      <c r="B187" t="s">
+        <v>714</v>
+      </c>
+      <c r="C187" t="s">
+        <v>715</v>
+      </c>
+      <c r="D187" t="s">
+        <v>85</v>
+      </c>
+      <c r="E187" t="s">
+        <v>58</v>
+      </c>
+      <c r="F187" t="s">
+        <v>13</v>
+      </c>
+      <c r="G187" t="s">
+        <v>307</v>
+      </c>
+      <c r="H187" t="s">
+        <v>233</v>
+      </c>
+      <c r="J187" t="s">
+        <v>104</v>
+      </c>
+      <c r="K187" t="s">
+        <v>55</v>
+      </c>
+      <c r="L187" t="s">
+        <v>14</v>
+      </c>
+      <c r="M187" t="s">
+        <v>15</v>
+      </c>
+      <c r="N187" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="188" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A188" s="1" t="s">
+        <v>704</v>
+      </c>
+      <c r="B188" t="s">
+        <v>721</v>
+      </c>
+      <c r="C188" t="s">
+        <v>722</v>
+      </c>
+      <c r="D188" t="s">
+        <v>85</v>
+      </c>
+      <c r="E188" t="s">
+        <v>33</v>
+      </c>
+      <c r="F188" t="s">
+        <v>13</v>
+      </c>
+      <c r="G188" t="s">
+        <v>167</v>
+      </c>
+      <c r="H188" t="s">
+        <v>233</v>
+      </c>
+      <c r="I188" t="s">
+        <v>156</v>
+      </c>
+      <c r="J188" t="s">
+        <v>381</v>
+      </c>
+      <c r="K188" t="s">
+        <v>55</v>
+      </c>
+      <c r="L188" t="s">
+        <v>14</v>
+      </c>
+      <c r="M188" t="s">
+        <v>15</v>
+      </c>
+      <c r="N188" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="189" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A189" s="1" t="s">
+        <v>705</v>
+      </c>
+      <c r="B189" t="s">
+        <v>723</v>
+      </c>
+      <c r="C189" t="s">
+        <v>724</v>
+      </c>
+      <c r="D189" t="s">
+        <v>85</v>
+      </c>
+      <c r="E189" t="s">
+        <v>58</v>
+      </c>
+      <c r="F189" t="s">
+        <v>32</v>
+      </c>
+      <c r="G189" t="s">
+        <v>254</v>
+      </c>
+      <c r="H189" t="s">
+        <v>234</v>
+      </c>
+      <c r="J189" t="s">
+        <v>102</v>
+      </c>
+      <c r="K189" t="s">
+        <v>55</v>
+      </c>
+      <c r="L189" t="s">
+        <v>14</v>
+      </c>
+      <c r="M189" t="s">
+        <v>15</v>
+      </c>
+      <c r="N189" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="190" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A190" s="1" t="s">
+        <v>706</v>
+      </c>
+      <c r="B190" t="s">
+        <v>725</v>
+      </c>
+      <c r="C190" t="s">
+        <v>726</v>
+      </c>
+      <c r="D190" t="s">
+        <v>85</v>
+      </c>
+      <c r="E190" t="s">
+        <v>58</v>
+      </c>
+      <c r="F190" t="s">
+        <v>32</v>
+      </c>
+      <c r="G190" t="s">
+        <v>515</v>
+      </c>
+      <c r="H190" t="s">
+        <v>234</v>
+      </c>
+      <c r="J190" t="s">
+        <v>102</v>
+      </c>
+      <c r="K190" t="s">
+        <v>55</v>
+      </c>
+      <c r="L190" t="s">
+        <v>14</v>
+      </c>
+      <c r="M190" t="s">
+        <v>15</v>
+      </c>
+      <c r="N190" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="191" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A191" s="1" t="s">
+        <v>707</v>
+      </c>
+      <c r="B191" t="s">
+        <v>727</v>
+      </c>
+      <c r="C191" t="s">
+        <v>728</v>
+      </c>
+      <c r="D191" t="s">
+        <v>85</v>
+      </c>
+      <c r="E191" t="s">
+        <v>33</v>
+      </c>
+      <c r="F191" t="s">
+        <v>13</v>
+      </c>
+      <c r="G191" t="s">
+        <v>167</v>
+      </c>
+      <c r="H191" t="s">
+        <v>233</v>
+      </c>
+      <c r="I191" t="s">
+        <v>156</v>
+      </c>
+      <c r="J191" t="s">
+        <v>391</v>
+      </c>
+      <c r="K191" t="s">
+        <v>55</v>
+      </c>
+      <c r="L191" t="s">
+        <v>14</v>
+      </c>
+      <c r="M191" t="s">
+        <v>15</v>
+      </c>
+      <c r="N191" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="192" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A192" s="1" t="s">
+        <v>708</v>
+      </c>
+      <c r="B192" t="s">
+        <v>729</v>
+      </c>
+      <c r="C192" t="s">
+        <v>730</v>
+      </c>
+      <c r="D192" t="s">
+        <v>85</v>
+      </c>
+      <c r="E192" t="s">
+        <v>33</v>
+      </c>
+      <c r="F192" t="s">
+        <v>32</v>
+      </c>
+      <c r="G192" t="s">
+        <v>515</v>
+      </c>
+      <c r="H192" t="s">
+        <v>317</v>
+      </c>
+      <c r="J192" t="s">
+        <v>218</v>
+      </c>
+      <c r="K192" t="s">
+        <v>55</v>
+      </c>
+      <c r="L192" t="s">
+        <v>14</v>
+      </c>
+      <c r="M192" t="s">
+        <v>15</v>
+      </c>
+      <c r="N192" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="193" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A193" s="1" t="s">
+        <v>689</v>
+      </c>
+      <c r="B193" t="s">
+        <v>731</v>
+      </c>
+      <c r="C193" t="s">
+        <v>732</v>
+      </c>
+      <c r="D193" t="s">
+        <v>54</v>
+      </c>
+      <c r="E193" t="s">
+        <v>33</v>
+      </c>
+      <c r="F193" t="s">
+        <v>13</v>
+      </c>
+      <c r="G193" t="s">
+        <v>167</v>
+      </c>
+      <c r="J193" t="s">
+        <v>208</v>
+      </c>
+      <c r="K193" t="s">
+        <v>55</v>
+      </c>
+      <c r="L193" t="s">
+        <v>14</v>
+      </c>
+      <c r="M193" t="s">
+        <v>15</v>
+      </c>
+      <c r="N193" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="194" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A194" s="1" t="s">
+        <v>690</v>
+      </c>
+      <c r="B194" t="s">
+        <v>733</v>
+      </c>
+      <c r="C194" t="s">
+        <v>734</v>
+      </c>
+      <c r="D194" t="s">
+        <v>54</v>
+      </c>
+      <c r="E194" t="s">
+        <v>33</v>
+      </c>
+      <c r="F194" t="s">
+        <v>13</v>
+      </c>
+      <c r="G194" t="s">
+        <v>167</v>
+      </c>
+      <c r="I194" t="s">
+        <v>61</v>
+      </c>
+      <c r="J194" t="s">
+        <v>208</v>
+      </c>
+      <c r="K194" t="s">
+        <v>55</v>
+      </c>
+      <c r="L194" t="s">
+        <v>14</v>
+      </c>
+      <c r="M194" t="s">
+        <v>15</v>
+      </c>
+      <c r="N194" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="195" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A195" s="1" t="s">
+        <v>691</v>
+      </c>
+      <c r="B195" t="s">
+        <v>735</v>
+      </c>
+      <c r="C195" t="s">
+        <v>511</v>
+      </c>
+      <c r="D195" t="s">
+        <v>54</v>
+      </c>
+      <c r="E195" t="s">
+        <v>33</v>
+      </c>
+      <c r="F195" t="s">
+        <v>13</v>
+      </c>
+      <c r="G195" t="s">
+        <v>119</v>
+      </c>
+      <c r="I195" t="s">
+        <v>61</v>
+      </c>
+      <c r="J195" t="s">
+        <v>209</v>
+      </c>
+      <c r="K195" t="s">
+        <v>55</v>
+      </c>
+      <c r="L195" t="s">
+        <v>14</v>
+      </c>
+      <c r="M195" t="s">
+        <v>15</v>
+      </c>
+      <c r="N195" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="196" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A196" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="B196" t="s">
+        <v>736</v>
+      </c>
+      <c r="C196" t="s">
+        <v>742</v>
+      </c>
+      <c r="D196" t="s">
+        <v>54</v>
+      </c>
+      <c r="E196" t="s">
+        <v>33</v>
+      </c>
+      <c r="F196" t="s">
+        <v>32</v>
+      </c>
+      <c r="G196" t="s">
+        <v>741</v>
+      </c>
+      <c r="H196" t="s">
+        <v>120</v>
+      </c>
+      <c r="J196" t="s">
+        <v>446</v>
+      </c>
+      <c r="K196" t="s">
+        <v>55</v>
+      </c>
+      <c r="L196" t="s">
+        <v>14</v>
+      </c>
+      <c r="M196" t="s">
+        <v>15</v>
+      </c>
+      <c r="N196" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="197" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A197" s="1" t="s">
+        <v>693</v>
+      </c>
+      <c r="B197" t="s">
+        <v>747</v>
+      </c>
+      <c r="D197" t="s">
+        <v>54</v>
+      </c>
+      <c r="E197" t="s">
+        <v>33</v>
+      </c>
+      <c r="F197" t="s">
+        <v>13</v>
+      </c>
+      <c r="G197" t="s">
+        <v>167</v>
+      </c>
+      <c r="H197" t="s">
+        <v>233</v>
+      </c>
+      <c r="I197" t="s">
+        <v>61</v>
+      </c>
+      <c r="J197" t="s">
+        <v>208</v>
+      </c>
+      <c r="K197" t="s">
+        <v>55</v>
+      </c>
+      <c r="L197" t="s">
+        <v>14</v>
+      </c>
+      <c r="M197" t="s">
+        <v>15</v>
+      </c>
+      <c r="N197" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="198" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A198" s="1" t="s">
+        <v>694</v>
+      </c>
+      <c r="B198" t="s">
+        <v>737</v>
+      </c>
+      <c r="C198" t="s">
+        <v>743</v>
+      </c>
+      <c r="D198" t="s">
+        <v>54</v>
+      </c>
+      <c r="E198" t="s">
+        <v>33</v>
+      </c>
+      <c r="F198" t="s">
+        <v>32</v>
+      </c>
+      <c r="G198" t="s">
+        <v>741</v>
+      </c>
+      <c r="H198" t="s">
+        <v>120</v>
+      </c>
+      <c r="J198" t="s">
+        <v>446</v>
+      </c>
+      <c r="K198" t="s">
+        <v>55</v>
+      </c>
+      <c r="L198" t="s">
+        <v>14</v>
+      </c>
+      <c r="M198" t="s">
+        <v>15</v>
+      </c>
+      <c r="N198" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="199" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A199" s="1" t="s">
+        <v>695</v>
+      </c>
+      <c r="B199" t="s">
+        <v>738</v>
+      </c>
+      <c r="C199" t="s">
+        <v>744</v>
+      </c>
+      <c r="D199" t="s">
+        <v>54</v>
+      </c>
+      <c r="E199" t="s">
+        <v>33</v>
+      </c>
+      <c r="F199" t="s">
+        <v>32</v>
+      </c>
+      <c r="G199" t="s">
+        <v>741</v>
+      </c>
+      <c r="H199" t="s">
+        <v>371</v>
+      </c>
+      <c r="J199" t="s">
+        <v>446</v>
+      </c>
+      <c r="K199" t="s">
+        <v>55</v>
+      </c>
+      <c r="L199" t="s">
+        <v>14</v>
+      </c>
+      <c r="M199" t="s">
+        <v>15</v>
+      </c>
+      <c r="N199" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="200" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A200" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="B200" t="s">
+        <v>748</v>
+      </c>
+      <c r="C200" t="s">
+        <v>749</v>
+      </c>
+      <c r="D200" t="s">
+        <v>54</v>
+      </c>
+      <c r="E200" t="s">
+        <v>133</v>
+      </c>
+      <c r="F200" t="s">
+        <v>32</v>
+      </c>
+      <c r="G200" t="s">
+        <v>167</v>
+      </c>
+      <c r="H200" t="s">
+        <v>153</v>
+      </c>
+      <c r="I200" t="s">
+        <v>483</v>
+      </c>
+      <c r="J200" t="s">
+        <v>84</v>
+      </c>
+      <c r="K200" t="s">
+        <v>55</v>
+      </c>
+      <c r="L200" t="s">
+        <v>14</v>
+      </c>
+      <c r="M200" t="s">
+        <v>15</v>
+      </c>
+      <c r="N200" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="201" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A201" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="B201" t="s">
+        <v>739</v>
+      </c>
+      <c r="C201" t="s">
+        <v>745</v>
+      </c>
+      <c r="D201" t="s">
+        <v>54</v>
+      </c>
+      <c r="E201" t="s">
+        <v>33</v>
+      </c>
+      <c r="F201" t="s">
+        <v>32</v>
+      </c>
+      <c r="G201" t="s">
+        <v>741</v>
+      </c>
+      <c r="H201" t="s">
+        <v>120</v>
+      </c>
+      <c r="J201" t="s">
+        <v>446</v>
+      </c>
+      <c r="K201" t="s">
+        <v>55</v>
+      </c>
+      <c r="L201" t="s">
+        <v>14</v>
+      </c>
+      <c r="M201" t="s">
+        <v>15</v>
+      </c>
+      <c r="N201" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="202" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A202" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="B202" t="s">
+        <v>750</v>
+      </c>
+      <c r="D202" t="s">
+        <v>54</v>
+      </c>
+      <c r="E202" t="s">
+        <v>133</v>
+      </c>
+      <c r="F202" t="s">
+        <v>32</v>
+      </c>
+      <c r="G202" t="s">
+        <v>169</v>
+      </c>
+      <c r="H202" t="s">
+        <v>317</v>
+      </c>
+      <c r="J202" t="s">
+        <v>208</v>
+      </c>
+      <c r="K202" t="s">
+        <v>55</v>
+      </c>
+      <c r="L202" t="s">
+        <v>14</v>
+      </c>
+      <c r="M202" t="s">
+        <v>15</v>
+      </c>
+      <c r="N202" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="203" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A203" s="1" t="s">
+        <v>699</v>
+      </c>
+      <c r="B203" t="s">
+        <v>740</v>
+      </c>
+      <c r="C203" t="s">
+        <v>746</v>
+      </c>
+      <c r="D203" t="s">
+        <v>54</v>
+      </c>
+      <c r="E203" t="s">
+        <v>33</v>
+      </c>
+      <c r="F203" t="s">
+        <v>32</v>
+      </c>
+      <c r="G203" t="s">
+        <v>741</v>
+      </c>
+      <c r="H203" t="s">
+        <v>120</v>
+      </c>
+      <c r="J203" t="s">
+        <v>446</v>
+      </c>
+      <c r="K203" t="s">
+        <v>55</v>
+      </c>
+      <c r="L203" t="s">
+        <v>14</v>
+      </c>
+      <c r="M203" t="s">
+        <v>15</v>
+      </c>
+      <c r="N203" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Incorporar ilustraciones y enlaces  3
</commit_message>
<xml_diff>
--- a/data/PortfolioArTeV1.xlsx
+++ b/data/PortfolioArTeV1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arturompw/portfolio/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BF708F7-193E-064B-9AC7-F0A981A5ECE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94DEF1BB-7C3E-A646-835C-63D8C6A14FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4100" yWindow="600" windowWidth="22940" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolio" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2980" uniqueCount="793">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3243" uniqueCount="844">
   <si>
     <t>id</t>
   </si>
@@ -2353,9 +2353,6 @@
     <t>Te espero</t>
   </si>
   <si>
-    <t>Reinz: Marist Moustard</t>
-  </si>
-  <si>
     <t>Bienvenido a la familia</t>
   </si>
   <si>
@@ -2398,7 +2395,163 @@
     <t>Para felicitación Infantil-Primaria</t>
   </si>
   <si>
-    <t>Como grano de mostaza</t>
+    <t>DIS-0089</t>
+  </si>
+  <si>
+    <t>DIS-0090</t>
+  </si>
+  <si>
+    <t>DIS-0091</t>
+  </si>
+  <si>
+    <t>DIS-0092</t>
+  </si>
+  <si>
+    <t>Piensa y Actúa</t>
+  </si>
+  <si>
+    <t>Campamento Urbano Huelva 2016</t>
+  </si>
+  <si>
+    <t>Camiseta SED</t>
+  </si>
+  <si>
+    <t>Camiseta Nuevo Horizonte 2026 (FMCH)</t>
+  </si>
+  <si>
+    <t>Conectados por María</t>
+  </si>
+  <si>
+    <t>Reinz: Marist Mustard</t>
+  </si>
+  <si>
+    <t>Como granos de mostaza</t>
+  </si>
+  <si>
+    <t>Un gran día para Dar Vida</t>
+  </si>
+  <si>
+    <t>Para taza GVX Sevilla</t>
+  </si>
+  <si>
+    <t>ILU-0131</t>
+  </si>
+  <si>
+    <t>ILU-0132</t>
+  </si>
+  <si>
+    <t>ILU-0133</t>
+  </si>
+  <si>
+    <t>ILU-0134</t>
+  </si>
+  <si>
+    <t>ILU-0135</t>
+  </si>
+  <si>
+    <t>ILU-0136</t>
+  </si>
+  <si>
+    <t>ILU-0137</t>
+  </si>
+  <si>
+    <t>ILU-0138</t>
+  </si>
+  <si>
+    <t>ILU-0139</t>
+  </si>
+  <si>
+    <t>ILU-0140</t>
+  </si>
+  <si>
+    <t>ILU-0141</t>
+  </si>
+  <si>
+    <t>ILU-0142</t>
+  </si>
+  <si>
+    <t>ILU-0143</t>
+  </si>
+  <si>
+    <t>ILU-0144</t>
+  </si>
+  <si>
+    <t>ILU-0145</t>
+  </si>
+  <si>
+    <t>ILU-0146</t>
+  </si>
+  <si>
+    <t>Caridad</t>
+  </si>
+  <si>
+    <t>Muévete (Jaén)</t>
+  </si>
+  <si>
+    <t>La Chispa IV</t>
+  </si>
+  <si>
+    <t>María Niña</t>
+  </si>
+  <si>
+    <t>Nº Sª de Fourvière II</t>
+  </si>
+  <si>
+    <t>Con un solo corazón</t>
+  </si>
+  <si>
+    <t>Literal</t>
+  </si>
+  <si>
+    <t>Para Marcha Toledo</t>
+  </si>
+  <si>
+    <t>Consumo Justo</t>
+  </si>
+  <si>
+    <t>Conversión</t>
+  </si>
+  <si>
+    <t>Limosna</t>
+  </si>
+  <si>
+    <t>Oración</t>
+  </si>
+  <si>
+    <t>Ayuno</t>
+  </si>
+  <si>
+    <t>Fuertes de Corazón</t>
+  </si>
+  <si>
+    <t>Ceda</t>
+  </si>
+  <si>
+    <t>Hojas de Olivo</t>
+  </si>
+  <si>
+    <t>Hojas de Olivo II</t>
+  </si>
+  <si>
+    <t>Dando paso a la Navidad</t>
+  </si>
+  <si>
+    <t>Para lema Cuaresma Mediterránea</t>
+  </si>
+  <si>
+    <t>Cuaresma</t>
+  </si>
+  <si>
+    <t>Para campaña SED local</t>
+  </si>
+  <si>
+    <t>Logo Asociación</t>
+  </si>
+  <si>
+    <t>maria;champagnat</t>
+  </si>
+  <si>
+    <t>Acoger</t>
   </si>
 </sst>
 </file>
@@ -2755,17 +2908,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N219"/>
+  <dimension ref="A1:N239"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="32.33203125" customWidth="1"/>
-    <col min="3" max="3" width="38.33203125" customWidth="1"/>
+    <col min="3" max="3" width="31.1640625" customWidth="1"/>
     <col min="4" max="4" width="10.33203125" customWidth="1"/>
     <col min="5" max="5" width="7.83203125" customWidth="1"/>
     <col min="6" max="6" width="9.5" customWidth="1"/>
     <col min="7" max="7" width="26.1640625" customWidth="1"/>
     <col min="8" max="8" width="30.1640625" customWidth="1"/>
-    <col min="9" max="10" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.1640625" customWidth="1"/>
     <col min="11" max="11" width="15.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5381,7 +5535,7 @@
         <v>302</v>
       </c>
       <c r="J61" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="K61" t="s">
         <v>55</v>
@@ -11815,10 +11969,10 @@
         <v>756</v>
       </c>
       <c r="B212" t="s">
-        <v>777</v>
+        <v>800</v>
       </c>
       <c r="C212" t="s">
-        <v>792</v>
+        <v>801</v>
       </c>
       <c r="D212" t="s">
         <v>54</v>
@@ -11856,7 +12010,7 @@
         <v>757</v>
       </c>
       <c r="B213" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="D213" t="s">
         <v>54</v>
@@ -11877,7 +12031,7 @@
         <v>82</v>
       </c>
       <c r="J213" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="K213" t="s">
         <v>55</v>
@@ -11897,7 +12051,7 @@
         <v>758</v>
       </c>
       <c r="B214" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="C214" t="s">
         <v>774</v>
@@ -11941,10 +12095,10 @@
         <v>759</v>
       </c>
       <c r="B215" t="s">
+        <v>780</v>
+      </c>
+      <c r="C215" t="s">
         <v>781</v>
-      </c>
-      <c r="C215" t="s">
-        <v>782</v>
       </c>
       <c r="D215" t="s">
         <v>54</v>
@@ -11985,7 +12139,7 @@
         <v>760</v>
       </c>
       <c r="B216" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C216" t="s">
         <v>380</v>
@@ -12026,10 +12180,10 @@
         <v>761</v>
       </c>
       <c r="B217" t="s">
+        <v>783</v>
+      </c>
+      <c r="C217" t="s">
         <v>784</v>
-      </c>
-      <c r="C217" t="s">
-        <v>785</v>
       </c>
       <c r="D217" t="s">
         <v>54</v>
@@ -12067,10 +12221,10 @@
         <v>762</v>
       </c>
       <c r="B218" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="C218" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="D218" t="s">
         <v>85</v>
@@ -12085,7 +12239,7 @@
         <v>167</v>
       </c>
       <c r="H218" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="J218" t="s">
         <v>218</v>
@@ -12108,10 +12262,10 @@
         <v>763</v>
       </c>
       <c r="B219" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="C219" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="D219" t="s">
         <v>85</v>
@@ -12144,6 +12298,835 @@
         <v>15</v>
       </c>
       <c r="N219" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="220" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A220" s="1" t="s">
+        <v>791</v>
+      </c>
+      <c r="B220" t="s">
+        <v>795</v>
+      </c>
+      <c r="C220" t="s">
+        <v>797</v>
+      </c>
+      <c r="D220" t="s">
+        <v>85</v>
+      </c>
+      <c r="E220" t="s">
+        <v>33</v>
+      </c>
+      <c r="F220" t="s">
+        <v>13</v>
+      </c>
+      <c r="G220" t="s">
+        <v>167</v>
+      </c>
+      <c r="H220" t="s">
+        <v>594</v>
+      </c>
+      <c r="J220" t="s">
+        <v>389</v>
+      </c>
+      <c r="K220" t="s">
+        <v>56</v>
+      </c>
+      <c r="L220" t="s">
+        <v>14</v>
+      </c>
+      <c r="M220" t="s">
+        <v>15</v>
+      </c>
+      <c r="N220" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="221" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A221" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="B221" t="s">
+        <v>796</v>
+      </c>
+      <c r="C221" t="s">
+        <v>798</v>
+      </c>
+      <c r="D221" t="s">
+        <v>85</v>
+      </c>
+      <c r="E221" t="s">
+        <v>33</v>
+      </c>
+      <c r="F221" t="s">
+        <v>13</v>
+      </c>
+      <c r="G221" t="s">
+        <v>167</v>
+      </c>
+      <c r="H221" t="s">
+        <v>662</v>
+      </c>
+      <c r="J221" t="s">
+        <v>218</v>
+      </c>
+      <c r="K221" t="s">
+        <v>56</v>
+      </c>
+      <c r="L221" t="s">
+        <v>14</v>
+      </c>
+      <c r="M221" t="s">
+        <v>15</v>
+      </c>
+      <c r="N221" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="222" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A222" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="B222" t="s">
+        <v>799</v>
+      </c>
+      <c r="D222" t="s">
+        <v>85</v>
+      </c>
+      <c r="E222" t="s">
+        <v>58</v>
+      </c>
+      <c r="F222" t="s">
+        <v>13</v>
+      </c>
+      <c r="G222" t="s">
+        <v>119</v>
+      </c>
+      <c r="H222" t="s">
+        <v>369</v>
+      </c>
+      <c r="I222" t="s">
+        <v>82</v>
+      </c>
+      <c r="J222" t="s">
+        <v>102</v>
+      </c>
+      <c r="K222" t="s">
+        <v>55</v>
+      </c>
+      <c r="L222" t="s">
+        <v>14</v>
+      </c>
+      <c r="M222" t="s">
+        <v>15</v>
+      </c>
+      <c r="N222" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="223" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A223" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="B223" t="s">
+        <v>802</v>
+      </c>
+      <c r="C223" t="s">
+        <v>803</v>
+      </c>
+      <c r="D223" t="s">
+        <v>85</v>
+      </c>
+      <c r="E223" t="s">
+        <v>58</v>
+      </c>
+      <c r="F223" t="s">
+        <v>13</v>
+      </c>
+      <c r="G223" t="s">
+        <v>167</v>
+      </c>
+      <c r="H223" t="s">
+        <v>380</v>
+      </c>
+      <c r="I223" t="s">
+        <v>82</v>
+      </c>
+      <c r="J223" t="s">
+        <v>379</v>
+      </c>
+      <c r="K223" t="s">
+        <v>55</v>
+      </c>
+      <c r="L223" t="s">
+        <v>14</v>
+      </c>
+      <c r="M223" t="s">
+        <v>15</v>
+      </c>
+      <c r="N223" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="224" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A224" s="1" t="s">
+        <v>804</v>
+      </c>
+      <c r="B224" t="s">
+        <v>835</v>
+      </c>
+      <c r="D224" t="s">
+        <v>54</v>
+      </c>
+      <c r="E224" t="s">
+        <v>33</v>
+      </c>
+      <c r="F224" t="s">
+        <v>13</v>
+      </c>
+      <c r="G224" t="s">
+        <v>167</v>
+      </c>
+      <c r="J224" t="s">
+        <v>208</v>
+      </c>
+      <c r="K224" t="s">
+        <v>55</v>
+      </c>
+      <c r="L224" t="s">
+        <v>14</v>
+      </c>
+      <c r="M224" t="s">
+        <v>15</v>
+      </c>
+      <c r="N224" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="225" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A225" s="1" t="s">
+        <v>805</v>
+      </c>
+      <c r="B225" t="s">
+        <v>836</v>
+      </c>
+      <c r="D225" t="s">
+        <v>54</v>
+      </c>
+      <c r="E225" t="s">
+        <v>33</v>
+      </c>
+      <c r="F225" t="s">
+        <v>13</v>
+      </c>
+      <c r="G225" t="s">
+        <v>167</v>
+      </c>
+      <c r="J225" t="s">
+        <v>208</v>
+      </c>
+      <c r="K225" t="s">
+        <v>55</v>
+      </c>
+      <c r="L225" t="s">
+        <v>14</v>
+      </c>
+      <c r="M225" t="s">
+        <v>15</v>
+      </c>
+      <c r="N225" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="226" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A226" s="1" t="s">
+        <v>806</v>
+      </c>
+      <c r="B226" t="s">
+        <v>834</v>
+      </c>
+      <c r="C226" t="s">
+        <v>837</v>
+      </c>
+      <c r="D226" t="s">
+        <v>54</v>
+      </c>
+      <c r="E226" t="s">
+        <v>33</v>
+      </c>
+      <c r="F226" t="s">
+        <v>32</v>
+      </c>
+      <c r="G226" t="s">
+        <v>252</v>
+      </c>
+      <c r="J226" t="s">
+        <v>208</v>
+      </c>
+      <c r="K226" t="s">
+        <v>55</v>
+      </c>
+      <c r="L226" t="s">
+        <v>14</v>
+      </c>
+      <c r="M226" t="s">
+        <v>15</v>
+      </c>
+      <c r="N226" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="227" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A227" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B227" t="s">
+        <v>833</v>
+      </c>
+      <c r="C227" t="s">
+        <v>838</v>
+      </c>
+      <c r="D227" t="s">
+        <v>54</v>
+      </c>
+      <c r="E227" t="s">
+        <v>58</v>
+      </c>
+      <c r="F227" t="s">
+        <v>13</v>
+      </c>
+      <c r="G227" t="s">
+        <v>306</v>
+      </c>
+      <c r="H227" t="s">
+        <v>237</v>
+      </c>
+      <c r="I227" t="s">
+        <v>236</v>
+      </c>
+      <c r="J227" t="s">
+        <v>208</v>
+      </c>
+      <c r="K227" t="s">
+        <v>55</v>
+      </c>
+      <c r="L227" t="s">
+        <v>14</v>
+      </c>
+      <c r="M227" t="s">
+        <v>15</v>
+      </c>
+      <c r="N227" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="228" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A228" s="1" t="s">
+        <v>808</v>
+      </c>
+      <c r="B228" t="s">
+        <v>832</v>
+      </c>
+      <c r="C228" t="s">
+        <v>839</v>
+      </c>
+      <c r="D228" t="s">
+        <v>54</v>
+      </c>
+      <c r="E228" t="s">
+        <v>33</v>
+      </c>
+      <c r="F228" t="s">
+        <v>13</v>
+      </c>
+      <c r="G228" t="s">
+        <v>306</v>
+      </c>
+      <c r="H228" t="s">
+        <v>316</v>
+      </c>
+      <c r="I228" t="s">
+        <v>61</v>
+      </c>
+      <c r="J228" t="s">
+        <v>208</v>
+      </c>
+      <c r="K228" t="s">
+        <v>55</v>
+      </c>
+      <c r="L228" t="s">
+        <v>14</v>
+      </c>
+      <c r="M228" t="s">
+        <v>15</v>
+      </c>
+      <c r="N228" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="229" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A229" s="1" t="s">
+        <v>809</v>
+      </c>
+      <c r="B229" t="s">
+        <v>831</v>
+      </c>
+      <c r="C229" t="s">
+        <v>839</v>
+      </c>
+      <c r="D229" t="s">
+        <v>54</v>
+      </c>
+      <c r="E229" t="s">
+        <v>33</v>
+      </c>
+      <c r="F229" t="s">
+        <v>13</v>
+      </c>
+      <c r="G229" t="s">
+        <v>306</v>
+      </c>
+      <c r="H229" t="s">
+        <v>316</v>
+      </c>
+      <c r="I229" t="s">
+        <v>61</v>
+      </c>
+      <c r="J229" t="s">
+        <v>208</v>
+      </c>
+      <c r="K229" t="s">
+        <v>55</v>
+      </c>
+      <c r="L229" t="s">
+        <v>14</v>
+      </c>
+      <c r="M229" t="s">
+        <v>15</v>
+      </c>
+      <c r="N229" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="230" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A230" s="1" t="s">
+        <v>810</v>
+      </c>
+      <c r="B230" t="s">
+        <v>830</v>
+      </c>
+      <c r="C230" t="s">
+        <v>839</v>
+      </c>
+      <c r="D230" t="s">
+        <v>54</v>
+      </c>
+      <c r="E230" t="s">
+        <v>33</v>
+      </c>
+      <c r="F230" t="s">
+        <v>13</v>
+      </c>
+      <c r="G230" t="s">
+        <v>306</v>
+      </c>
+      <c r="H230" t="s">
+        <v>316</v>
+      </c>
+      <c r="I230" t="s">
+        <v>61</v>
+      </c>
+      <c r="J230" t="s">
+        <v>208</v>
+      </c>
+      <c r="K230" t="s">
+        <v>55</v>
+      </c>
+      <c r="L230" t="s">
+        <v>14</v>
+      </c>
+      <c r="M230" t="s">
+        <v>15</v>
+      </c>
+      <c r="N230" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="231" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A231" s="1" t="s">
+        <v>811</v>
+      </c>
+      <c r="B231" t="s">
+        <v>829</v>
+      </c>
+      <c r="C231" t="s">
+        <v>839</v>
+      </c>
+      <c r="D231" t="s">
+        <v>54</v>
+      </c>
+      <c r="E231" t="s">
+        <v>33</v>
+      </c>
+      <c r="F231" t="s">
+        <v>13</v>
+      </c>
+      <c r="G231" t="s">
+        <v>306</v>
+      </c>
+      <c r="H231" t="s">
+        <v>316</v>
+      </c>
+      <c r="I231" t="s">
+        <v>166</v>
+      </c>
+      <c r="J231" t="s">
+        <v>208</v>
+      </c>
+      <c r="K231" t="s">
+        <v>55</v>
+      </c>
+      <c r="L231" t="s">
+        <v>14</v>
+      </c>
+      <c r="M231" t="s">
+        <v>15</v>
+      </c>
+      <c r="N231" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="232" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A232" s="1" t="s">
+        <v>812</v>
+      </c>
+      <c r="B232" t="s">
+        <v>828</v>
+      </c>
+      <c r="C232" t="s">
+        <v>840</v>
+      </c>
+      <c r="D232" t="s">
+        <v>54</v>
+      </c>
+      <c r="E232" t="s">
+        <v>58</v>
+      </c>
+      <c r="F232" t="s">
+        <v>13</v>
+      </c>
+      <c r="G232" t="s">
+        <v>167</v>
+      </c>
+      <c r="H232" t="s">
+        <v>557</v>
+      </c>
+      <c r="I232" t="s">
+        <v>82</v>
+      </c>
+      <c r="J232" t="s">
+        <v>227</v>
+      </c>
+      <c r="K232" t="s">
+        <v>55</v>
+      </c>
+      <c r="L232" t="s">
+        <v>14</v>
+      </c>
+      <c r="M232" t="s">
+        <v>15</v>
+      </c>
+      <c r="N232" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="233" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A233" s="1" t="s">
+        <v>813</v>
+      </c>
+      <c r="B233" t="s">
+        <v>827</v>
+      </c>
+      <c r="C233" t="s">
+        <v>623</v>
+      </c>
+      <c r="D233" t="s">
+        <v>54</v>
+      </c>
+      <c r="E233" t="s">
+        <v>58</v>
+      </c>
+      <c r="F233" t="s">
+        <v>13</v>
+      </c>
+      <c r="G233" t="s">
+        <v>167</v>
+      </c>
+      <c r="J233" t="s">
+        <v>208</v>
+      </c>
+      <c r="K233" t="s">
+        <v>55</v>
+      </c>
+      <c r="L233" t="s">
+        <v>14</v>
+      </c>
+      <c r="M233" t="s">
+        <v>15</v>
+      </c>
+      <c r="N233" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="234" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A234" s="1" t="s">
+        <v>814</v>
+      </c>
+      <c r="B234" t="s">
+        <v>825</v>
+      </c>
+      <c r="C234" t="s">
+        <v>826</v>
+      </c>
+      <c r="D234" t="s">
+        <v>54</v>
+      </c>
+      <c r="E234" t="s">
+        <v>33</v>
+      </c>
+      <c r="F234" t="s">
+        <v>13</v>
+      </c>
+      <c r="G234" t="s">
+        <v>167</v>
+      </c>
+      <c r="H234" t="s">
+        <v>120</v>
+      </c>
+      <c r="J234" t="s">
+        <v>208</v>
+      </c>
+      <c r="K234" t="s">
+        <v>55</v>
+      </c>
+      <c r="L234" t="s">
+        <v>14</v>
+      </c>
+      <c r="M234" t="s">
+        <v>15</v>
+      </c>
+      <c r="N234" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="235" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A235" s="1" t="s">
+        <v>815</v>
+      </c>
+      <c r="B235" t="s">
+        <v>824</v>
+      </c>
+      <c r="D235" t="s">
+        <v>54</v>
+      </c>
+      <c r="E235" t="s">
+        <v>133</v>
+      </c>
+      <c r="F235" t="s">
+        <v>32</v>
+      </c>
+      <c r="G235" t="s">
+        <v>169</v>
+      </c>
+      <c r="H235" t="s">
+        <v>842</v>
+      </c>
+      <c r="J235" t="s">
+        <v>443</v>
+      </c>
+      <c r="K235" t="s">
+        <v>55</v>
+      </c>
+      <c r="L235" t="s">
+        <v>14</v>
+      </c>
+      <c r="M235" t="s">
+        <v>15</v>
+      </c>
+      <c r="N235" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="236" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A236" s="1" t="s">
+        <v>816</v>
+      </c>
+      <c r="B236" t="s">
+        <v>823</v>
+      </c>
+      <c r="C236" t="s">
+        <v>843</v>
+      </c>
+      <c r="D236" t="s">
+        <v>54</v>
+      </c>
+      <c r="E236" t="s">
+        <v>133</v>
+      </c>
+      <c r="F236" t="s">
+        <v>32</v>
+      </c>
+      <c r="G236" t="s">
+        <v>512</v>
+      </c>
+      <c r="H236" t="s">
+        <v>153</v>
+      </c>
+      <c r="I236" t="s">
+        <v>61</v>
+      </c>
+      <c r="J236" t="s">
+        <v>208</v>
+      </c>
+      <c r="K236" t="s">
+        <v>55</v>
+      </c>
+      <c r="L236" t="s">
+        <v>14</v>
+      </c>
+      <c r="M236" t="s">
+        <v>15</v>
+      </c>
+      <c r="N236" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="237" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A237" s="1" t="s">
+        <v>817</v>
+      </c>
+      <c r="B237" t="s">
+        <v>822</v>
+      </c>
+      <c r="D237" t="s">
+        <v>54</v>
+      </c>
+      <c r="E237" t="s">
+        <v>33</v>
+      </c>
+      <c r="F237" t="s">
+        <v>13</v>
+      </c>
+      <c r="G237" t="s">
+        <v>167</v>
+      </c>
+      <c r="H237" t="s">
+        <v>380</v>
+      </c>
+      <c r="I237" t="s">
+        <v>61</v>
+      </c>
+      <c r="J237" t="s">
+        <v>443</v>
+      </c>
+      <c r="K237" t="s">
+        <v>55</v>
+      </c>
+      <c r="L237" t="s">
+        <v>14</v>
+      </c>
+      <c r="M237" t="s">
+        <v>15</v>
+      </c>
+      <c r="N237" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="238" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A238" s="1" t="s">
+        <v>818</v>
+      </c>
+      <c r="B238" t="s">
+        <v>821</v>
+      </c>
+      <c r="C238" t="s">
+        <v>841</v>
+      </c>
+      <c r="D238" t="s">
+        <v>54</v>
+      </c>
+      <c r="E238" t="s">
+        <v>58</v>
+      </c>
+      <c r="F238" t="s">
+        <v>32</v>
+      </c>
+      <c r="G238" t="s">
+        <v>169</v>
+      </c>
+      <c r="H238" t="s">
+        <v>594</v>
+      </c>
+      <c r="I238" t="s">
+        <v>166</v>
+      </c>
+      <c r="J238" t="s">
+        <v>208</v>
+      </c>
+      <c r="K238" t="s">
+        <v>55</v>
+      </c>
+      <c r="L238" t="s">
+        <v>14</v>
+      </c>
+      <c r="M238" t="s">
+        <v>15</v>
+      </c>
+      <c r="N238" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="239" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A239" s="1" t="s">
+        <v>819</v>
+      </c>
+      <c r="B239" t="s">
+        <v>820</v>
+      </c>
+      <c r="C239" t="s">
+        <v>839</v>
+      </c>
+      <c r="D239" t="s">
+        <v>54</v>
+      </c>
+      <c r="E239" t="s">
+        <v>33</v>
+      </c>
+      <c r="F239" t="s">
+        <v>13</v>
+      </c>
+      <c r="G239" t="s">
+        <v>306</v>
+      </c>
+      <c r="H239" t="s">
+        <v>316</v>
+      </c>
+      <c r="I239" t="s">
+        <v>61</v>
+      </c>
+      <c r="J239" t="s">
+        <v>208</v>
+      </c>
+      <c r="K239" t="s">
+        <v>55</v>
+      </c>
+      <c r="L239" t="s">
+        <v>14</v>
+      </c>
+      <c r="M239" t="s">
+        <v>15</v>
+      </c>
+      <c r="N239" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Nuevas ilustraciones y cambio papeleras
</commit_message>
<xml_diff>
--- a/data/PortfolioArTeV1.xlsx
+++ b/data/PortfolioArTeV1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arturompw/portfolio/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB1F5BCC-203A-654A-82D1-127CD2D1C105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A072300-84FC-D644-9355-4EC1B6069662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4652" uniqueCount="1461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4754" uniqueCount="1484">
   <si>
     <t>id</t>
   </si>
@@ -4403,6 +4403,75 @@
   </si>
   <si>
     <t>Double G - Heart GVX</t>
+  </si>
+  <si>
+    <t>ILU-0198</t>
+  </si>
+  <si>
+    <t>ILU-0199</t>
+  </si>
+  <si>
+    <t>ILU-0200</t>
+  </si>
+  <si>
+    <t>ILU-0201</t>
+  </si>
+  <si>
+    <t>ILU-0202</t>
+  </si>
+  <si>
+    <t>Tu mano II</t>
+  </si>
+  <si>
+    <t>Tu mano III</t>
+  </si>
+  <si>
+    <t>Tu mano IV</t>
+  </si>
+  <si>
+    <t>Your hand II</t>
+  </si>
+  <si>
+    <t>Your hand III</t>
+  </si>
+  <si>
+    <t>Your hand IV</t>
+  </si>
+  <si>
+    <t>3 cruces</t>
+  </si>
+  <si>
+    <t>3 cross</t>
+  </si>
+  <si>
+    <t>Sal + luz</t>
+  </si>
+  <si>
+    <t>Salt + Light</t>
+  </si>
+  <si>
+    <t>Estrella de Belén</t>
+  </si>
+  <si>
+    <t>Bethleem Star</t>
+  </si>
+  <si>
+    <t>DIS-0106</t>
+  </si>
+  <si>
+    <t>DIS-0107</t>
+  </si>
+  <si>
+    <t>¿Estás en casa?</t>
+  </si>
+  <si>
+    <t>Are you at home?</t>
+  </si>
+  <si>
+    <t>En voz alta</t>
+  </si>
+  <si>
+    <t>Aloud</t>
   </si>
 </sst>
 </file>
@@ -4759,7 +4828,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P303"/>
+  <dimension ref="A1:P310"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="27.5" customWidth="1"/>
@@ -14697,19 +14766,19 @@
     </row>
     <row r="207" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A207" s="1" t="s">
-        <v>301</v>
+        <v>1478</v>
       </c>
       <c r="B207" t="s">
-        <v>325</v>
+        <v>1482</v>
       </c>
       <c r="C207" t="s">
-        <v>1174</v>
+        <v>1483</v>
       </c>
       <c r="D207" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="E207" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="F207" t="s">
         <v>78</v>
@@ -14797,22 +14866,22 @@
     </row>
     <row r="209" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A209" s="1" t="s">
-        <v>302</v>
+        <v>716</v>
       </c>
       <c r="B209" t="s">
-        <v>327</v>
+        <v>739</v>
       </c>
       <c r="C209" t="s">
-        <v>1176</v>
+        <v>1219</v>
       </c>
       <c r="D209" t="s">
-        <v>796</v>
+        <v>744</v>
       </c>
       <c r="E209" t="s">
-        <v>972</v>
+        <v>1018</v>
       </c>
       <c r="F209" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G209" t="s">
         <v>51</v>
@@ -14827,10 +14896,10 @@
         <v>206</v>
       </c>
       <c r="K209" t="s">
-        <v>75</v>
+        <v>205</v>
       </c>
       <c r="L209" t="s">
-        <v>97</v>
+        <v>179</v>
       </c>
       <c r="M209" t="s">
         <v>48</v>
@@ -14847,19 +14916,19 @@
     </row>
     <row r="210" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A210" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B210" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C210" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="D210" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="E210" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="F210" t="s">
         <v>78</v>
@@ -14897,22 +14966,22 @@
     </row>
     <row r="211" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A211" s="1" t="s">
-        <v>716</v>
+        <v>303</v>
       </c>
       <c r="B211" t="s">
-        <v>739</v>
+        <v>328</v>
       </c>
       <c r="C211" t="s">
-        <v>1219</v>
+        <v>1177</v>
       </c>
       <c r="D211" t="s">
-        <v>744</v>
+        <v>798</v>
       </c>
       <c r="E211" t="s">
-        <v>1018</v>
+        <v>973</v>
       </c>
       <c r="F211" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G211" t="s">
         <v>51</v>
@@ -14927,10 +14996,10 @@
         <v>206</v>
       </c>
       <c r="K211" t="s">
-        <v>205</v>
+        <v>75</v>
       </c>
       <c r="L211" t="s">
-        <v>179</v>
+        <v>97</v>
       </c>
       <c r="M211" t="s">
         <v>48</v>
@@ -15197,19 +15266,19 @@
     </row>
     <row r="217" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A217" s="1" t="s">
-        <v>1280</v>
+        <v>580</v>
       </c>
       <c r="B217" t="s">
-        <v>1304</v>
+        <v>586</v>
       </c>
       <c r="C217" t="s">
-        <v>1305</v>
+        <v>1195</v>
       </c>
       <c r="D217" t="s">
-        <v>1249</v>
+        <v>594</v>
       </c>
       <c r="E217" t="s">
-        <v>1251</v>
+        <v>990</v>
       </c>
       <c r="F217" t="s">
         <v>47</v>
@@ -15221,19 +15290,19 @@
         <v>31</v>
       </c>
       <c r="I217" t="s">
-        <v>446</v>
+        <v>587</v>
       </c>
       <c r="J217" t="s">
         <v>277</v>
       </c>
       <c r="K217" t="s">
-        <v>415</v>
+        <v>75</v>
       </c>
       <c r="L217" t="s">
         <v>179</v>
       </c>
       <c r="M217" t="s">
-        <v>833</v>
+        <v>48</v>
       </c>
       <c r="N217" t="s">
         <v>14</v>
@@ -15247,19 +15316,19 @@
     </row>
     <row r="218" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A218" s="1" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="B218" t="s">
-        <v>1306</v>
+        <v>1304</v>
       </c>
       <c r="C218" t="s">
-        <v>1307</v>
+        <v>1305</v>
       </c>
       <c r="D218" t="s">
-        <v>1308</v>
+        <v>1249</v>
       </c>
       <c r="E218" t="s">
-        <v>1308</v>
+        <v>1251</v>
       </c>
       <c r="F218" t="s">
         <v>47</v>
@@ -15268,22 +15337,22 @@
         <v>32</v>
       </c>
       <c r="H218" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I218" t="s">
-        <v>141</v>
+        <v>446</v>
       </c>
       <c r="J218" t="s">
         <v>277</v>
       </c>
       <c r="K218" t="s">
-        <v>140</v>
+        <v>415</v>
       </c>
       <c r="L218" t="s">
         <v>179</v>
       </c>
       <c r="M218" t="s">
-        <v>48</v>
+        <v>833</v>
       </c>
       <c r="N218" t="s">
         <v>14</v>
@@ -15297,35 +15366,38 @@
     </row>
     <row r="219" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A219" s="1" t="s">
-        <v>615</v>
+        <v>1281</v>
       </c>
       <c r="B219" t="s">
-        <v>658</v>
+        <v>1306</v>
       </c>
       <c r="C219" t="s">
-        <v>1207</v>
+        <v>1307</v>
       </c>
       <c r="D219" t="s">
-        <v>817</v>
+        <v>1308</v>
       </c>
       <c r="E219" t="s">
-        <v>1006</v>
+        <v>1308</v>
       </c>
       <c r="F219" t="s">
         <v>47</v>
       </c>
       <c r="G219" t="s">
-        <v>119</v>
+        <v>32</v>
       </c>
       <c r="H219" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I219" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J219" t="s">
         <v>277</v>
       </c>
+      <c r="K219" t="s">
+        <v>140</v>
+      </c>
       <c r="L219" t="s">
         <v>179</v>
       </c>
@@ -15344,37 +15416,34 @@
     </row>
     <row r="220" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A220" s="1" t="s">
-        <v>580</v>
+        <v>615</v>
       </c>
       <c r="B220" t="s">
-        <v>586</v>
+        <v>658</v>
       </c>
       <c r="C220" t="s">
-        <v>1195</v>
+        <v>1207</v>
       </c>
       <c r="D220" t="s">
-        <v>594</v>
+        <v>817</v>
       </c>
       <c r="E220" t="s">
-        <v>990</v>
+        <v>1006</v>
       </c>
       <c r="F220" t="s">
         <v>47</v>
       </c>
       <c r="G220" t="s">
-        <v>32</v>
+        <v>119</v>
       </c>
       <c r="H220" t="s">
         <v>31</v>
       </c>
       <c r="I220" t="s">
-        <v>587</v>
+        <v>143</v>
       </c>
       <c r="J220" t="s">
         <v>277</v>
-      </c>
-      <c r="K220" t="s">
-        <v>75</v>
       </c>
       <c r="L220" t="s">
         <v>179</v>
@@ -15541,22 +15610,16 @@
     </row>
     <row r="224" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A224" s="1" t="s">
-        <v>1266</v>
+        <v>1461</v>
       </c>
       <c r="B224" t="s">
-        <v>1269</v>
+        <v>1466</v>
       </c>
       <c r="C224" t="s">
-        <v>1271</v>
-      </c>
-      <c r="D224" t="s">
-        <v>683</v>
-      </c>
-      <c r="E224" t="s">
-        <v>1009</v>
+        <v>1469</v>
       </c>
       <c r="F224" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G224" t="s">
         <v>32</v>
@@ -15565,13 +15628,13 @@
         <v>31</v>
       </c>
       <c r="I224" t="s">
-        <v>1274</v>
-      </c>
-      <c r="J224" t="s">
-        <v>277</v>
+        <v>446</v>
+      </c>
+      <c r="K224" t="s">
+        <v>54</v>
       </c>
       <c r="L224" t="s">
-        <v>97</v>
+        <v>179</v>
       </c>
       <c r="M224" t="s">
         <v>48</v>
@@ -15588,34 +15651,25 @@
     </row>
     <row r="225" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A225" s="1" t="s">
-        <v>1334</v>
+        <v>1462</v>
       </c>
       <c r="B225" t="s">
-        <v>1359</v>
+        <v>1467</v>
       </c>
       <c r="C225" t="s">
-        <v>1360</v>
-      </c>
-      <c r="D225" t="s">
-        <v>1363</v>
-      </c>
-      <c r="E225" t="s">
-        <v>1364</v>
+        <v>1470</v>
       </c>
       <c r="F225" t="s">
         <v>47</v>
       </c>
       <c r="G225" t="s">
-        <v>119</v>
+        <v>32</v>
       </c>
       <c r="H225" t="s">
         <v>31</v>
       </c>
       <c r="I225" t="s">
-        <v>108</v>
-      </c>
-      <c r="J225" t="s">
-        <v>277</v>
+        <v>446</v>
       </c>
       <c r="K225" t="s">
         <v>54</v>
@@ -15624,7 +15678,7 @@
         <v>179</v>
       </c>
       <c r="M225" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N225" t="s">
         <v>14</v>
@@ -15638,19 +15692,13 @@
     </row>
     <row r="226" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A226" s="1" t="s">
-        <v>256</v>
+        <v>1463</v>
       </c>
       <c r="B226" t="s">
-        <v>281</v>
+        <v>1468</v>
       </c>
       <c r="C226" t="s">
-        <v>1094</v>
-      </c>
-      <c r="D226" t="s">
-        <v>282</v>
-      </c>
-      <c r="E226" t="s">
-        <v>899</v>
+        <v>1471</v>
       </c>
       <c r="F226" t="s">
         <v>47</v>
@@ -15659,19 +15707,19 @@
         <v>32</v>
       </c>
       <c r="H226" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I226" t="s">
-        <v>141</v>
-      </c>
-      <c r="J226" t="s">
-        <v>110</v>
+        <v>446</v>
+      </c>
+      <c r="K226" t="s">
+        <v>54</v>
       </c>
       <c r="L226" t="s">
-        <v>95</v>
+        <v>179</v>
       </c>
       <c r="M226" t="s">
-        <v>833</v>
+        <v>48</v>
       </c>
       <c r="N226" t="s">
         <v>14</v>
@@ -15685,31 +15733,37 @@
     </row>
     <row r="227" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A227" s="1" t="s">
-        <v>1286</v>
+        <v>1266</v>
       </c>
       <c r="B227" t="s">
-        <v>1318</v>
+        <v>1269</v>
       </c>
       <c r="C227" t="s">
-        <v>1319</v>
+        <v>1271</v>
+      </c>
+      <c r="D227" t="s">
+        <v>683</v>
+      </c>
+      <c r="E227" t="s">
+        <v>1009</v>
       </c>
       <c r="F227" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G227" t="s">
         <v>32</v>
       </c>
       <c r="H227" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I227" t="s">
-        <v>141</v>
+        <v>1274</v>
       </c>
       <c r="J227" t="s">
-        <v>110</v>
+        <v>277</v>
       </c>
       <c r="L227" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="M227" t="s">
         <v>48</v>
@@ -15726,43 +15780,43 @@
     </row>
     <row r="228" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A228" s="1" t="s">
-        <v>338</v>
+        <v>1334</v>
       </c>
       <c r="B228" t="s">
-        <v>801</v>
+        <v>1359</v>
       </c>
       <c r="C228" t="s">
-        <v>1180</v>
+        <v>1360</v>
       </c>
       <c r="D228" t="s">
-        <v>351</v>
+        <v>1363</v>
       </c>
       <c r="E228" t="s">
-        <v>976</v>
+        <v>1364</v>
       </c>
       <c r="F228" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G228" t="s">
-        <v>51</v>
+        <v>119</v>
       </c>
       <c r="H228" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I228" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J228" t="s">
-        <v>520</v>
+        <v>277</v>
       </c>
       <c r="K228" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="L228" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="M228" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N228" t="s">
         <v>14</v>
@@ -15776,43 +15830,40 @@
     </row>
     <row r="229" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A229" s="1" t="s">
-        <v>666</v>
+        <v>256</v>
       </c>
       <c r="B229" t="s">
-        <v>686</v>
+        <v>281</v>
       </c>
       <c r="C229" t="s">
-        <v>1211</v>
+        <v>1094</v>
       </c>
       <c r="D229" t="s">
-        <v>687</v>
+        <v>282</v>
       </c>
       <c r="E229" t="s">
-        <v>1011</v>
+        <v>899</v>
       </c>
       <c r="F229" t="s">
         <v>47</v>
       </c>
       <c r="G229" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H229" t="s">
         <v>13</v>
       </c>
       <c r="I229" t="s">
-        <v>109</v>
+        <v>141</v>
       </c>
       <c r="J229" t="s">
-        <v>277</v>
-      </c>
-      <c r="K229" t="s">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="L229" t="s">
-        <v>179</v>
+        <v>95</v>
       </c>
       <c r="M229" t="s">
-        <v>48</v>
+        <v>833</v>
       </c>
       <c r="N229" t="s">
         <v>14</v>
@@ -15826,19 +15877,13 @@
     </row>
     <row r="230" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A230" s="1" t="s">
-        <v>247</v>
+        <v>1286</v>
       </c>
       <c r="B230" t="s">
-        <v>257</v>
+        <v>1318</v>
       </c>
       <c r="C230" t="s">
-        <v>1087</v>
-      </c>
-      <c r="D230" t="s">
-        <v>258</v>
-      </c>
-      <c r="E230" t="s">
-        <v>1028</v>
+        <v>1319</v>
       </c>
       <c r="F230" t="s">
         <v>47</v>
@@ -15853,16 +15898,13 @@
         <v>141</v>
       </c>
       <c r="J230" t="s">
-        <v>206</v>
-      </c>
-      <c r="K230" t="s">
-        <v>53</v>
+        <v>110</v>
       </c>
       <c r="L230" t="s">
-        <v>265</v>
+        <v>95</v>
       </c>
       <c r="M230" t="s">
-        <v>833</v>
+        <v>48</v>
       </c>
       <c r="N230" t="s">
         <v>14</v>
@@ -15876,37 +15918,40 @@
     </row>
     <row r="231" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A231" s="1" t="s">
-        <v>462</v>
+        <v>338</v>
       </c>
       <c r="B231" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="C231" t="s">
-        <v>1185</v>
+        <v>1180</v>
       </c>
       <c r="D231" t="s">
-        <v>470</v>
+        <v>351</v>
       </c>
       <c r="E231" t="s">
-        <v>982</v>
+        <v>976</v>
       </c>
       <c r="F231" t="s">
         <v>78</v>
       </c>
       <c r="G231" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H231" t="s">
         <v>13</v>
       </c>
       <c r="I231" t="s">
-        <v>141</v>
+        <v>109</v>
       </c>
       <c r="J231" t="s">
-        <v>277</v>
+        <v>520</v>
+      </c>
+      <c r="K231" t="s">
+        <v>75</v>
       </c>
       <c r="L231" t="s">
-        <v>493</v>
+        <v>187</v>
       </c>
       <c r="M231" t="s">
         <v>48</v>
@@ -15923,40 +15968,40 @@
     </row>
     <row r="232" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A232" s="1" t="s">
-        <v>252</v>
+        <v>301</v>
       </c>
       <c r="B232" t="s">
-        <v>273</v>
+        <v>325</v>
       </c>
       <c r="C232" t="s">
-        <v>1091</v>
+        <v>1174</v>
       </c>
       <c r="D232" t="s">
-        <v>274</v>
+        <v>799</v>
       </c>
       <c r="E232" t="s">
-        <v>1029</v>
+        <v>974</v>
       </c>
       <c r="F232" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G232" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H232" t="s">
         <v>13</v>
       </c>
       <c r="I232" t="s">
-        <v>141</v>
+        <v>326</v>
       </c>
       <c r="J232" t="s">
-        <v>275</v>
+        <v>206</v>
       </c>
       <c r="K232" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="L232" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="M232" t="s">
         <v>48</v>
@@ -15973,37 +16018,40 @@
     </row>
     <row r="233" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A233" s="1" t="s">
-        <v>407</v>
+        <v>1479</v>
       </c>
       <c r="B233" t="s">
-        <v>802</v>
+        <v>1480</v>
       </c>
       <c r="C233" t="s">
-        <v>1183</v>
+        <v>1481</v>
       </c>
       <c r="D233" t="s">
-        <v>803</v>
+        <v>799</v>
       </c>
       <c r="E233" t="s">
-        <v>979</v>
+        <v>974</v>
       </c>
       <c r="F233" t="s">
         <v>78</v>
       </c>
       <c r="G233" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H233" t="s">
         <v>13</v>
       </c>
       <c r="I233" t="s">
-        <v>141</v>
+        <v>268</v>
       </c>
       <c r="J233" t="s">
-        <v>490</v>
+        <v>206</v>
+      </c>
+      <c r="K233" t="s">
+        <v>75</v>
       </c>
       <c r="L233" t="s">
-        <v>182</v>
+        <v>97</v>
       </c>
       <c r="M233" t="s">
         <v>48</v>
@@ -16020,40 +16068,40 @@
     </row>
     <row r="234" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A234" s="1" t="s">
-        <v>590</v>
+        <v>666</v>
       </c>
       <c r="B234" t="s">
-        <v>596</v>
+        <v>686</v>
       </c>
       <c r="C234" t="s">
-        <v>1197</v>
+        <v>1211</v>
       </c>
       <c r="D234" t="s">
-        <v>597</v>
+        <v>687</v>
       </c>
       <c r="E234" t="s">
-        <v>992</v>
+        <v>1011</v>
       </c>
       <c r="F234" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G234" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H234" t="s">
         <v>13</v>
       </c>
       <c r="I234" t="s">
-        <v>268</v>
+        <v>109</v>
       </c>
       <c r="J234" t="s">
-        <v>598</v>
+        <v>277</v>
       </c>
       <c r="K234" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="L234" t="s">
-        <v>493</v>
+        <v>179</v>
       </c>
       <c r="M234" t="s">
         <v>48</v>
@@ -16070,19 +16118,19 @@
     </row>
     <row r="235" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A235" s="1" t="s">
-        <v>670</v>
+        <v>247</v>
       </c>
       <c r="B235" t="s">
-        <v>690</v>
+        <v>257</v>
       </c>
       <c r="C235" t="s">
-        <v>1213</v>
+        <v>1087</v>
       </c>
       <c r="D235" t="s">
-        <v>691</v>
+        <v>258</v>
       </c>
       <c r="E235" t="s">
-        <v>1013</v>
+        <v>1028</v>
       </c>
       <c r="F235" t="s">
         <v>47</v>
@@ -16091,22 +16139,22 @@
         <v>32</v>
       </c>
       <c r="H235" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I235" t="s">
-        <v>108</v>
+        <v>141</v>
       </c>
       <c r="J235" t="s">
-        <v>277</v>
+        <v>206</v>
       </c>
       <c r="K235" t="s">
-        <v>415</v>
+        <v>53</v>
       </c>
       <c r="L235" t="s">
-        <v>179</v>
+        <v>265</v>
       </c>
       <c r="M235" t="s">
-        <v>48</v>
+        <v>833</v>
       </c>
       <c r="N235" t="s">
         <v>14</v>
@@ -16120,40 +16168,37 @@
     </row>
     <row r="236" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A236" s="1" t="s">
-        <v>498</v>
+        <v>462</v>
       </c>
       <c r="B236" t="s">
-        <v>504</v>
+        <v>804</v>
       </c>
       <c r="C236" t="s">
-        <v>1125</v>
+        <v>1185</v>
       </c>
       <c r="D236" t="s">
-        <v>505</v>
+        <v>470</v>
       </c>
       <c r="E236" t="s">
-        <v>926</v>
+        <v>982</v>
       </c>
       <c r="F236" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G236" t="s">
         <v>32</v>
       </c>
       <c r="H236" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I236" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J236" t="s">
         <v>277</v>
       </c>
-      <c r="K236" t="s">
-        <v>54</v>
-      </c>
       <c r="L236" t="s">
-        <v>179</v>
+        <v>493</v>
       </c>
       <c r="M236" t="s">
         <v>48</v>
@@ -16170,37 +16215,37 @@
     </row>
     <row r="237" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A237" s="1" t="s">
-        <v>460</v>
+        <v>252</v>
       </c>
       <c r="B237" t="s">
-        <v>467</v>
+        <v>273</v>
       </c>
       <c r="C237" t="s">
-        <v>1184</v>
+        <v>1091</v>
       </c>
       <c r="D237" t="s">
-        <v>468</v>
+        <v>274</v>
       </c>
       <c r="E237" t="s">
-        <v>981</v>
+        <v>1029</v>
       </c>
       <c r="F237" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G237" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H237" t="s">
         <v>13</v>
       </c>
       <c r="I237" t="s">
-        <v>268</v>
+        <v>141</v>
       </c>
       <c r="J237" t="s">
-        <v>306</v>
+        <v>275</v>
       </c>
       <c r="K237" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="L237" t="s">
         <v>95</v>
@@ -16220,37 +16265,37 @@
     </row>
     <row r="238" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A238" s="1" t="s">
-        <v>556</v>
+        <v>407</v>
       </c>
       <c r="B238" t="s">
-        <v>561</v>
+        <v>802</v>
       </c>
       <c r="C238" t="s">
-        <v>1189</v>
+        <v>1183</v>
       </c>
       <c r="D238" t="s">
-        <v>595</v>
+        <v>803</v>
       </c>
       <c r="E238" t="s">
-        <v>986</v>
+        <v>979</v>
       </c>
       <c r="F238" t="s">
         <v>78</v>
       </c>
       <c r="G238" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H238" t="s">
         <v>13</v>
       </c>
       <c r="I238" t="s">
-        <v>109</v>
-      </c>
-      <c r="K238" t="s">
-        <v>75</v>
+        <v>141</v>
+      </c>
+      <c r="J238" t="s">
+        <v>490</v>
       </c>
       <c r="L238" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="M238" t="s">
         <v>48</v>
@@ -16267,43 +16312,43 @@
     </row>
     <row r="239" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A239" s="1" t="s">
-        <v>435</v>
+        <v>590</v>
       </c>
       <c r="B239" t="s">
-        <v>448</v>
+        <v>596</v>
       </c>
       <c r="C239" t="s">
-        <v>1113</v>
+        <v>1197</v>
       </c>
       <c r="D239" t="s">
-        <v>449</v>
+        <v>597</v>
       </c>
       <c r="E239" t="s">
-        <v>917</v>
+        <v>992</v>
       </c>
       <c r="F239" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G239" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H239" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I239" t="s">
-        <v>108</v>
+        <v>268</v>
       </c>
       <c r="J239" t="s">
-        <v>522</v>
+        <v>598</v>
       </c>
       <c r="K239" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L239" t="s">
-        <v>179</v>
+        <v>493</v>
       </c>
       <c r="M239" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N239" t="s">
         <v>14</v>
@@ -16317,19 +16362,19 @@
     </row>
     <row r="240" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A240" s="1" t="s">
-        <v>438</v>
+        <v>670</v>
       </c>
       <c r="B240" t="s">
-        <v>455</v>
+        <v>690</v>
       </c>
       <c r="C240" t="s">
-        <v>1115</v>
+        <v>1213</v>
       </c>
       <c r="D240" t="s">
-        <v>456</v>
+        <v>691</v>
       </c>
       <c r="E240" t="s">
-        <v>919</v>
+        <v>1013</v>
       </c>
       <c r="F240" t="s">
         <v>47</v>
@@ -16341,13 +16386,13 @@
         <v>31</v>
       </c>
       <c r="I240" t="s">
-        <v>143</v>
+        <v>108</v>
       </c>
       <c r="J240" t="s">
-        <v>524</v>
+        <v>277</v>
       </c>
       <c r="K240" t="s">
-        <v>54</v>
+        <v>415</v>
       </c>
       <c r="L240" t="s">
         <v>179</v>
@@ -16367,43 +16412,43 @@
     </row>
     <row r="241" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A241" s="1" t="s">
-        <v>591</v>
+        <v>498</v>
       </c>
       <c r="B241" t="s">
-        <v>600</v>
+        <v>504</v>
       </c>
       <c r="C241" t="s">
-        <v>1198</v>
+        <v>1125</v>
       </c>
       <c r="D241" t="s">
-        <v>601</v>
+        <v>505</v>
       </c>
       <c r="E241" t="s">
-        <v>993</v>
+        <v>926</v>
       </c>
       <c r="F241" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G241" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H241" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I241" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J241" t="s">
-        <v>488</v>
+        <v>277</v>
       </c>
       <c r="K241" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="L241" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="M241" t="s">
-        <v>832</v>
+        <v>48</v>
       </c>
       <c r="N241" t="s">
         <v>14</v>
@@ -16417,19 +16462,13 @@
     </row>
     <row r="242" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A242" s="1" t="s">
-        <v>1245</v>
+        <v>1465</v>
       </c>
       <c r="B242" t="s">
-        <v>1261</v>
+        <v>1476</v>
       </c>
       <c r="C242" t="s">
-        <v>1262</v>
-      </c>
-      <c r="D242" t="s">
-        <v>456</v>
-      </c>
-      <c r="E242" t="s">
-        <v>919</v>
+        <v>1477</v>
       </c>
       <c r="F242" t="s">
         <v>47</v>
@@ -16441,13 +16480,16 @@
         <v>31</v>
       </c>
       <c r="I242" t="s">
-        <v>143</v>
+        <v>446</v>
       </c>
       <c r="J242" t="s">
-        <v>1263</v>
+        <v>277</v>
+      </c>
+      <c r="K242" t="s">
+        <v>54</v>
       </c>
       <c r="L242" t="s">
-        <v>95</v>
+        <v>179</v>
       </c>
       <c r="M242" t="s">
         <v>48</v>
@@ -16464,34 +16506,40 @@
     </row>
     <row r="243" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A243" s="1" t="s">
-        <v>1332</v>
+        <v>460</v>
       </c>
       <c r="B243" t="s">
-        <v>1355</v>
+        <v>467</v>
       </c>
       <c r="C243" t="s">
-        <v>1356</v>
+        <v>1184</v>
+      </c>
+      <c r="D243" t="s">
+        <v>468</v>
+      </c>
+      <c r="E243" t="s">
+        <v>981</v>
       </c>
       <c r="F243" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G243" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H243" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I243" t="s">
-        <v>1274</v>
+        <v>268</v>
       </c>
       <c r="J243" t="s">
-        <v>1263</v>
+        <v>306</v>
       </c>
       <c r="K243" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="L243" t="s">
-        <v>179</v>
+        <v>95</v>
       </c>
       <c r="M243" t="s">
         <v>48</v>
@@ -16508,37 +16556,40 @@
     </row>
     <row r="244" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A244" s="1" t="s">
-        <v>610</v>
+        <v>556</v>
       </c>
       <c r="B244" t="s">
-        <v>656</v>
+        <v>561</v>
       </c>
       <c r="C244" t="s">
-        <v>1206</v>
+        <v>1189</v>
+      </c>
+      <c r="D244" t="s">
+        <v>595</v>
+      </c>
+      <c r="E244" t="s">
+        <v>986</v>
       </c>
       <c r="F244" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G244" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H244" t="s">
         <v>13</v>
       </c>
       <c r="I244" t="s">
-        <v>141</v>
-      </c>
-      <c r="J244" t="s">
-        <v>201</v>
+        <v>109</v>
       </c>
       <c r="K244" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="L244" t="s">
-        <v>179</v>
+        <v>196</v>
       </c>
       <c r="M244" t="s">
-        <v>832</v>
+        <v>48</v>
       </c>
       <c r="N244" t="s">
         <v>14</v>
@@ -16552,19 +16603,19 @@
     </row>
     <row r="245" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A245" s="1" t="s">
-        <v>662</v>
+        <v>435</v>
       </c>
       <c r="B245" t="s">
-        <v>678</v>
+        <v>448</v>
       </c>
       <c r="C245" t="s">
-        <v>1208</v>
+        <v>1113</v>
       </c>
       <c r="D245" t="s">
-        <v>679</v>
+        <v>449</v>
       </c>
       <c r="E245" t="s">
-        <v>1007</v>
+        <v>917</v>
       </c>
       <c r="F245" t="s">
         <v>47</v>
@@ -16573,22 +16624,22 @@
         <v>51</v>
       </c>
       <c r="H245" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I245" t="s">
-        <v>141</v>
+        <v>108</v>
       </c>
       <c r="J245" t="s">
-        <v>202</v>
+        <v>522</v>
       </c>
       <c r="K245" t="s">
-        <v>133</v>
+        <v>54</v>
       </c>
       <c r="L245" t="s">
         <v>179</v>
       </c>
       <c r="M245" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N245" t="s">
         <v>14</v>
@@ -16602,19 +16653,19 @@
     </row>
     <row r="246" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A246" s="1" t="s">
-        <v>567</v>
+        <v>438</v>
       </c>
       <c r="B246" t="s">
-        <v>571</v>
+        <v>455</v>
       </c>
       <c r="C246" t="s">
-        <v>1191</v>
+        <v>1115</v>
       </c>
       <c r="D246" t="s">
-        <v>383</v>
+        <v>456</v>
       </c>
       <c r="E246" t="s">
-        <v>904</v>
+        <v>919</v>
       </c>
       <c r="F246" t="s">
         <v>47</v>
@@ -16623,19 +16674,22 @@
         <v>32</v>
       </c>
       <c r="H246" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I246" t="s">
-        <v>268</v>
+        <v>143</v>
       </c>
       <c r="J246" t="s">
-        <v>202</v>
+        <v>524</v>
+      </c>
+      <c r="K246" t="s">
+        <v>54</v>
       </c>
       <c r="L246" t="s">
         <v>179</v>
       </c>
       <c r="M246" t="s">
-        <v>832</v>
+        <v>48</v>
       </c>
       <c r="N246" t="s">
         <v>14</v>
@@ -16649,22 +16703,22 @@
     </row>
     <row r="247" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A247" s="1" t="s">
-        <v>362</v>
+        <v>591</v>
       </c>
       <c r="B247" t="s">
-        <v>384</v>
+        <v>600</v>
       </c>
       <c r="C247" t="s">
-        <v>1099</v>
+        <v>1198</v>
       </c>
       <c r="D247" t="s">
-        <v>385</v>
+        <v>601</v>
       </c>
       <c r="E247" t="s">
-        <v>905</v>
+        <v>993</v>
       </c>
       <c r="F247" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G247" t="s">
         <v>51</v>
@@ -16676,13 +16730,16 @@
         <v>141</v>
       </c>
       <c r="J247" t="s">
-        <v>519</v>
+        <v>488</v>
+      </c>
+      <c r="K247" t="s">
+        <v>75</v>
       </c>
       <c r="L247" t="s">
-        <v>386</v>
+        <v>187</v>
       </c>
       <c r="M247" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="N247" t="s">
         <v>14</v>
@@ -16696,40 +16753,37 @@
     </row>
     <row r="248" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A248" s="1" t="s">
-        <v>363</v>
+        <v>1245</v>
       </c>
       <c r="B248" t="s">
-        <v>387</v>
+        <v>1261</v>
       </c>
       <c r="C248" t="s">
-        <v>1100</v>
+        <v>1262</v>
       </c>
       <c r="D248" t="s">
-        <v>388</v>
+        <v>456</v>
       </c>
       <c r="E248" t="s">
-        <v>906</v>
+        <v>919</v>
       </c>
       <c r="F248" t="s">
         <v>47</v>
       </c>
       <c r="G248" t="s">
-        <v>119</v>
+        <v>32</v>
       </c>
       <c r="H248" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I248" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J248" t="s">
-        <v>201</v>
-      </c>
-      <c r="K248" t="s">
-        <v>54</v>
+        <v>1263</v>
       </c>
       <c r="L248" t="s">
-        <v>179</v>
+        <v>95</v>
       </c>
       <c r="M248" t="s">
         <v>48</v>
@@ -16746,19 +16800,13 @@
     </row>
     <row r="249" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A249" s="1" t="s">
-        <v>568</v>
+        <v>1332</v>
       </c>
       <c r="B249" t="s">
-        <v>572</v>
+        <v>1355</v>
       </c>
       <c r="C249" t="s">
-        <v>1192</v>
-      </c>
-      <c r="D249" t="s">
-        <v>383</v>
-      </c>
-      <c r="E249" t="s">
-        <v>904</v>
+        <v>1356</v>
       </c>
       <c r="F249" t="s">
         <v>47</v>
@@ -16767,16 +16815,19 @@
         <v>32</v>
       </c>
       <c r="H249" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I249" t="s">
-        <v>268</v>
+        <v>1274</v>
       </c>
       <c r="J249" t="s">
-        <v>520</v>
+        <v>1263</v>
+      </c>
+      <c r="K249" t="s">
+        <v>54</v>
       </c>
       <c r="L249" t="s">
-        <v>574</v>
+        <v>179</v>
       </c>
       <c r="M249" t="s">
         <v>48</v>
@@ -16793,19 +16844,13 @@
     </row>
     <row r="250" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A250" s="1" t="s">
-        <v>578</v>
+        <v>610</v>
       </c>
       <c r="B250" t="s">
-        <v>582</v>
+        <v>656</v>
       </c>
       <c r="C250" t="s">
-        <v>1193</v>
-      </c>
-      <c r="D250" t="s">
-        <v>583</v>
-      </c>
-      <c r="E250" t="s">
-        <v>989</v>
+        <v>1206</v>
       </c>
       <c r="F250" t="s">
         <v>47</v>
@@ -16820,16 +16865,16 @@
         <v>141</v>
       </c>
       <c r="J250" t="s">
-        <v>488</v>
+        <v>201</v>
       </c>
       <c r="K250" t="s">
-        <v>140</v>
+        <v>54</v>
       </c>
       <c r="L250" t="s">
         <v>179</v>
       </c>
       <c r="M250" t="s">
-        <v>48</v>
+        <v>832</v>
       </c>
       <c r="N250" t="s">
         <v>14</v>
@@ -16843,25 +16888,25 @@
     </row>
     <row r="251" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A251" s="1" t="s">
-        <v>621</v>
+        <v>662</v>
       </c>
       <c r="B251" t="s">
-        <v>810</v>
+        <v>678</v>
       </c>
       <c r="C251" t="s">
-        <v>1201</v>
+        <v>1208</v>
       </c>
       <c r="D251" t="s">
-        <v>638</v>
+        <v>679</v>
       </c>
       <c r="E251" t="s">
-        <v>996</v>
+        <v>1007</v>
       </c>
       <c r="F251" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G251" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H251" t="s">
         <v>13</v>
@@ -16870,13 +16915,13 @@
         <v>141</v>
       </c>
       <c r="J251" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="K251" t="s">
         <v>133</v>
       </c>
       <c r="L251" t="s">
-        <v>331</v>
+        <v>179</v>
       </c>
       <c r="M251" t="s">
         <v>48</v>
@@ -16893,19 +16938,19 @@
     </row>
     <row r="252" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A252" s="1" t="s">
-        <v>190</v>
+        <v>567</v>
       </c>
       <c r="B252" t="s">
-        <v>199</v>
+        <v>571</v>
       </c>
       <c r="C252" t="s">
-        <v>1076</v>
+        <v>1191</v>
       </c>
       <c r="D252" t="s">
-        <v>200</v>
+        <v>383</v>
       </c>
       <c r="E252" t="s">
-        <v>886</v>
+        <v>904</v>
       </c>
       <c r="F252" t="s">
         <v>47</v>
@@ -16917,19 +16962,16 @@
         <v>13</v>
       </c>
       <c r="I252" t="s">
-        <v>141</v>
+        <v>268</v>
       </c>
       <c r="J252" t="s">
-        <v>201</v>
-      </c>
-      <c r="K252" t="s">
-        <v>53</v>
+        <v>202</v>
       </c>
       <c r="L252" t="s">
         <v>179</v>
       </c>
       <c r="M252" t="s">
-        <v>48</v>
+        <v>832</v>
       </c>
       <c r="N252" t="s">
         <v>14</v>
@@ -16943,43 +16985,40 @@
     </row>
     <row r="253" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A253" s="1" t="s">
-        <v>191</v>
+        <v>362</v>
       </c>
       <c r="B253" t="s">
-        <v>203</v>
+        <v>384</v>
       </c>
       <c r="C253" t="s">
-        <v>1077</v>
+        <v>1099</v>
       </c>
       <c r="D253" t="s">
-        <v>204</v>
+        <v>385</v>
       </c>
       <c r="E253" t="s">
-        <v>887</v>
+        <v>905</v>
       </c>
       <c r="F253" t="s">
         <v>47</v>
       </c>
       <c r="G253" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H253" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I253" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J253" t="s">
-        <v>206</v>
-      </c>
-      <c r="K253" t="s">
-        <v>54</v>
+        <v>519</v>
       </c>
       <c r="L253" t="s">
-        <v>179</v>
+        <v>386</v>
       </c>
       <c r="M253" t="s">
-        <v>48</v>
+        <v>833</v>
       </c>
       <c r="N253" t="s">
         <v>14</v>
@@ -16993,25 +17032,25 @@
     </row>
     <row r="254" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A254" s="1" t="s">
-        <v>192</v>
+        <v>363</v>
       </c>
       <c r="B254" t="s">
-        <v>207</v>
+        <v>387</v>
       </c>
       <c r="C254" t="s">
-        <v>1078</v>
+        <v>1100</v>
       </c>
       <c r="D254" t="s">
-        <v>208</v>
+        <v>388</v>
       </c>
       <c r="E254" t="s">
-        <v>888</v>
+        <v>906</v>
       </c>
       <c r="F254" t="s">
         <v>47</v>
       </c>
       <c r="G254" t="s">
-        <v>32</v>
+        <v>119</v>
       </c>
       <c r="H254" t="s">
         <v>13</v>
@@ -17023,10 +17062,10 @@
         <v>201</v>
       </c>
       <c r="K254" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L254" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="M254" t="s">
         <v>48</v>
@@ -17043,19 +17082,19 @@
     </row>
     <row r="255" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A255" s="1" t="s">
-        <v>189</v>
+        <v>568</v>
       </c>
       <c r="B255" t="s">
-        <v>197</v>
+        <v>572</v>
       </c>
       <c r="C255" t="s">
-        <v>1075</v>
+        <v>1192</v>
       </c>
       <c r="D255" t="s">
-        <v>198</v>
+        <v>383</v>
       </c>
       <c r="E255" t="s">
-        <v>885</v>
+        <v>904</v>
       </c>
       <c r="F255" t="s">
         <v>47</v>
@@ -17064,19 +17103,16 @@
         <v>32</v>
       </c>
       <c r="H255" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I255" t="s">
-        <v>108</v>
+        <v>268</v>
       </c>
       <c r="J255" t="s">
-        <v>202</v>
-      </c>
-      <c r="K255" t="s">
-        <v>53</v>
+        <v>520</v>
       </c>
       <c r="L255" t="s">
-        <v>386</v>
+        <v>574</v>
       </c>
       <c r="M255" t="s">
         <v>48</v>
@@ -17093,37 +17129,40 @@
     </row>
     <row r="256" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A256" s="1" t="s">
-        <v>622</v>
+        <v>578</v>
       </c>
       <c r="B256" t="s">
-        <v>639</v>
+        <v>582</v>
       </c>
       <c r="C256" t="s">
-        <v>1202</v>
+        <v>1193</v>
       </c>
       <c r="D256" t="s">
-        <v>640</v>
+        <v>583</v>
       </c>
       <c r="E256" t="s">
-        <v>997</v>
+        <v>989</v>
       </c>
       <c r="F256" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G256" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H256" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I256" t="s">
-        <v>218</v>
+        <v>141</v>
       </c>
       <c r="J256" t="s">
-        <v>202</v>
+        <v>488</v>
+      </c>
+      <c r="K256" t="s">
+        <v>140</v>
       </c>
       <c r="L256" t="s">
-        <v>95</v>
+        <v>179</v>
       </c>
       <c r="M256" t="s">
         <v>48</v>
@@ -17140,37 +17179,40 @@
     </row>
     <row r="257" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A257" s="1" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="B257" t="s">
-        <v>641</v>
+        <v>810</v>
       </c>
       <c r="C257" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="D257" t="s">
-        <v>642</v>
+        <v>638</v>
       </c>
       <c r="E257" t="s">
-        <v>1042</v>
+        <v>996</v>
       </c>
       <c r="F257" t="s">
         <v>78</v>
       </c>
       <c r="G257" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H257" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I257" t="s">
-        <v>446</v>
+        <v>141</v>
       </c>
       <c r="J257" t="s">
-        <v>202</v>
+        <v>201</v>
+      </c>
+      <c r="K257" t="s">
+        <v>133</v>
       </c>
       <c r="L257" t="s">
-        <v>95</v>
+        <v>331</v>
       </c>
       <c r="M257" t="s">
         <v>48</v>
@@ -17187,40 +17229,40 @@
     </row>
     <row r="258" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A258" s="1" t="s">
-        <v>674</v>
+        <v>190</v>
       </c>
       <c r="B258" t="s">
-        <v>696</v>
+        <v>199</v>
       </c>
       <c r="C258" t="s">
-        <v>1215</v>
+        <v>1076</v>
       </c>
       <c r="D258" t="s">
-        <v>699</v>
+        <v>200</v>
       </c>
       <c r="E258" t="s">
-        <v>1015</v>
+        <v>886</v>
       </c>
       <c r="F258" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G258" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H258" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I258" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J258" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K258" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="L258" t="s">
-        <v>95</v>
+        <v>179</v>
       </c>
       <c r="M258" t="s">
         <v>48</v>
@@ -17237,19 +17279,19 @@
     </row>
     <row r="259" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A259" s="1" t="s">
-        <v>1284</v>
+        <v>191</v>
       </c>
       <c r="B259" t="s">
-        <v>1312</v>
+        <v>203</v>
       </c>
       <c r="C259" t="s">
-        <v>1313</v>
+        <v>1077</v>
       </c>
       <c r="D259" t="s">
-        <v>1314</v>
+        <v>204</v>
       </c>
       <c r="E259" t="s">
-        <v>1308</v>
+        <v>887</v>
       </c>
       <c r="F259" t="s">
         <v>47</v>
@@ -17261,19 +17303,19 @@
         <v>31</v>
       </c>
       <c r="I259" t="s">
-        <v>1315</v>
+        <v>143</v>
       </c>
       <c r="J259" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="K259" t="s">
-        <v>140</v>
+        <v>54</v>
       </c>
       <c r="L259" t="s">
         <v>179</v>
       </c>
       <c r="M259" t="s">
-        <v>832</v>
+        <v>48</v>
       </c>
       <c r="N259" t="s">
         <v>14</v>
@@ -17287,25 +17329,25 @@
     </row>
     <row r="260" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A260" s="1" t="s">
-        <v>1289</v>
+        <v>192</v>
       </c>
       <c r="B260" t="s">
-        <v>1293</v>
+        <v>207</v>
       </c>
       <c r="C260" t="s">
-        <v>1294</v>
+        <v>1078</v>
       </c>
       <c r="D260" t="s">
-        <v>1295</v>
+        <v>208</v>
       </c>
       <c r="E260" t="s">
-        <v>1296</v>
+        <v>888</v>
       </c>
       <c r="F260" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G260" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H260" t="s">
         <v>13</v>
@@ -17314,16 +17356,16 @@
         <v>141</v>
       </c>
       <c r="J260" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K260" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="L260" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="M260" t="s">
-        <v>832</v>
+        <v>48</v>
       </c>
       <c r="N260" t="s">
         <v>14</v>
@@ -17337,13 +17379,19 @@
     </row>
     <row r="261" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A261" s="1" t="s">
-        <v>1335</v>
+        <v>189</v>
       </c>
       <c r="B261" t="s">
-        <v>1361</v>
+        <v>197</v>
       </c>
       <c r="C261" t="s">
-        <v>1362</v>
+        <v>1075</v>
+      </c>
+      <c r="D261" t="s">
+        <v>198</v>
+      </c>
+      <c r="E261" t="s">
+        <v>885</v>
       </c>
       <c r="F261" t="s">
         <v>47</v>
@@ -17352,16 +17400,19 @@
         <v>32</v>
       </c>
       <c r="H261" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I261" t="s">
-        <v>141</v>
+        <v>108</v>
       </c>
       <c r="J261" t="s">
-        <v>520</v>
+        <v>202</v>
+      </c>
+      <c r="K261" t="s">
+        <v>53</v>
       </c>
       <c r="L261" t="s">
-        <v>95</v>
+        <v>386</v>
       </c>
       <c r="M261" t="s">
         <v>48</v>
@@ -17378,37 +17429,37 @@
     </row>
     <row r="262" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A262" s="1" t="s">
-        <v>608</v>
+        <v>622</v>
       </c>
       <c r="B262" t="s">
-        <v>649</v>
+        <v>639</v>
       </c>
       <c r="C262" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="D262" t="s">
-        <v>443</v>
+        <v>640</v>
       </c>
       <c r="E262" t="s">
-        <v>915</v>
+        <v>997</v>
       </c>
       <c r="F262" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G262" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H262" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I262" t="s">
-        <v>109</v>
-      </c>
-      <c r="K262" t="s">
-        <v>54</v>
+        <v>218</v>
+      </c>
+      <c r="J262" t="s">
+        <v>202</v>
       </c>
       <c r="L262" t="s">
-        <v>180</v>
+        <v>95</v>
       </c>
       <c r="M262" t="s">
         <v>48</v>
@@ -17425,31 +17476,37 @@
     </row>
     <row r="263" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A263" s="1" t="s">
-        <v>1381</v>
+        <v>623</v>
       </c>
       <c r="B263" t="s">
-        <v>1390</v>
+        <v>641</v>
       </c>
       <c r="C263" t="s">
-        <v>1391</v>
+        <v>1203</v>
+      </c>
+      <c r="D263" t="s">
+        <v>642</v>
+      </c>
+      <c r="E263" t="s">
+        <v>1042</v>
       </c>
       <c r="F263" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G263" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H263" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I263" t="s">
-        <v>141</v>
-      </c>
-      <c r="K263" t="s">
-        <v>54</v>
+        <v>446</v>
+      </c>
+      <c r="J263" t="s">
+        <v>202</v>
       </c>
       <c r="L263" t="s">
-        <v>179</v>
+        <v>95</v>
       </c>
       <c r="M263" t="s">
         <v>48</v>
@@ -17466,40 +17523,40 @@
     </row>
     <row r="264" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A264" s="1" t="s">
-        <v>431</v>
+        <v>674</v>
       </c>
       <c r="B264" t="s">
-        <v>440</v>
+        <v>696</v>
       </c>
       <c r="C264" t="s">
-        <v>1109</v>
+        <v>1215</v>
       </c>
       <c r="D264" t="s">
-        <v>443</v>
+        <v>699</v>
       </c>
       <c r="E264" t="s">
-        <v>915</v>
+        <v>1015</v>
       </c>
       <c r="F264" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G264" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H264" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I264" t="s">
-        <v>109</v>
+        <v>143</v>
       </c>
       <c r="J264" t="s">
-        <v>441</v>
+        <v>202</v>
       </c>
       <c r="K264" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="L264" t="s">
-        <v>179</v>
+        <v>95</v>
       </c>
       <c r="M264" t="s">
         <v>48</v>
@@ -17516,19 +17573,19 @@
     </row>
     <row r="265" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A265" s="1" t="s">
-        <v>432</v>
+        <v>1284</v>
       </c>
       <c r="B265" t="s">
-        <v>442</v>
+        <v>1312</v>
       </c>
       <c r="C265" t="s">
-        <v>1110</v>
+        <v>1313</v>
       </c>
       <c r="D265" t="s">
-        <v>443</v>
+        <v>1314</v>
       </c>
       <c r="E265" t="s">
-        <v>915</v>
+        <v>1308</v>
       </c>
       <c r="F265" t="s">
         <v>47</v>
@@ -17537,22 +17594,22 @@
         <v>32</v>
       </c>
       <c r="H265" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I265" t="s">
-        <v>109</v>
+        <v>1315</v>
       </c>
       <c r="J265" t="s">
         <v>202</v>
       </c>
       <c r="K265" t="s">
-        <v>54</v>
+        <v>140</v>
       </c>
       <c r="L265" t="s">
         <v>179</v>
       </c>
       <c r="M265" t="s">
-        <v>48</v>
+        <v>832</v>
       </c>
       <c r="N265" t="s">
         <v>14</v>
@@ -17566,43 +17623,43 @@
     </row>
     <row r="266" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A266" s="1" t="s">
-        <v>439</v>
+        <v>1289</v>
       </c>
       <c r="B266" t="s">
-        <v>457</v>
+        <v>1293</v>
       </c>
       <c r="C266" t="s">
-        <v>1116</v>
+        <v>1294</v>
       </c>
       <c r="D266" t="s">
-        <v>443</v>
+        <v>1295</v>
       </c>
       <c r="E266" t="s">
-        <v>915</v>
+        <v>1296</v>
       </c>
       <c r="F266" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G266" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H266" t="s">
         <v>13</v>
       </c>
       <c r="I266" t="s">
-        <v>109</v>
+        <v>141</v>
       </c>
       <c r="J266" t="s">
         <v>202</v>
       </c>
       <c r="K266" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="L266" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="M266" t="s">
-        <v>50</v>
+        <v>832</v>
       </c>
       <c r="N266" t="s">
         <v>14</v>
@@ -17616,19 +17673,13 @@
     </row>
     <row r="267" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A267" s="1" t="s">
-        <v>665</v>
+        <v>1335</v>
       </c>
       <c r="B267" t="s">
-        <v>684</v>
+        <v>1361</v>
       </c>
       <c r="C267" t="s">
-        <v>684</v>
-      </c>
-      <c r="D267" t="s">
-        <v>685</v>
-      </c>
-      <c r="E267" t="s">
-        <v>1010</v>
+        <v>1362</v>
       </c>
       <c r="F267" t="s">
         <v>47</v>
@@ -17640,16 +17691,13 @@
         <v>13</v>
       </c>
       <c r="I267" t="s">
-        <v>446</v>
+        <v>141</v>
       </c>
       <c r="J267" t="s">
-        <v>202</v>
-      </c>
-      <c r="K267" t="s">
-        <v>133</v>
+        <v>520</v>
       </c>
       <c r="L267" t="s">
-        <v>386</v>
+        <v>95</v>
       </c>
       <c r="M267" t="s">
         <v>48</v>
@@ -17666,19 +17714,19 @@
     </row>
     <row r="268" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A268" s="1" t="s">
-        <v>669</v>
+        <v>608</v>
       </c>
       <c r="B268" t="s">
-        <v>820</v>
+        <v>649</v>
       </c>
       <c r="C268" t="s">
-        <v>1212</v>
+        <v>1205</v>
       </c>
       <c r="D268" t="s">
-        <v>685</v>
+        <v>443</v>
       </c>
       <c r="E268" t="s">
-        <v>1010</v>
+        <v>915</v>
       </c>
       <c r="F268" t="s">
         <v>47</v>
@@ -17690,13 +17738,10 @@
         <v>13</v>
       </c>
       <c r="I268" t="s">
-        <v>446</v>
-      </c>
-      <c r="J268" t="s">
-        <v>202</v>
+        <v>109</v>
       </c>
       <c r="K268" t="s">
-        <v>205</v>
+        <v>54</v>
       </c>
       <c r="L268" t="s">
         <v>180</v>
@@ -17716,34 +17761,25 @@
     </row>
     <row r="269" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A269" s="1" t="s">
-        <v>437</v>
+        <v>1381</v>
       </c>
       <c r="B269" t="s">
-        <v>453</v>
+        <v>1390</v>
       </c>
       <c r="C269" t="s">
-        <v>1114</v>
-      </c>
-      <c r="D269" t="s">
-        <v>454</v>
-      </c>
-      <c r="E269" t="s">
-        <v>918</v>
+        <v>1391</v>
       </c>
       <c r="F269" t="s">
         <v>47</v>
       </c>
       <c r="G269" t="s">
-        <v>119</v>
+        <v>32</v>
       </c>
       <c r="H269" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I269" t="s">
-        <v>143</v>
-      </c>
-      <c r="J269" t="s">
-        <v>202</v>
+        <v>141</v>
       </c>
       <c r="K269" t="s">
         <v>54</v>
@@ -17766,13 +17802,19 @@
     </row>
     <row r="270" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A270" s="1" t="s">
-        <v>1239</v>
+        <v>431</v>
       </c>
       <c r="B270" t="s">
-        <v>1247</v>
+        <v>440</v>
       </c>
       <c r="C270" t="s">
-        <v>1247</v>
+        <v>1109</v>
+      </c>
+      <c r="D270" t="s">
+        <v>443</v>
+      </c>
+      <c r="E270" t="s">
+        <v>915</v>
       </c>
       <c r="F270" t="s">
         <v>47</v>
@@ -17781,13 +17823,13 @@
         <v>32</v>
       </c>
       <c r="H270" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I270" t="s">
-        <v>446</v>
+        <v>109</v>
       </c>
       <c r="J270" t="s">
-        <v>202</v>
+        <v>441</v>
       </c>
       <c r="K270" t="s">
         <v>54</v>
@@ -17810,19 +17852,19 @@
     </row>
     <row r="271" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A271" s="1" t="s">
-        <v>607</v>
+        <v>432</v>
       </c>
       <c r="B271" t="s">
-        <v>648</v>
+        <v>442</v>
       </c>
       <c r="C271" t="s">
-        <v>648</v>
+        <v>1110</v>
       </c>
       <c r="D271" t="s">
-        <v>812</v>
+        <v>443</v>
       </c>
       <c r="E271" t="s">
-        <v>1000</v>
+        <v>915</v>
       </c>
       <c r="F271" t="s">
         <v>47</v>
@@ -17834,7 +17876,10 @@
         <v>13</v>
       </c>
       <c r="I271" t="s">
-        <v>141</v>
+        <v>109</v>
+      </c>
+      <c r="J271" t="s">
+        <v>202</v>
       </c>
       <c r="K271" t="s">
         <v>54</v>
@@ -17843,7 +17888,7 @@
         <v>179</v>
       </c>
       <c r="M271" t="s">
-        <v>833</v>
+        <v>48</v>
       </c>
       <c r="N271" t="s">
         <v>14</v>
@@ -17857,40 +17902,43 @@
     </row>
     <row r="272" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A272" s="1" t="s">
-        <v>361</v>
+        <v>439</v>
       </c>
       <c r="B272" t="s">
-        <v>382</v>
+        <v>457</v>
       </c>
       <c r="C272" t="s">
-        <v>1098</v>
+        <v>1116</v>
       </c>
       <c r="D272" t="s">
-        <v>383</v>
+        <v>443</v>
       </c>
       <c r="E272" t="s">
-        <v>904</v>
+        <v>915</v>
       </c>
       <c r="F272" t="s">
         <v>47</v>
       </c>
       <c r="G272" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H272" t="s">
         <v>13</v>
       </c>
       <c r="I272" t="s">
-        <v>268</v>
+        <v>109</v>
       </c>
       <c r="J272" t="s">
-        <v>488</v>
+        <v>202</v>
+      </c>
+      <c r="K272" t="s">
+        <v>54</v>
       </c>
       <c r="L272" t="s">
-        <v>386</v>
+        <v>179</v>
       </c>
       <c r="M272" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="N272" t="s">
         <v>14</v>
@@ -17904,40 +17952,43 @@
     </row>
     <row r="273" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A273" s="1" t="s">
-        <v>673</v>
+        <v>665</v>
       </c>
       <c r="B273" t="s">
-        <v>694</v>
+        <v>684</v>
       </c>
       <c r="C273" t="s">
-        <v>1214</v>
+        <v>684</v>
       </c>
       <c r="D273" t="s">
-        <v>698</v>
+        <v>685</v>
       </c>
       <c r="E273" t="s">
-        <v>1014</v>
+        <v>1010</v>
       </c>
       <c r="F273" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G273" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H273" t="s">
         <v>13</v>
       </c>
       <c r="I273" t="s">
-        <v>141</v>
+        <v>446</v>
       </c>
       <c r="J273" t="s">
-        <v>695</v>
+        <v>202</v>
+      </c>
+      <c r="K273" t="s">
+        <v>133</v>
       </c>
       <c r="L273" t="s">
-        <v>187</v>
+        <v>386</v>
       </c>
       <c r="M273" t="s">
-        <v>833</v>
+        <v>48</v>
       </c>
       <c r="N273" t="s">
         <v>14</v>
@@ -17951,22 +18002,22 @@
     </row>
     <row r="274" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A274" s="1" t="s">
-        <v>700</v>
+        <v>669</v>
       </c>
       <c r="B274" t="s">
-        <v>704</v>
+        <v>820</v>
       </c>
       <c r="C274" t="s">
-        <v>1216</v>
+        <v>1212</v>
       </c>
       <c r="D274" t="s">
-        <v>706</v>
+        <v>685</v>
       </c>
       <c r="E274" t="s">
-        <v>1016</v>
+        <v>1010</v>
       </c>
       <c r="F274" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G274" t="s">
         <v>32</v>
@@ -17975,16 +18026,19 @@
         <v>13</v>
       </c>
       <c r="I274" t="s">
-        <v>141</v>
+        <v>446</v>
       </c>
       <c r="J274" t="s">
-        <v>520</v>
+        <v>202</v>
+      </c>
+      <c r="K274" t="s">
+        <v>205</v>
       </c>
       <c r="L274" t="s">
-        <v>341</v>
+        <v>180</v>
       </c>
       <c r="M274" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N274" t="s">
         <v>14</v>
@@ -17998,40 +18052,43 @@
     </row>
     <row r="275" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A275" s="1" t="s">
-        <v>618</v>
+        <v>437</v>
       </c>
       <c r="B275" t="s">
-        <v>627</v>
+        <v>453</v>
       </c>
       <c r="C275" t="s">
-        <v>1200</v>
+        <v>1114</v>
       </c>
       <c r="D275" t="s">
-        <v>628</v>
+        <v>454</v>
       </c>
       <c r="E275" t="s">
-        <v>995</v>
+        <v>918</v>
       </c>
       <c r="F275" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G275" t="s">
-        <v>51</v>
+        <v>119</v>
       </c>
       <c r="H275" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I275" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J275" t="s">
-        <v>520</v>
+        <v>202</v>
+      </c>
+      <c r="K275" t="s">
+        <v>54</v>
       </c>
       <c r="L275" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="M275" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N275" t="s">
         <v>14</v>
@@ -18045,37 +18102,31 @@
     </row>
     <row r="276" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A276" s="1" t="s">
-        <v>579</v>
+        <v>1239</v>
       </c>
       <c r="B276" t="s">
-        <v>584</v>
+        <v>1247</v>
       </c>
       <c r="C276" t="s">
-        <v>1194</v>
-      </c>
-      <c r="D276" t="s">
-        <v>547</v>
-      </c>
-      <c r="E276" t="s">
-        <v>980</v>
+        <v>1247</v>
       </c>
       <c r="F276" t="s">
         <v>47</v>
       </c>
       <c r="G276" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H276" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I276" t="s">
-        <v>141</v>
+        <v>446</v>
       </c>
       <c r="J276" t="s">
-        <v>585</v>
+        <v>202</v>
       </c>
       <c r="K276" t="s">
-        <v>133</v>
+        <v>54</v>
       </c>
       <c r="L276" t="s">
         <v>179</v>
@@ -18095,25 +18146,25 @@
     </row>
     <row r="277" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A277" s="1" t="s">
-        <v>558</v>
+        <v>607</v>
       </c>
       <c r="B277" t="s">
-        <v>807</v>
+        <v>648</v>
       </c>
       <c r="C277" t="s">
-        <v>1234</v>
+        <v>648</v>
       </c>
       <c r="D277" t="s">
-        <v>563</v>
+        <v>812</v>
       </c>
       <c r="E277" t="s">
-        <v>988</v>
+        <v>1000</v>
       </c>
       <c r="F277" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G277" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H277" t="s">
         <v>13</v>
@@ -18121,17 +18172,14 @@
       <c r="I277" t="s">
         <v>141</v>
       </c>
-      <c r="J277" t="s">
-        <v>488</v>
-      </c>
       <c r="K277" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="L277" t="s">
-        <v>564</v>
+        <v>179</v>
       </c>
       <c r="M277" t="s">
-        <v>48</v>
+        <v>833</v>
       </c>
       <c r="N277" t="s">
         <v>14</v>
@@ -18145,40 +18193,40 @@
     </row>
     <row r="278" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A278" s="1" t="s">
-        <v>701</v>
+        <v>361</v>
       </c>
       <c r="B278" t="s">
-        <v>705</v>
+        <v>382</v>
       </c>
       <c r="C278" t="s">
-        <v>1217</v>
+        <v>1098</v>
       </c>
       <c r="D278" t="s">
-        <v>707</v>
+        <v>383</v>
       </c>
       <c r="E278" t="s">
-        <v>1043</v>
+        <v>904</v>
       </c>
       <c r="F278" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G278" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H278" t="s">
         <v>13</v>
       </c>
       <c r="I278" t="s">
-        <v>141</v>
+        <v>268</v>
       </c>
       <c r="J278" t="s">
         <v>488</v>
       </c>
       <c r="L278" t="s">
-        <v>187</v>
+        <v>386</v>
       </c>
       <c r="M278" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N278" t="s">
         <v>14</v>
@@ -18192,19 +18240,19 @@
     </row>
     <row r="279" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A279" s="1" t="s">
-        <v>1291</v>
+        <v>673</v>
       </c>
       <c r="B279" t="s">
-        <v>1299</v>
+        <v>694</v>
       </c>
       <c r="C279" t="s">
-        <v>1300</v>
+        <v>1214</v>
       </c>
       <c r="D279" t="s">
-        <v>1301</v>
+        <v>698</v>
       </c>
       <c r="E279" t="s">
-        <v>1302</v>
+        <v>1014</v>
       </c>
       <c r="F279" t="s">
         <v>78</v>
@@ -18219,16 +18267,13 @@
         <v>141</v>
       </c>
       <c r="J279" t="s">
-        <v>488</v>
-      </c>
-      <c r="K279" t="s">
-        <v>75</v>
+        <v>695</v>
       </c>
       <c r="L279" t="s">
         <v>187</v>
       </c>
       <c r="M279" t="s">
-        <v>48</v>
+        <v>833</v>
       </c>
       <c r="N279" t="s">
         <v>14</v>
@@ -18242,37 +18287,40 @@
     </row>
     <row r="280" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A280" s="1" t="s">
-        <v>715</v>
+        <v>700</v>
       </c>
       <c r="B280" t="s">
-        <v>740</v>
+        <v>704</v>
       </c>
       <c r="C280" t="s">
-        <v>1218</v>
+        <v>1216</v>
       </c>
       <c r="D280" t="s">
-        <v>743</v>
+        <v>706</v>
       </c>
       <c r="E280" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="F280" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G280" t="s">
         <v>32</v>
       </c>
       <c r="H280" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I280" t="s">
-        <v>217</v>
+        <v>141</v>
+      </c>
+      <c r="J280" t="s">
+        <v>520</v>
       </c>
       <c r="L280" t="s">
-        <v>179</v>
+        <v>341</v>
       </c>
       <c r="M280" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N280" t="s">
         <v>14</v>
@@ -18286,22 +18334,22 @@
     </row>
     <row r="281" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A281" s="1" t="s">
-        <v>721</v>
+        <v>618</v>
       </c>
       <c r="B281" t="s">
-        <v>734</v>
+        <v>627</v>
       </c>
       <c r="C281" t="s">
-        <v>1225</v>
+        <v>1200</v>
       </c>
       <c r="D281" t="s">
-        <v>746</v>
+        <v>628</v>
       </c>
       <c r="E281" t="s">
-        <v>1020</v>
+        <v>995</v>
       </c>
       <c r="F281" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G281" t="s">
         <v>51</v>
@@ -18313,16 +18361,13 @@
         <v>141</v>
       </c>
       <c r="J281" t="s">
-        <v>488</v>
-      </c>
-      <c r="K281" t="s">
-        <v>75</v>
+        <v>520</v>
       </c>
       <c r="L281" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="M281" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N281" t="s">
         <v>14</v>
@@ -18336,19 +18381,19 @@
     </row>
     <row r="282" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A282" s="1" t="s">
-        <v>727</v>
+        <v>579</v>
       </c>
       <c r="B282" t="s">
-        <v>730</v>
+        <v>584</v>
       </c>
       <c r="C282" t="s">
-        <v>1227</v>
+        <v>1194</v>
       </c>
       <c r="D282" t="s">
-        <v>747</v>
+        <v>547</v>
       </c>
       <c r="E282" t="s">
-        <v>1021</v>
+        <v>980</v>
       </c>
       <c r="F282" t="s">
         <v>47</v>
@@ -18363,10 +18408,10 @@
         <v>141</v>
       </c>
       <c r="J282" t="s">
-        <v>520</v>
+        <v>585</v>
       </c>
       <c r="K282" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="L282" t="s">
         <v>179</v>
@@ -18386,37 +18431,40 @@
     </row>
     <row r="283" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A283" s="1" t="s">
-        <v>1268</v>
+        <v>558</v>
       </c>
       <c r="B283" t="s">
-        <v>1275</v>
+        <v>807</v>
       </c>
       <c r="C283" t="s">
-        <v>1273</v>
+        <v>1234</v>
       </c>
       <c r="D283" t="s">
-        <v>1276</v>
+        <v>563</v>
       </c>
       <c r="E283" t="s">
-        <v>1276</v>
+        <v>988</v>
       </c>
       <c r="F283" t="s">
         <v>78</v>
       </c>
       <c r="G283" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H283" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I283" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J283" t="s">
-        <v>277</v>
+        <v>488</v>
+      </c>
+      <c r="K283" t="s">
+        <v>75</v>
       </c>
       <c r="L283" t="s">
-        <v>95</v>
+        <v>564</v>
       </c>
       <c r="M283" t="s">
         <v>48</v>
@@ -18433,37 +18481,40 @@
     </row>
     <row r="284" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A284" s="1" t="s">
-        <v>1288</v>
+        <v>701</v>
       </c>
       <c r="B284" t="s">
-        <v>1292</v>
+        <v>705</v>
       </c>
       <c r="C284" t="s">
-        <v>1303</v>
+        <v>1217</v>
+      </c>
+      <c r="D284" t="s">
+        <v>707</v>
+      </c>
+      <c r="E284" t="s">
+        <v>1043</v>
       </c>
       <c r="F284" t="s">
         <v>78</v>
       </c>
       <c r="G284" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H284" t="s">
         <v>13</v>
       </c>
       <c r="I284" t="s">
-        <v>109</v>
+        <v>141</v>
       </c>
       <c r="J284" t="s">
-        <v>110</v>
-      </c>
-      <c r="K284" t="s">
-        <v>75</v>
+        <v>488</v>
       </c>
       <c r="L284" t="s">
-        <v>95</v>
+        <v>187</v>
       </c>
       <c r="M284" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N284" t="s">
         <v>14</v>
@@ -18477,22 +18528,22 @@
     </row>
     <row r="285" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A285" s="1" t="s">
-        <v>1323</v>
+        <v>1291</v>
       </c>
       <c r="B285" t="s">
-        <v>1338</v>
+        <v>1299</v>
       </c>
       <c r="C285" t="s">
-        <v>1346</v>
+        <v>1300</v>
       </c>
       <c r="D285" t="s">
-        <v>383</v>
+        <v>1301</v>
       </c>
       <c r="E285" t="s">
-        <v>904</v>
+        <v>1302</v>
       </c>
       <c r="F285" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G285" t="s">
         <v>51</v>
@@ -18506,8 +18557,11 @@
       <c r="J285" t="s">
         <v>488</v>
       </c>
+      <c r="K285" t="s">
+        <v>75</v>
+      </c>
       <c r="L285" t="s">
-        <v>95</v>
+        <v>187</v>
       </c>
       <c r="M285" t="s">
         <v>48</v>
@@ -18524,19 +18578,19 @@
     </row>
     <row r="286" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A286" s="1" t="s">
-        <v>393</v>
+        <v>715</v>
       </c>
       <c r="B286" t="s">
-        <v>786</v>
+        <v>740</v>
       </c>
       <c r="C286" t="s">
-        <v>1104</v>
+        <v>1218</v>
       </c>
       <c r="D286" t="s">
-        <v>398</v>
+        <v>743</v>
       </c>
       <c r="E286" t="s">
-        <v>908</v>
+        <v>1017</v>
       </c>
       <c r="F286" t="s">
         <v>47</v>
@@ -18545,13 +18599,10 @@
         <v>32</v>
       </c>
       <c r="H286" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I286" t="s">
-        <v>141</v>
-      </c>
-      <c r="J286" t="s">
-        <v>520</v>
+        <v>217</v>
       </c>
       <c r="L286" t="s">
         <v>179</v>
@@ -18571,19 +18622,19 @@
     </row>
     <row r="287" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A287" s="1" t="s">
-        <v>188</v>
+        <v>721</v>
       </c>
       <c r="B287" t="s">
-        <v>193</v>
+        <v>734</v>
       </c>
       <c r="C287" t="s">
-        <v>1074</v>
+        <v>1225</v>
       </c>
       <c r="D287" t="s">
-        <v>194</v>
+        <v>746</v>
       </c>
       <c r="E287" t="s">
-        <v>1025</v>
+        <v>1020</v>
       </c>
       <c r="F287" t="s">
         <v>47</v>
@@ -18598,7 +18649,7 @@
         <v>141</v>
       </c>
       <c r="J287" t="s">
-        <v>195</v>
+        <v>488</v>
       </c>
       <c r="K287" t="s">
         <v>75</v>
@@ -18621,25 +18672,25 @@
     </row>
     <row r="288" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A288" s="1" t="s">
-        <v>366</v>
+        <v>727</v>
       </c>
       <c r="B288" t="s">
-        <v>392</v>
+        <v>730</v>
       </c>
       <c r="C288" t="s">
-        <v>1103</v>
+        <v>1227</v>
       </c>
       <c r="D288" t="s">
-        <v>391</v>
+        <v>747</v>
       </c>
       <c r="E288" t="s">
-        <v>1030</v>
+        <v>1021</v>
       </c>
       <c r="F288" t="s">
         <v>47</v>
       </c>
       <c r="G288" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H288" t="s">
         <v>13</v>
@@ -18648,10 +18699,13 @@
         <v>141</v>
       </c>
       <c r="J288" t="s">
-        <v>277</v>
+        <v>520</v>
+      </c>
+      <c r="K288" t="s">
+        <v>140</v>
       </c>
       <c r="L288" t="s">
-        <v>196</v>
+        <v>179</v>
       </c>
       <c r="M288" t="s">
         <v>48</v>
@@ -18668,31 +18722,31 @@
     </row>
     <row r="289" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A289" s="1" t="s">
-        <v>1325</v>
+        <v>1268</v>
       </c>
       <c r="B289" t="s">
-        <v>1340</v>
+        <v>1275</v>
       </c>
       <c r="C289" t="s">
-        <v>1340</v>
+        <v>1273</v>
       </c>
       <c r="D289" t="s">
-        <v>1349</v>
+        <v>1276</v>
       </c>
       <c r="E289" t="s">
-        <v>1348</v>
+        <v>1276</v>
       </c>
       <c r="F289" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G289" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H289" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="I289" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J289" t="s">
         <v>277</v>
@@ -18715,19 +18769,13 @@
     </row>
     <row r="290" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A290" s="1" t="s">
-        <v>61</v>
+        <v>1288</v>
       </c>
       <c r="B290" t="s">
-        <v>70</v>
+        <v>1292</v>
       </c>
       <c r="C290" t="s">
-        <v>1128</v>
-      </c>
-      <c r="D290" t="s">
-        <v>289</v>
-      </c>
-      <c r="E290" t="s">
-        <v>929</v>
+        <v>1303</v>
       </c>
       <c r="F290" t="s">
         <v>78</v>
@@ -18739,13 +18787,16 @@
         <v>13</v>
       </c>
       <c r="I290" t="s">
-        <v>141</v>
+        <v>109</v>
       </c>
       <c r="J290" t="s">
-        <v>520</v>
+        <v>110</v>
+      </c>
+      <c r="K290" t="s">
+        <v>75</v>
       </c>
       <c r="L290" t="s">
-        <v>179</v>
+        <v>95</v>
       </c>
       <c r="M290" t="s">
         <v>48</v>
@@ -18762,22 +18813,22 @@
     </row>
     <row r="291" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A291" s="1" t="s">
-        <v>125</v>
+        <v>1323</v>
       </c>
       <c r="B291" t="s">
-        <v>131</v>
+        <v>1338</v>
       </c>
       <c r="C291" t="s">
-        <v>1130</v>
+        <v>1346</v>
       </c>
       <c r="D291" t="s">
-        <v>132</v>
+        <v>383</v>
       </c>
       <c r="E291" t="s">
-        <v>931</v>
+        <v>904</v>
       </c>
       <c r="F291" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G291" t="s">
         <v>51</v>
@@ -18789,16 +18840,13 @@
         <v>141</v>
       </c>
       <c r="J291" t="s">
-        <v>110</v>
-      </c>
-      <c r="K291" t="s">
-        <v>133</v>
+        <v>488</v>
       </c>
       <c r="L291" t="s">
-        <v>179</v>
+        <v>95</v>
       </c>
       <c r="M291" t="s">
-        <v>832</v>
+        <v>48</v>
       </c>
       <c r="N291" t="s">
         <v>14</v>
@@ -18812,13 +18860,19 @@
     </row>
     <row r="292" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A292" s="1" t="s">
-        <v>713</v>
+        <v>393</v>
       </c>
       <c r="B292" t="s">
-        <v>741</v>
+        <v>786</v>
       </c>
       <c r="C292" t="s">
-        <v>1229</v>
+        <v>1104</v>
+      </c>
+      <c r="D292" t="s">
+        <v>398</v>
+      </c>
+      <c r="E292" t="s">
+        <v>908</v>
       </c>
       <c r="F292" t="s">
         <v>47</v>
@@ -18832,6 +18886,9 @@
       <c r="I292" t="s">
         <v>141</v>
       </c>
+      <c r="J292" t="s">
+        <v>520</v>
+      </c>
       <c r="L292" t="s">
         <v>179</v>
       </c>
@@ -18850,19 +18907,25 @@
     </row>
     <row r="293" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A293" s="1" t="s">
-        <v>714</v>
+        <v>188</v>
       </c>
       <c r="B293" t="s">
-        <v>742</v>
+        <v>193</v>
       </c>
       <c r="C293" t="s">
-        <v>1230</v>
+        <v>1074</v>
+      </c>
+      <c r="D293" t="s">
+        <v>194</v>
+      </c>
+      <c r="E293" t="s">
+        <v>1025</v>
       </c>
       <c r="F293" t="s">
         <v>47</v>
       </c>
       <c r="G293" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H293" t="s">
         <v>13</v>
@@ -18870,8 +18933,14 @@
       <c r="I293" t="s">
         <v>141</v>
       </c>
+      <c r="J293" t="s">
+        <v>195</v>
+      </c>
+      <c r="K293" t="s">
+        <v>75</v>
+      </c>
       <c r="L293" t="s">
-        <v>179</v>
+        <v>196</v>
       </c>
       <c r="M293" t="s">
         <v>48</v>
@@ -18888,13 +18957,19 @@
     </row>
     <row r="294" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A294" s="1" t="s">
-        <v>835</v>
+        <v>366</v>
       </c>
       <c r="B294" t="s">
-        <v>838</v>
+        <v>392</v>
       </c>
       <c r="C294" t="s">
-        <v>1231</v>
+        <v>1103</v>
+      </c>
+      <c r="D294" t="s">
+        <v>391</v>
+      </c>
+      <c r="E294" t="s">
+        <v>1030</v>
       </c>
       <c r="F294" t="s">
         <v>47</v>
@@ -18911,11 +18986,8 @@
       <c r="J294" t="s">
         <v>277</v>
       </c>
-      <c r="K294" t="s">
-        <v>54</v>
-      </c>
       <c r="L294" t="s">
-        <v>179</v>
+        <v>196</v>
       </c>
       <c r="M294" t="s">
         <v>48</v>
@@ -18932,28 +19004,37 @@
     </row>
     <row r="295" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A295" s="1" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="B295" t="s">
-        <v>1341</v>
+        <v>1340</v>
+      </c>
+      <c r="C295" t="s">
+        <v>1340</v>
+      </c>
+      <c r="D295" t="s">
+        <v>1349</v>
+      </c>
+      <c r="E295" t="s">
+        <v>1348</v>
       </c>
       <c r="F295" t="s">
         <v>47</v>
       </c>
       <c r="G295" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H295" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I295" t="s">
-        <v>108</v>
-      </c>
-      <c r="K295" t="s">
-        <v>54</v>
+        <v>141</v>
+      </c>
+      <c r="J295" t="s">
+        <v>277</v>
       </c>
       <c r="L295" t="s">
-        <v>179</v>
+        <v>95</v>
       </c>
       <c r="M295" t="s">
         <v>48</v>
@@ -18970,22 +19051,22 @@
     </row>
     <row r="296" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A296" s="1" t="s">
-        <v>1333</v>
+        <v>61</v>
       </c>
       <c r="B296" t="s">
-        <v>1357</v>
+        <v>70</v>
       </c>
       <c r="C296" t="s">
-        <v>1358</v>
+        <v>1128</v>
       </c>
       <c r="D296" t="s">
-        <v>1314</v>
+        <v>289</v>
       </c>
       <c r="E296" t="s">
-        <v>980</v>
+        <v>929</v>
       </c>
       <c r="F296" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="G296" t="s">
         <v>51</v>
@@ -18997,10 +19078,10 @@
         <v>141</v>
       </c>
       <c r="J296" t="s">
-        <v>110</v>
+        <v>520</v>
       </c>
       <c r="L296" t="s">
-        <v>95</v>
+        <v>179</v>
       </c>
       <c r="M296" t="s">
         <v>48</v>
@@ -19017,19 +19098,19 @@
     </row>
     <row r="297" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A297" s="1" t="s">
-        <v>458</v>
+        <v>125</v>
       </c>
       <c r="B297" t="s">
-        <v>546</v>
+        <v>131</v>
       </c>
       <c r="C297" t="s">
-        <v>1235</v>
+        <v>1130</v>
       </c>
       <c r="D297" t="s">
-        <v>547</v>
+        <v>132</v>
       </c>
       <c r="E297" t="s">
-        <v>980</v>
+        <v>931</v>
       </c>
       <c r="F297" t="s">
         <v>78</v>
@@ -19053,7 +19134,7 @@
         <v>179</v>
       </c>
       <c r="M297" t="s">
-        <v>48</v>
+        <v>832</v>
       </c>
       <c r="N297" t="s">
         <v>14</v>
@@ -19067,25 +19148,19 @@
     </row>
     <row r="298" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A298" s="1" t="s">
-        <v>722</v>
+        <v>713</v>
       </c>
       <c r="B298" t="s">
-        <v>733</v>
+        <v>741</v>
       </c>
       <c r="C298" t="s">
-        <v>1232</v>
-      </c>
-      <c r="D298" t="s">
-        <v>547</v>
-      </c>
-      <c r="E298" t="s">
-        <v>980</v>
+        <v>1229</v>
       </c>
       <c r="F298" t="s">
         <v>47</v>
       </c>
       <c r="G298" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H298" t="s">
         <v>13</v>
@@ -19111,25 +19186,19 @@
     </row>
     <row r="299" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A299" s="1" t="s">
-        <v>593</v>
+        <v>714</v>
       </c>
       <c r="B299" t="s">
-        <v>602</v>
+        <v>742</v>
       </c>
       <c r="C299" t="s">
-        <v>1199</v>
-      </c>
-      <c r="D299" t="s">
-        <v>603</v>
-      </c>
-      <c r="E299" t="s">
-        <v>994</v>
+        <v>1230</v>
       </c>
       <c r="F299" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G299" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="H299" t="s">
         <v>13</v>
@@ -19137,17 +19206,11 @@
       <c r="I299" t="s">
         <v>141</v>
       </c>
-      <c r="J299" t="s">
-        <v>277</v>
-      </c>
-      <c r="K299" t="s">
-        <v>75</v>
-      </c>
       <c r="L299" t="s">
-        <v>95</v>
+        <v>179</v>
       </c>
       <c r="M299" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N299" t="s">
         <v>14</v>
@@ -19161,22 +19224,16 @@
     </row>
     <row r="300" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A300" s="1" t="s">
-        <v>294</v>
+        <v>835</v>
       </c>
       <c r="B300" t="s">
-        <v>310</v>
+        <v>838</v>
       </c>
       <c r="C300" t="s">
-        <v>1169</v>
-      </c>
-      <c r="D300" t="s">
-        <v>311</v>
-      </c>
-      <c r="E300" t="s">
-        <v>968</v>
+        <v>1231</v>
       </c>
       <c r="F300" t="s">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="G300" t="s">
         <v>32</v>
@@ -19190,11 +19247,14 @@
       <c r="J300" t="s">
         <v>277</v>
       </c>
+      <c r="K300" t="s">
+        <v>54</v>
+      </c>
       <c r="L300" t="s">
-        <v>95</v>
+        <v>179</v>
       </c>
       <c r="M300" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N300" t="s">
         <v>14</v>
@@ -19208,19 +19268,13 @@
     </row>
     <row r="301" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A301" s="1" t="s">
-        <v>1379</v>
+        <v>1416</v>
       </c>
       <c r="B301" t="s">
-        <v>1384</v>
+        <v>1437</v>
       </c>
       <c r="C301" t="s">
-        <v>1384</v>
-      </c>
-      <c r="D301" t="s">
-        <v>1388</v>
-      </c>
-      <c r="E301" t="s">
-        <v>1389</v>
+        <v>1437</v>
       </c>
       <c r="F301" t="s">
         <v>47</v>
@@ -19255,40 +19309,31 @@
     </row>
     <row r="302" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A302" s="1" t="s">
-        <v>1380</v>
+        <v>1326</v>
       </c>
       <c r="B302" t="s">
-        <v>1385</v>
-      </c>
-      <c r="C302" t="s">
-        <v>1386</v>
-      </c>
-      <c r="D302" t="s">
-        <v>1387</v>
-      </c>
-      <c r="E302" t="s">
-        <v>1113</v>
+        <v>1341</v>
       </c>
       <c r="F302" t="s">
         <v>47</v>
       </c>
       <c r="G302" t="s">
-        <v>119</v>
+        <v>32</v>
       </c>
       <c r="H302" t="s">
         <v>31</v>
       </c>
       <c r="I302" t="s">
-        <v>446</v>
-      </c>
-      <c r="J302" t="s">
-        <v>206</v>
+        <v>108</v>
+      </c>
+      <c r="K302" t="s">
+        <v>54</v>
       </c>
       <c r="L302" t="s">
         <v>179</v>
       </c>
       <c r="M302" t="s">
-        <v>833</v>
+        <v>48</v>
       </c>
       <c r="N302" t="s">
         <v>14</v>
@@ -19302,19 +19347,25 @@
     </row>
     <row r="303" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A303" s="1" t="s">
-        <v>1416</v>
+        <v>1333</v>
       </c>
       <c r="B303" t="s">
-        <v>1437</v>
+        <v>1357</v>
       </c>
       <c r="C303" t="s">
-        <v>1437</v>
+        <v>1358</v>
+      </c>
+      <c r="D303" t="s">
+        <v>1314</v>
+      </c>
+      <c r="E303" t="s">
+        <v>980</v>
       </c>
       <c r="F303" t="s">
         <v>47</v>
       </c>
       <c r="G303" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H303" t="s">
         <v>13</v>
@@ -19322,22 +19373,360 @@
       <c r="I303" t="s">
         <v>141</v>
       </c>
-      <c r="K303" t="s">
+      <c r="J303" t="s">
+        <v>110</v>
+      </c>
+      <c r="L303" t="s">
+        <v>95</v>
+      </c>
+      <c r="M303" t="s">
+        <v>48</v>
+      </c>
+      <c r="N303" t="s">
+        <v>14</v>
+      </c>
+      <c r="O303" t="s">
+        <v>15</v>
+      </c>
+      <c r="P303" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="304" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A304" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B304" t="s">
+        <v>546</v>
+      </c>
+      <c r="C304" t="s">
+        <v>1235</v>
+      </c>
+      <c r="D304" t="s">
+        <v>547</v>
+      </c>
+      <c r="E304" t="s">
+        <v>980</v>
+      </c>
+      <c r="F304" t="s">
+        <v>78</v>
+      </c>
+      <c r="G304" t="s">
+        <v>51</v>
+      </c>
+      <c r="H304" t="s">
+        <v>13</v>
+      </c>
+      <c r="I304" t="s">
+        <v>141</v>
+      </c>
+      <c r="J304" t="s">
+        <v>110</v>
+      </c>
+      <c r="K304" t="s">
+        <v>133</v>
+      </c>
+      <c r="L304" t="s">
+        <v>179</v>
+      </c>
+      <c r="M304" t="s">
+        <v>48</v>
+      </c>
+      <c r="N304" t="s">
+        <v>14</v>
+      </c>
+      <c r="O304" t="s">
+        <v>15</v>
+      </c>
+      <c r="P304" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="305" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A305" s="1" t="s">
+        <v>722</v>
+      </c>
+      <c r="B305" t="s">
+        <v>733</v>
+      </c>
+      <c r="C305" t="s">
+        <v>1232</v>
+      </c>
+      <c r="D305" t="s">
+        <v>547</v>
+      </c>
+      <c r="E305" t="s">
+        <v>980</v>
+      </c>
+      <c r="F305" t="s">
+        <v>47</v>
+      </c>
+      <c r="G305" t="s">
+        <v>51</v>
+      </c>
+      <c r="H305" t="s">
+        <v>13</v>
+      </c>
+      <c r="I305" t="s">
+        <v>141</v>
+      </c>
+      <c r="L305" t="s">
+        <v>179</v>
+      </c>
+      <c r="M305" t="s">
+        <v>48</v>
+      </c>
+      <c r="N305" t="s">
+        <v>14</v>
+      </c>
+      <c r="O305" t="s">
+        <v>15</v>
+      </c>
+      <c r="P305" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="306" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A306" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="B306" t="s">
+        <v>602</v>
+      </c>
+      <c r="C306" t="s">
+        <v>1199</v>
+      </c>
+      <c r="D306" t="s">
+        <v>603</v>
+      </c>
+      <c r="E306" t="s">
+        <v>994</v>
+      </c>
+      <c r="F306" t="s">
+        <v>78</v>
+      </c>
+      <c r="G306" t="s">
+        <v>51</v>
+      </c>
+      <c r="H306" t="s">
+        <v>13</v>
+      </c>
+      <c r="I306" t="s">
+        <v>141</v>
+      </c>
+      <c r="J306" t="s">
+        <v>277</v>
+      </c>
+      <c r="K306" t="s">
+        <v>75</v>
+      </c>
+      <c r="L306" t="s">
+        <v>95</v>
+      </c>
+      <c r="M306" t="s">
+        <v>49</v>
+      </c>
+      <c r="N306" t="s">
+        <v>14</v>
+      </c>
+      <c r="O306" t="s">
+        <v>15</v>
+      </c>
+      <c r="P306" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="307" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A307" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="B307" t="s">
+        <v>310</v>
+      </c>
+      <c r="C307" t="s">
+        <v>1169</v>
+      </c>
+      <c r="D307" t="s">
+        <v>311</v>
+      </c>
+      <c r="E307" t="s">
+        <v>968</v>
+      </c>
+      <c r="F307" t="s">
+        <v>78</v>
+      </c>
+      <c r="G307" t="s">
+        <v>32</v>
+      </c>
+      <c r="H307" t="s">
+        <v>13</v>
+      </c>
+      <c r="I307" t="s">
+        <v>141</v>
+      </c>
+      <c r="J307" t="s">
+        <v>277</v>
+      </c>
+      <c r="L307" t="s">
+        <v>95</v>
+      </c>
+      <c r="M307" t="s">
+        <v>49</v>
+      </c>
+      <c r="N307" t="s">
+        <v>14</v>
+      </c>
+      <c r="O307" t="s">
+        <v>15</v>
+      </c>
+      <c r="P307" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="308" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A308" s="1" t="s">
+        <v>1379</v>
+      </c>
+      <c r="B308" t="s">
+        <v>1384</v>
+      </c>
+      <c r="C308" t="s">
+        <v>1384</v>
+      </c>
+      <c r="D308" t="s">
+        <v>1388</v>
+      </c>
+      <c r="E308" t="s">
+        <v>1389</v>
+      </c>
+      <c r="F308" t="s">
+        <v>47</v>
+      </c>
+      <c r="G308" t="s">
+        <v>32</v>
+      </c>
+      <c r="H308" t="s">
+        <v>13</v>
+      </c>
+      <c r="I308" t="s">
+        <v>141</v>
+      </c>
+      <c r="K308" t="s">
         <v>54</v>
       </c>
-      <c r="L303" t="s">
+      <c r="L308" t="s">
         <v>179</v>
       </c>
-      <c r="M303" t="s">
-        <v>48</v>
-      </c>
-      <c r="N303" t="s">
-        <v>14</v>
-      </c>
-      <c r="O303" t="s">
-        <v>15</v>
-      </c>
-      <c r="P303" t="s">
+      <c r="M308" t="s">
+        <v>48</v>
+      </c>
+      <c r="N308" t="s">
+        <v>14</v>
+      </c>
+      <c r="O308" t="s">
+        <v>15</v>
+      </c>
+      <c r="P308" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="309" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A309" s="1" t="s">
+        <v>1380</v>
+      </c>
+      <c r="B309" t="s">
+        <v>1385</v>
+      </c>
+      <c r="C309" t="s">
+        <v>1386</v>
+      </c>
+      <c r="D309" t="s">
+        <v>1387</v>
+      </c>
+      <c r="E309" t="s">
+        <v>1113</v>
+      </c>
+      <c r="F309" t="s">
+        <v>47</v>
+      </c>
+      <c r="G309" t="s">
+        <v>119</v>
+      </c>
+      <c r="H309" t="s">
+        <v>31</v>
+      </c>
+      <c r="I309" t="s">
+        <v>446</v>
+      </c>
+      <c r="J309" t="s">
+        <v>206</v>
+      </c>
+      <c r="K309" t="s">
+        <v>54</v>
+      </c>
+      <c r="L309" t="s">
+        <v>179</v>
+      </c>
+      <c r="M309" t="s">
+        <v>833</v>
+      </c>
+      <c r="N309" t="s">
+        <v>14</v>
+      </c>
+      <c r="O309" t="s">
+        <v>15</v>
+      </c>
+      <c r="P309" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="310" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A310" s="1" t="s">
+        <v>1464</v>
+      </c>
+      <c r="B310" t="s">
+        <v>1472</v>
+      </c>
+      <c r="C310" t="s">
+        <v>1473</v>
+      </c>
+      <c r="D310" t="s">
+        <v>1474</v>
+      </c>
+      <c r="E310" t="s">
+        <v>1475</v>
+      </c>
+      <c r="F310" t="s">
+        <v>47</v>
+      </c>
+      <c r="G310" t="s">
+        <v>32</v>
+      </c>
+      <c r="H310" t="s">
+        <v>31</v>
+      </c>
+      <c r="I310" t="s">
+        <v>446</v>
+      </c>
+      <c r="J310" t="s">
+        <v>277</v>
+      </c>
+      <c r="K310" t="s">
+        <v>54</v>
+      </c>
+      <c r="L310" t="s">
+        <v>179</v>
+      </c>
+      <c r="M310" t="s">
+        <v>48</v>
+      </c>
+      <c r="N310" t="s">
+        <v>14</v>
+      </c>
+      <c r="O310" t="s">
+        <v>15</v>
+      </c>
+      <c r="P310" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Cambios scroll y temas
</commit_message>
<xml_diff>
--- a/data/PortfolioArTeV1.xlsx
+++ b/data/PortfolioArTeV1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arturompw/portfolio/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F067A5D-96F1-4441-B9E9-B2CBCC0D2345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B48A061-3E45-3A42-828D-2D1A569CEC49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4100" yWindow="600" windowWidth="22940" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolio" sheetId="1" r:id="rId1"/>
@@ -4714,9 +4714,6 @@
     <t>tiempos litúrgicos;educación;social;María</t>
   </si>
   <si>
-    <t>social;educación;tiempos litúrgicos;María, Jesús</t>
-  </si>
-  <si>
     <t>tiempos litúrgicos;María;Jesús</t>
   </si>
   <si>
@@ -4736,6 +4733,9 @@
   </si>
   <si>
     <t>social;educación;maristas</t>
+  </si>
+  <si>
+    <t>social;educación;tiempos litúrgicos;María;Jesús</t>
   </si>
 </sst>
 </file>
@@ -17168,7 +17168,7 @@
         <v>256</v>
       </c>
       <c r="J250" t="s">
-        <v>1564</v>
+        <v>1571</v>
       </c>
       <c r="K250" t="s">
         <v>50</v>
@@ -17218,7 +17218,7 @@
         <v>102</v>
       </c>
       <c r="J251" t="s">
-        <v>1565</v>
+        <v>1564</v>
       </c>
       <c r="K251" t="s">
         <v>395</v>
@@ -17612,7 +17612,7 @@
         <v>134</v>
       </c>
       <c r="J259" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="K259" t="s">
         <v>70</v>
@@ -17941,7 +17941,7 @@
         <v>134</v>
       </c>
       <c r="J266" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
       <c r="L266" t="s">
         <v>368</v>
@@ -18338,7 +18338,7 @@
         <v>206</v>
       </c>
       <c r="J274" t="s">
-        <v>1568</v>
+        <v>1567</v>
       </c>
       <c r="L274" t="s">
         <v>90</v>
@@ -18385,7 +18385,7 @@
         <v>424</v>
       </c>
       <c r="J275" t="s">
-        <v>1569</v>
+        <v>1568</v>
       </c>
       <c r="L275" t="s">
         <v>90</v>
@@ -18532,7 +18532,7 @@
         <v>1256</v>
       </c>
       <c r="J278" t="s">
-        <v>1569</v>
+        <v>1568</v>
       </c>
       <c r="K278" t="s">
         <v>133</v>
@@ -19205,7 +19205,7 @@
         <v>256</v>
       </c>
       <c r="J292" t="s">
-        <v>1570</v>
+        <v>1569</v>
       </c>
       <c r="L292" t="s">
         <v>528</v>
@@ -19252,7 +19252,7 @@
         <v>256</v>
       </c>
       <c r="J293" t="s">
-        <v>1571</v>
+        <v>1570</v>
       </c>
       <c r="L293" t="s">
         <v>368</v>
@@ -19834,7 +19834,7 @@
         <v>134</v>
       </c>
       <c r="J305" t="s">
-        <v>1570</v>
+        <v>1569</v>
       </c>
       <c r="K305" t="s">
         <v>133</v>

</xml_diff>

<commit_message>
Cambios scroll y temas intento 3
</commit_message>
<xml_diff>
--- a/data/PortfolioArTeV1.xlsx
+++ b/data/PortfolioArTeV1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arturompw/portfolio/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B48A061-3E45-3A42-828D-2D1A569CEC49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A06D280-8170-9A45-A17E-F1C5DE7D5630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4100" yWindow="600" windowWidth="22940" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolio" sheetId="1" r:id="rId1"/>
@@ -4684,39 +4684,6 @@
     <t>maristas;educación;social;violetas</t>
   </si>
   <si>
-    <t>educación;tiempos litúrgicos</t>
-  </si>
-  <si>
-    <t>maristas;educación;tiempos litúrgicos</t>
-  </si>
-  <si>
-    <t>evangelio;educación;maristas;tiempos litúrgicos</t>
-  </si>
-  <si>
-    <t>evangelio;tiempos litúrgicos</t>
-  </si>
-  <si>
-    <t>tiempos litúrgicos</t>
-  </si>
-  <si>
-    <t>evangelio;tiempos litúrgicos;Jesús</t>
-  </si>
-  <si>
-    <t>social;tiempos litúrgicos</t>
-  </si>
-  <si>
-    <t>tiempos litúrgicos;social;Jesús;violetas</t>
-  </si>
-  <si>
-    <t>tiempos litúrgicos;violetas;Jesús</t>
-  </si>
-  <si>
-    <t>tiempos litúrgicos;educación;social;María</t>
-  </si>
-  <si>
-    <t>tiempos litúrgicos;María;Jesús</t>
-  </si>
-  <si>
     <t>social;educación;paz</t>
   </si>
   <si>
@@ -4735,7 +4702,40 @@
     <t>social;educación;maristas</t>
   </si>
   <si>
-    <t>social;educación;tiempos litúrgicos;María;Jesús</t>
+    <t>maristas;educación;tiempos_liturgicos</t>
+  </si>
+  <si>
+    <t>evangelio;educación;maristas;tiempos_liturgicos</t>
+  </si>
+  <si>
+    <t>educación;tiempos_liturgicos</t>
+  </si>
+  <si>
+    <t>evangelio;tiempos_liturgicos</t>
+  </si>
+  <si>
+    <t>tiempos_liturgicos</t>
+  </si>
+  <si>
+    <t>evangelio;tiempos_liturgicos;Jesús</t>
+  </si>
+  <si>
+    <t>social;tiempos_liturgicos</t>
+  </si>
+  <si>
+    <t>tiempos_liturgicos;social;Jesús;violetas</t>
+  </si>
+  <si>
+    <t>tiempos_liturgicos;violetas;Jesús</t>
+  </si>
+  <si>
+    <t>tiempos_liturgicos;educación;social;María</t>
+  </si>
+  <si>
+    <t>social;educación;tiempos_liturgicos;María;Jesús</t>
+  </si>
+  <si>
+    <t>tiempos_liturgicos;María;Jesús</t>
   </si>
 </sst>
 </file>
@@ -15513,7 +15513,7 @@
         <v>256</v>
       </c>
       <c r="J216" t="s">
-        <v>1555</v>
+        <v>1560</v>
       </c>
       <c r="K216" t="s">
         <v>70</v>
@@ -15563,7 +15563,7 @@
         <v>256</v>
       </c>
       <c r="J217" t="s">
-        <v>1555</v>
+        <v>1560</v>
       </c>
       <c r="K217" t="s">
         <v>70</v>
@@ -15613,7 +15613,7 @@
         <v>310</v>
       </c>
       <c r="J218" t="s">
-        <v>1555</v>
+        <v>1560</v>
       </c>
       <c r="K218" t="s">
         <v>70</v>
@@ -15663,7 +15663,7 @@
         <v>256</v>
       </c>
       <c r="J219" t="s">
-        <v>1556</v>
+        <v>1561</v>
       </c>
       <c r="K219" t="s">
         <v>70</v>
@@ -15713,7 +15713,7 @@
         <v>256</v>
       </c>
       <c r="J220" t="s">
-        <v>1554</v>
+        <v>1562</v>
       </c>
       <c r="K220" t="s">
         <v>194</v>
@@ -15763,7 +15763,7 @@
         <v>256</v>
       </c>
       <c r="J221" t="s">
-        <v>1554</v>
+        <v>1562</v>
       </c>
       <c r="K221" t="s">
         <v>70</v>
@@ -15813,7 +15813,7 @@
         <v>256</v>
       </c>
       <c r="J222" t="s">
-        <v>1554</v>
+        <v>1562</v>
       </c>
       <c r="K222" t="s">
         <v>70</v>
@@ -15863,7 +15863,7 @@
         <v>256</v>
       </c>
       <c r="J223" t="s">
-        <v>1557</v>
+        <v>1563</v>
       </c>
       <c r="K223" t="s">
         <v>51</v>
@@ -15913,7 +15913,7 @@
         <v>256</v>
       </c>
       <c r="J224" t="s">
-        <v>1557</v>
+        <v>1563</v>
       </c>
       <c r="K224" t="s">
         <v>51</v>
@@ -15963,7 +15963,7 @@
         <v>256</v>
       </c>
       <c r="J225" t="s">
-        <v>1557</v>
+        <v>1563</v>
       </c>
       <c r="K225" t="s">
         <v>51</v>
@@ -16013,7 +16013,7 @@
         <v>256</v>
       </c>
       <c r="J226" t="s">
-        <v>1557</v>
+        <v>1563</v>
       </c>
       <c r="K226" t="s">
         <v>133</v>
@@ -16063,7 +16063,7 @@
         <v>256</v>
       </c>
       <c r="J227" t="s">
-        <v>1557</v>
+        <v>1563</v>
       </c>
       <c r="K227" t="s">
         <v>51</v>
@@ -16163,7 +16163,7 @@
         <v>424</v>
       </c>
       <c r="J229" t="s">
-        <v>1557</v>
+        <v>1563</v>
       </c>
       <c r="K229" t="s">
         <v>395</v>
@@ -16213,7 +16213,7 @@
         <v>134</v>
       </c>
       <c r="J230" t="s">
-        <v>1558</v>
+        <v>1564</v>
       </c>
       <c r="K230" t="s">
         <v>133</v>
@@ -16263,7 +16263,7 @@
         <v>136</v>
       </c>
       <c r="J231" t="s">
-        <v>1559</v>
+        <v>1565</v>
       </c>
       <c r="L231" t="s">
         <v>172</v>
@@ -16357,7 +16357,7 @@
         <v>134</v>
       </c>
       <c r="J233" t="s">
-        <v>1557</v>
+        <v>1563</v>
       </c>
       <c r="K233" t="s">
         <v>51</v>
@@ -16407,7 +16407,7 @@
         <v>134</v>
       </c>
       <c r="J234" t="s">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="K234" t="s">
         <v>51</v>
@@ -16451,7 +16451,7 @@
         <v>424</v>
       </c>
       <c r="J235" t="s">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="K235" t="s">
         <v>51</v>
@@ -16495,7 +16495,7 @@
         <v>424</v>
       </c>
       <c r="J236" t="s">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="K236" t="s">
         <v>51</v>
@@ -16539,7 +16539,7 @@
         <v>424</v>
       </c>
       <c r="J237" t="s">
-        <v>1560</v>
+        <v>1566</v>
       </c>
       <c r="K237" t="s">
         <v>51</v>
@@ -16639,7 +16639,7 @@
         <v>1216</v>
       </c>
       <c r="J239" t="s">
-        <v>1557</v>
+        <v>1563</v>
       </c>
       <c r="L239" t="s">
         <v>92</v>
@@ -16824,7 +16824,7 @@
         <v>310</v>
       </c>
       <c r="J243" t="s">
-        <v>1554</v>
+        <v>1562</v>
       </c>
       <c r="K243" t="s">
         <v>70</v>
@@ -16874,7 +16874,7 @@
         <v>256</v>
       </c>
       <c r="J244" t="s">
-        <v>1554</v>
+        <v>1562</v>
       </c>
       <c r="K244" t="s">
         <v>70</v>
@@ -16924,7 +16924,7 @@
         <v>103</v>
       </c>
       <c r="J245" t="s">
-        <v>1558</v>
+        <v>1564</v>
       </c>
       <c r="K245" t="s">
         <v>70</v>
@@ -16974,7 +16974,7 @@
         <v>134</v>
       </c>
       <c r="J246" t="s">
-        <v>1558</v>
+        <v>1564</v>
       </c>
       <c r="K246" t="s">
         <v>50</v>
@@ -17024,7 +17024,7 @@
         <v>134</v>
       </c>
       <c r="J247" t="s">
-        <v>1561</v>
+        <v>1567</v>
       </c>
       <c r="L247" t="s">
         <v>457</v>
@@ -17071,7 +17071,7 @@
         <v>134</v>
       </c>
       <c r="J248" t="s">
-        <v>1562</v>
+        <v>1568</v>
       </c>
       <c r="K248" t="s">
         <v>51</v>
@@ -17121,7 +17121,7 @@
         <v>134</v>
       </c>
       <c r="J249" t="s">
-        <v>1563</v>
+        <v>1569</v>
       </c>
       <c r="L249" t="s">
         <v>175</v>
@@ -17168,7 +17168,7 @@
         <v>256</v>
       </c>
       <c r="J250" t="s">
-        <v>1571</v>
+        <v>1570</v>
       </c>
       <c r="K250" t="s">
         <v>50</v>
@@ -17218,7 +17218,7 @@
         <v>102</v>
       </c>
       <c r="J251" t="s">
-        <v>1564</v>
+        <v>1571</v>
       </c>
       <c r="K251" t="s">
         <v>395</v>
@@ -17268,7 +17268,7 @@
         <v>136</v>
       </c>
       <c r="J252" t="s">
-        <v>1559</v>
+        <v>1565</v>
       </c>
       <c r="K252" t="s">
         <v>51</v>
@@ -17312,7 +17312,7 @@
         <v>424</v>
       </c>
       <c r="J253" t="s">
-        <v>1558</v>
+        <v>1564</v>
       </c>
       <c r="K253" t="s">
         <v>51</v>
@@ -17612,7 +17612,7 @@
         <v>134</v>
       </c>
       <c r="J259" t="s">
-        <v>1565</v>
+        <v>1554</v>
       </c>
       <c r="K259" t="s">
         <v>70</v>
@@ -17941,7 +17941,7 @@
         <v>134</v>
       </c>
       <c r="J266" t="s">
-        <v>1566</v>
+        <v>1555</v>
       </c>
       <c r="L266" t="s">
         <v>368</v>
@@ -18338,7 +18338,7 @@
         <v>206</v>
       </c>
       <c r="J274" t="s">
-        <v>1567</v>
+        <v>1556</v>
       </c>
       <c r="L274" t="s">
         <v>90</v>
@@ -18385,7 +18385,7 @@
         <v>424</v>
       </c>
       <c r="J275" t="s">
-        <v>1568</v>
+        <v>1557</v>
       </c>
       <c r="L275" t="s">
         <v>90</v>
@@ -18532,7 +18532,7 @@
         <v>1256</v>
       </c>
       <c r="J278" t="s">
-        <v>1568</v>
+        <v>1557</v>
       </c>
       <c r="K278" t="s">
         <v>133</v>
@@ -19205,7 +19205,7 @@
         <v>256</v>
       </c>
       <c r="J292" t="s">
-        <v>1569</v>
+        <v>1558</v>
       </c>
       <c r="L292" t="s">
         <v>528</v>
@@ -19252,7 +19252,7 @@
         <v>256</v>
       </c>
       <c r="J293" t="s">
-        <v>1570</v>
+        <v>1559</v>
       </c>
       <c r="L293" t="s">
         <v>368</v>
@@ -19737,7 +19737,7 @@
         <v>205</v>
       </c>
       <c r="J303" t="s">
-        <v>1558</v>
+        <v>1564</v>
       </c>
       <c r="L303" t="s">
         <v>172</v>
@@ -19834,7 +19834,7 @@
         <v>134</v>
       </c>
       <c r="J305" t="s">
-        <v>1569</v>
+        <v>1558</v>
       </c>
       <c r="K305" t="s">
         <v>133</v>

</xml_diff>

<commit_message>
Cambios scroll y temas 4b
</commit_message>
<xml_diff>
--- a/data/PortfolioArTeV1.xlsx
+++ b/data/PortfolioArTeV1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arturompw/portfolio/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4673E36-D525-4047-A5AF-35895D77E0B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{446B6F8A-1EBF-F444-9749-D053D52B6B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4100" yWindow="600" windowWidth="22940" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolio" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5076" uniqueCount="1581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5076" uniqueCount="1582">
   <si>
     <t>id</t>
   </si>
@@ -4763,6 +4763,9 @@
   </si>
   <si>
     <t>Smug</t>
+  </si>
+  <si>
+    <t>ILU-0219</t>
   </si>
 </sst>
 </file>
@@ -20330,7 +20333,7 @@
     </row>
     <row r="316" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A316" s="1" t="s">
-        <v>1475</v>
+        <v>1581</v>
       </c>
       <c r="B316" t="s">
         <v>1574</v>

</xml_diff>